<commit_message>
Corrigeer Totaal gefactureerd: tel alle 5 termijnen (F27:F31)
Voorheen telde F33 alleen termijn 1-3 (SUM(F27:F29)).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5wVhvLcrmmgSCsGwdMWTF
</commit_message>
<xml_diff>
--- a/Kostencalculatie_Compleet.xlsx
+++ b/Kostencalculatie_Compleet.xlsx
@@ -398,7 +398,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="83">
+  <borders count="86">
     <border>
       <left/>
       <right/>
@@ -1467,6 +1467,39 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -1475,7 +1508,7 @@
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="395">
+  <cellXfs count="396">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2267,6 +2300,7 @@
     <xf numFmtId="170" fontId="0" fillId="16" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="21" fillId="11" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="28" fillId="10" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="85" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -4203,7 +4237,7 @@
       <c r="D33" s="275" t="n"/>
       <c r="E33" s="273" t="n"/>
       <c r="F33" s="276">
-        <f>SUM(F27:F29)</f>
+        <f>SUM(F27:F31)</f>
         <v/>
       </c>
       <c r="G33" s="273" t="n"/>
@@ -19666,11 +19700,13 @@
           <t>Hoog tarief</t>
         </is>
       </c>
+      <c r="E3" s="395" t="n"/>
       <c r="F3" s="315" t="inlineStr">
         <is>
           <t>Laag tarief</t>
         </is>
       </c>
+      <c r="G3" s="395" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="315" t="inlineStr">

</xml_diff>

<commit_message>
Kousen: dry-linerdeel apart prijzen + SAERTEX-indexering
- Kolom hernoemd naar 'Geïmpregneerde lengte' (direct invoeren)
- Aparte kolom 'Dry/omslag lengte' + instelbaar dry-liner €/m-tarief:
  kosten dry-liner = dry-lengte x tarief (omslag/eindstuk niet geïmpregneerd)
- Kostprijs totaal = geïmpregneerd + dry-liner
- Indexering op SAERTEX-prijslijst instelbaar (cel op SAERTEX 2026);
  werkt door in alle €/m via (1 + indexering)
- Handlingstaffel nu op totale linerlengte (geïmpregneerd + dry)
- Totalen doorgekoppeld naar Periode-overzicht, Prognose en Overzicht

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5wVhvLcrmmgSCsGwdMWTF
</commit_message>
<xml_diff>
--- a/Kostencalculatie_Compleet.xlsx
+++ b/Kostencalculatie_Compleet.xlsx
@@ -99,7 +99,7 @@
     <numFmt numFmtId="173" formatCode="#,##0.00\ &quot;€&quot;;-#,##0.00\ &quot;€&quot;;&quot;&quot;"/>
     <numFmt numFmtId="174" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="45">
+  <fonts count="46">
     <font>
       <name val="Tahoma"/>
       <family val="2"/>
@@ -331,6 +331,10 @@
     </font>
     <font>
       <color rgb="00000000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
     </font>
   </fonts>
   <fills count="19">
@@ -1544,7 +1548,7 @@
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="441">
+  <cellXfs count="444">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2406,6 +2410,9 @@
     </xf>
     <xf numFmtId="170" fontId="43" fillId="11" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="44" fillId="12" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="16" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="21" fillId="12" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -3642,7 +3649,7 @@
       </c>
       <c r="C26" s="244" t="n"/>
       <c r="D26" s="245">
-        <f>'Kousen'!K81</f>
+        <f>'Kousen'!N81</f>
         <v/>
       </c>
     </row>
@@ -3962,7 +3969,7 @@
         </is>
       </c>
       <c r="B17" s="437">
-        <f>SUM(Kousen!$K$5:$K$80)</f>
+        <f>SUM(Kousen!$N$5:$N$80)</f>
         <v/>
       </c>
     </row>
@@ -4057,11 +4064,11 @@
         <v/>
       </c>
       <c r="D25" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C25)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C25)</f>
         <v/>
       </c>
       <c r="E25" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D25</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D25</f>
         <v/>
       </c>
       <c r="F25" s="385" t="n"/>
@@ -4090,11 +4097,11 @@
         <v/>
       </c>
       <c r="D26" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C26)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C26)</f>
         <v/>
       </c>
       <c r="E26" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D26</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D26</f>
         <v/>
       </c>
       <c r="F26" s="385" t="n"/>
@@ -4123,11 +4130,11 @@
         <v/>
       </c>
       <c r="D27" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C27)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C27)</f>
         <v/>
       </c>
       <c r="E27" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D27</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D27</f>
         <v/>
       </c>
       <c r="F27" s="385" t="n"/>
@@ -4156,11 +4163,11 @@
         <v/>
       </c>
       <c r="D28" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C28)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C28)</f>
         <v/>
       </c>
       <c r="E28" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D28</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D28</f>
         <v/>
       </c>
       <c r="F28" s="385" t="n"/>
@@ -4189,11 +4196,11 @@
         <v/>
       </c>
       <c r="D29" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C29)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C29)</f>
         <v/>
       </c>
       <c r="E29" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D29</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D29</f>
         <v/>
       </c>
       <c r="F29" s="385" t="n"/>
@@ -4222,11 +4229,11 @@
         <v/>
       </c>
       <c r="D30" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C30)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C30)</f>
         <v/>
       </c>
       <c r="E30" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D30</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D30</f>
         <v/>
       </c>
       <c r="F30" s="385" t="n"/>
@@ -4255,11 +4262,11 @@
         <v/>
       </c>
       <c r="D31" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C31)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C31)</f>
         <v/>
       </c>
       <c r="E31" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D31</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D31</f>
         <v/>
       </c>
       <c r="F31" s="385" t="n"/>
@@ -4288,11 +4295,11 @@
         <v/>
       </c>
       <c r="D32" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C32)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C32)</f>
         <v/>
       </c>
       <c r="E32" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D32</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D32</f>
         <v/>
       </c>
       <c r="F32" s="385" t="n"/>
@@ -4321,11 +4328,11 @@
         <v/>
       </c>
       <c r="D33" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C33)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C33)</f>
         <v/>
       </c>
       <c r="E33" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D33</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D33</f>
         <v/>
       </c>
       <c r="F33" s="385" t="n"/>
@@ -4354,11 +4361,11 @@
         <v/>
       </c>
       <c r="D34" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C34)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C34)</f>
         <v/>
       </c>
       <c r="E34" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D34</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D34</f>
         <v/>
       </c>
       <c r="F34" s="385" t="n"/>
@@ -4387,11 +4394,11 @@
         <v/>
       </c>
       <c r="D35" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C35)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C35)</f>
         <v/>
       </c>
       <c r="E35" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D35</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D35</f>
         <v/>
       </c>
       <c r="F35" s="385" t="n"/>
@@ -4420,11 +4427,11 @@
         <v/>
       </c>
       <c r="D36" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C36)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C36)</f>
         <v/>
       </c>
       <c r="E36" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D36</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D36</f>
         <v/>
       </c>
       <c r="F36" s="385" t="n"/>
@@ -4453,11 +4460,11 @@
         <v/>
       </c>
       <c r="D37" s="392">
-        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C37)</f>
+        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C37)</f>
         <v/>
       </c>
       <c r="E37" s="392">
-        <f>SUM(Kousen!$K$5:$K$80)-$D37</f>
+        <f>SUM(Kousen!$N$5:$N$80)-$D37</f>
         <v/>
       </c>
       <c r="F37" s="385" t="n"/>
@@ -4487,21 +4494,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:O81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4514,14 +4524,14 @@
     <row r="2">
       <c r="A2" s="386" t="inlineStr">
         <is>
-          <t>Geel = invoer. €/m, handlingstoeslag, kostprijs en periode rekenen automatisch.</t>
+          <t>Geel = invoer. €/m (incl. indexering), handling, kosten en periode rekenen automatisch.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="421" t="inlineStr">
         <is>
-          <t>Handlingstoeslag meerekenen:</t>
+          <t>Handling meerekenen:</t>
         </is>
       </c>
       <c r="B3" s="306" t="inlineStr">
@@ -4529,13 +4539,28 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="C3" s="422" t="inlineStr">
-        <is>
-          <t>(SAERTEX: &lt;15m +25%, 15-50m +3,5%, 50-200m +2,5%, &gt;200m +1,0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+      <c r="D3" s="421" t="inlineStr">
+        <is>
+          <t>Dry-liner €/m:</t>
+        </is>
+      </c>
+      <c r="E3" s="385" t="n"/>
+      <c r="F3" s="421" t="inlineStr">
+        <is>
+          <t>Indexering SAERTEX:</t>
+        </is>
+      </c>
+      <c r="G3" s="441">
+        <f>'SAERTEX 2026'!$B$3</f>
+        <v/>
+      </c>
+      <c r="I3" s="422" t="inlineStr">
+        <is>
+          <t>(dry-€/m = tarief voor omslag/eindstuk; indexering stel je in op SAERTEX 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="315" t="inlineStr">
         <is>
           <t>Kousnr</t>
@@ -4569,35 +4594,53 @@
       </c>
       <c r="G4" s="315" t="inlineStr">
         <is>
-          <t>Lengte
-(m)</t>
+          <t>Geïmpreg.
+lengte (m)</t>
         </is>
       </c>
       <c r="H4" s="315" t="inlineStr">
+        <is>
+          <t>Dry/omslag
+lengte (m)</t>
+        </is>
+      </c>
+      <c r="I4" s="315" t="inlineStr">
         <is>
           <t>Inbreng-
 datum</t>
         </is>
       </c>
-      <c r="I4" s="315" t="inlineStr">
+      <c r="J4" s="315" t="inlineStr">
         <is>
           <t>€/m
 (basis)</t>
         </is>
       </c>
-      <c r="J4" s="315" t="inlineStr">
+      <c r="K4" s="315" t="inlineStr">
         <is>
           <t>Handling
 %</t>
         </is>
       </c>
-      <c r="K4" s="315" t="inlineStr">
+      <c r="L4" s="315" t="inlineStr">
+        <is>
+          <t>Kosten
+geïmpreg.</t>
+        </is>
+      </c>
+      <c r="M4" s="315" t="inlineStr">
+        <is>
+          <t>Kosten
+dry-liner</t>
+        </is>
+      </c>
+      <c r="N4" s="315" t="inlineStr">
         <is>
           <t>Kostprijs
-(€)</t>
-        </is>
-      </c>
-      <c r="L4" s="315" t="inlineStr">
+totaal (€)</t>
+        </is>
+      </c>
+      <c r="O4" s="315" t="inlineStr">
         <is>
           <t>Periode
 (auto)</t>
@@ -4634,23 +4677,34 @@
       <c r="G5" s="391" t="n">
         <v>121.8</v>
       </c>
-      <c r="H5" s="417" t="n">
+      <c r="H5" s="391" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I5" s="417" t="n">
         <v>45294</v>
       </c>
-      <c r="I5" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C5,'SAERTEX-prijstabel'!$B$2:$B$496,$D5,'SAERTEX-prijstabel'!$C$2:$C$496,$E5,'SAERTEX-prijstabel'!$D$2:$D$496,$F5),0)</f>
-        <v/>
-      </c>
-      <c r="J5" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G5="","",IF($G5&lt;15,0.25,IF($G5&lt;=50,0.035,IF($G5&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K5" s="392">
-        <f>IF($I5=0,0,$G5*$I5*(1+N($J5)))</f>
-        <v/>
-      </c>
-      <c r="L5" s="401">
-        <f>IF($H5="","nog te plannen",IFERROR(LOOKUP($H5,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J5" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C5,'SAERTEX-prijstabel'!$B$2:$B$496,$D5,'SAERTEX-prijstabel'!$C$2:$C$496,$E5,'SAERTEX-prijstabel'!$D$2:$D$496,$F5),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K5" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G5)+N($H5))=0,0,IF((N($G5)+N($H5))&lt;15,0.25,IF((N($G5)+N($H5))&lt;=50,0.035,IF((N($G5)+N($H5))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L5" s="392">
+        <f>IF($J5=0,0,$G5*$J5*(1+$K5))</f>
+        <v/>
+      </c>
+      <c r="M5" s="392">
+        <f>N($H5)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N5" s="398">
+        <f>$L5+$M5</f>
+        <v/>
+      </c>
+      <c r="O5" s="401">
+        <f>IF($I5="","nog te plannen",IFERROR(LOOKUP($I5,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4684,23 +4738,34 @@
       <c r="G6" s="391" t="n">
         <v>30.6</v>
       </c>
-      <c r="H6" s="417" t="n">
+      <c r="H6" s="391" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="I6" s="417" t="n">
         <v>45296</v>
       </c>
-      <c r="I6" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C6,'SAERTEX-prijstabel'!$B$2:$B$496,$D6,'SAERTEX-prijstabel'!$C$2:$C$496,$E6,'SAERTEX-prijstabel'!$D$2:$D$496,$F6),0)</f>
-        <v/>
-      </c>
-      <c r="J6" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G6="","",IF($G6&lt;15,0.25,IF($G6&lt;=50,0.035,IF($G6&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K6" s="392">
-        <f>IF($I6=0,0,$G6*$I6*(1+N($J6)))</f>
-        <v/>
-      </c>
-      <c r="L6" s="401">
-        <f>IF($H6="","nog te plannen",IFERROR(LOOKUP($H6,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J6" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C6,'SAERTEX-prijstabel'!$B$2:$B$496,$D6,'SAERTEX-prijstabel'!$C$2:$C$496,$E6,'SAERTEX-prijstabel'!$D$2:$D$496,$F6),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K6" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G6)+N($H6))=0,0,IF((N($G6)+N($H6))&lt;15,0.25,IF((N($G6)+N($H6))&lt;=50,0.035,IF((N($G6)+N($H6))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L6" s="392">
+        <f>IF($J6=0,0,$G6*$J6*(1+$K6))</f>
+        <v/>
+      </c>
+      <c r="M6" s="392">
+        <f>N($H6)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N6" s="398">
+        <f>$L6+$M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="401">
+        <f>IF($I6="","nog te plannen",IFERROR(LOOKUP($I6,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4734,23 +4799,34 @@
       <c r="G7" s="391" t="n">
         <v>60</v>
       </c>
-      <c r="H7" s="417" t="n">
+      <c r="H7" s="391" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="I7" s="417" t="n">
         <v>45298</v>
       </c>
-      <c r="I7" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C7,'SAERTEX-prijstabel'!$B$2:$B$496,$D7,'SAERTEX-prijstabel'!$C$2:$C$496,$E7,'SAERTEX-prijstabel'!$D$2:$D$496,$F7),0)</f>
-        <v/>
-      </c>
-      <c r="J7" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G7="","",IF($G7&lt;15,0.25,IF($G7&lt;=50,0.035,IF($G7&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K7" s="392">
-        <f>IF($I7=0,0,$G7*$I7*(1+N($J7)))</f>
-        <v/>
-      </c>
-      <c r="L7" s="401">
-        <f>IF($H7="","nog te plannen",IFERROR(LOOKUP($H7,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J7" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C7,'SAERTEX-prijstabel'!$B$2:$B$496,$D7,'SAERTEX-prijstabel'!$C$2:$C$496,$E7,'SAERTEX-prijstabel'!$D$2:$D$496,$F7),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K7" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G7)+N($H7))=0,0,IF((N($G7)+N($H7))&lt;15,0.25,IF((N($G7)+N($H7))&lt;=50,0.035,IF((N($G7)+N($H7))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L7" s="392">
+        <f>IF($J7=0,0,$G7*$J7*(1+$K7))</f>
+        <v/>
+      </c>
+      <c r="M7" s="392">
+        <f>N($H7)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N7" s="398">
+        <f>$L7+$M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="401">
+        <f>IF($I7="","nog te plannen",IFERROR(LOOKUP($I7,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4784,23 +4860,34 @@
       <c r="G8" s="391" t="n">
         <v>104.7</v>
       </c>
-      <c r="H8" s="417" t="n">
+      <c r="H8" s="391" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="I8" s="417" t="n">
         <v>45300</v>
       </c>
-      <c r="I8" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C8,'SAERTEX-prijstabel'!$B$2:$B$496,$D8,'SAERTEX-prijstabel'!$C$2:$C$496,$E8,'SAERTEX-prijstabel'!$D$2:$D$496,$F8),0)</f>
-        <v/>
-      </c>
-      <c r="J8" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G8="","",IF($G8&lt;15,0.25,IF($G8&lt;=50,0.035,IF($G8&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K8" s="392">
-        <f>IF($I8=0,0,$G8*$I8*(1+N($J8)))</f>
-        <v/>
-      </c>
-      <c r="L8" s="401">
-        <f>IF($H8="","nog te plannen",IFERROR(LOOKUP($H8,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J8" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C8,'SAERTEX-prijstabel'!$B$2:$B$496,$D8,'SAERTEX-prijstabel'!$C$2:$C$496,$E8,'SAERTEX-prijstabel'!$D$2:$D$496,$F8),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K8" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G8)+N($H8))=0,0,IF((N($G8)+N($H8))&lt;15,0.25,IF((N($G8)+N($H8))&lt;=50,0.035,IF((N($G8)+N($H8))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L8" s="392">
+        <f>IF($J8=0,0,$G8*$J8*(1+$K8))</f>
+        <v/>
+      </c>
+      <c r="M8" s="392">
+        <f>N($H8)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N8" s="398">
+        <f>$L8+$M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="401">
+        <f>IF($I8="","nog te plannen",IFERROR(LOOKUP($I8,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4834,23 +4921,34 @@
       <c r="G9" s="391" t="n">
         <v>67.3</v>
       </c>
-      <c r="H9" s="417" t="n">
+      <c r="H9" s="391" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="I9" s="417" t="n">
         <v>45302</v>
       </c>
-      <c r="I9" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C9,'SAERTEX-prijstabel'!$B$2:$B$496,$D9,'SAERTEX-prijstabel'!$C$2:$C$496,$E9,'SAERTEX-prijstabel'!$D$2:$D$496,$F9),0)</f>
-        <v/>
-      </c>
-      <c r="J9" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G9="","",IF($G9&lt;15,0.25,IF($G9&lt;=50,0.035,IF($G9&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K9" s="392">
-        <f>IF($I9=0,0,$G9*$I9*(1+N($J9)))</f>
-        <v/>
-      </c>
-      <c r="L9" s="401">
-        <f>IF($H9="","nog te plannen",IFERROR(LOOKUP($H9,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J9" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C9,'SAERTEX-prijstabel'!$B$2:$B$496,$D9,'SAERTEX-prijstabel'!$C$2:$C$496,$E9,'SAERTEX-prijstabel'!$D$2:$D$496,$F9),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K9" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G9)+N($H9))=0,0,IF((N($G9)+N($H9))&lt;15,0.25,IF((N($G9)+N($H9))&lt;=50,0.035,IF((N($G9)+N($H9))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L9" s="392">
+        <f>IF($J9=0,0,$G9*$J9*(1+$K9))</f>
+        <v/>
+      </c>
+      <c r="M9" s="392">
+        <f>N($H9)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N9" s="398">
+        <f>$L9+$M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="401">
+        <f>IF($I9="","nog te plannen",IFERROR(LOOKUP($I9,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4884,23 +4982,34 @@
       <c r="G10" s="391" t="n">
         <v>42.1</v>
       </c>
-      <c r="H10" s="417" t="n">
+      <c r="H10" s="391" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="I10" s="417" t="n">
         <v>45304</v>
       </c>
-      <c r="I10" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C10,'SAERTEX-prijstabel'!$B$2:$B$496,$D10,'SAERTEX-prijstabel'!$C$2:$C$496,$E10,'SAERTEX-prijstabel'!$D$2:$D$496,$F10),0)</f>
-        <v/>
-      </c>
-      <c r="J10" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G10="","",IF($G10&lt;15,0.25,IF($G10&lt;=50,0.035,IF($G10&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K10" s="392">
-        <f>IF($I10=0,0,$G10*$I10*(1+N($J10)))</f>
-        <v/>
-      </c>
-      <c r="L10" s="401">
-        <f>IF($H10="","nog te plannen",IFERROR(LOOKUP($H10,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J10" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C10,'SAERTEX-prijstabel'!$B$2:$B$496,$D10,'SAERTEX-prijstabel'!$C$2:$C$496,$E10,'SAERTEX-prijstabel'!$D$2:$D$496,$F10),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K10" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G10)+N($H10))=0,0,IF((N($G10)+N($H10))&lt;15,0.25,IF((N($G10)+N($H10))&lt;=50,0.035,IF((N($G10)+N($H10))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L10" s="392">
+        <f>IF($J10=0,0,$G10*$J10*(1+$K10))</f>
+        <v/>
+      </c>
+      <c r="M10" s="392">
+        <f>N($H10)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N10" s="398">
+        <f>$L10+$M10</f>
+        <v/>
+      </c>
+      <c r="O10" s="401">
+        <f>IF($I10="","nog te plannen",IFERROR(LOOKUP($I10,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4934,23 +5043,34 @@
       <c r="G11" s="391" t="n">
         <v>35.4</v>
       </c>
-      <c r="H11" s="417" t="n">
+      <c r="H11" s="391" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="I11" s="417" t="n">
         <v>45306</v>
       </c>
-      <c r="I11" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C11,'SAERTEX-prijstabel'!$B$2:$B$496,$D11,'SAERTEX-prijstabel'!$C$2:$C$496,$E11,'SAERTEX-prijstabel'!$D$2:$D$496,$F11),0)</f>
-        <v/>
-      </c>
-      <c r="J11" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G11="","",IF($G11&lt;15,0.25,IF($G11&lt;=50,0.035,IF($G11&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K11" s="392">
-        <f>IF($I11=0,0,$G11*$I11*(1+N($J11)))</f>
-        <v/>
-      </c>
-      <c r="L11" s="401">
-        <f>IF($H11="","nog te plannen",IFERROR(LOOKUP($H11,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J11" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C11,'SAERTEX-prijstabel'!$B$2:$B$496,$D11,'SAERTEX-prijstabel'!$C$2:$C$496,$E11,'SAERTEX-prijstabel'!$D$2:$D$496,$F11),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K11" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G11)+N($H11))=0,0,IF((N($G11)+N($H11))&lt;15,0.25,IF((N($G11)+N($H11))&lt;=50,0.035,IF((N($G11)+N($H11))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L11" s="392">
+        <f>IF($J11=0,0,$G11*$J11*(1+$K11))</f>
+        <v/>
+      </c>
+      <c r="M11" s="392">
+        <f>N($H11)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N11" s="398">
+        <f>$L11+$M11</f>
+        <v/>
+      </c>
+      <c r="O11" s="401">
+        <f>IF($I11="","nog te plannen",IFERROR(LOOKUP($I11,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4984,23 +5104,34 @@
       <c r="G12" s="391" t="n">
         <v>41.1</v>
       </c>
-      <c r="H12" s="417" t="n">
+      <c r="H12" s="391" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="I12" s="417" t="n">
         <v>45308</v>
       </c>
-      <c r="I12" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C12,'SAERTEX-prijstabel'!$B$2:$B$496,$D12,'SAERTEX-prijstabel'!$C$2:$C$496,$E12,'SAERTEX-prijstabel'!$D$2:$D$496,$F12),0)</f>
-        <v/>
-      </c>
-      <c r="J12" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G12="","",IF($G12&lt;15,0.25,IF($G12&lt;=50,0.035,IF($G12&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K12" s="392">
-        <f>IF($I12=0,0,$G12*$I12*(1+N($J12)))</f>
-        <v/>
-      </c>
-      <c r="L12" s="401">
-        <f>IF($H12="","nog te plannen",IFERROR(LOOKUP($H12,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J12" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C12,'SAERTEX-prijstabel'!$B$2:$B$496,$D12,'SAERTEX-prijstabel'!$C$2:$C$496,$E12,'SAERTEX-prijstabel'!$D$2:$D$496,$F12),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K12" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G12)+N($H12))=0,0,IF((N($G12)+N($H12))&lt;15,0.25,IF((N($G12)+N($H12))&lt;=50,0.035,IF((N($G12)+N($H12))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L12" s="392">
+        <f>IF($J12=0,0,$G12*$J12*(1+$K12))</f>
+        <v/>
+      </c>
+      <c r="M12" s="392">
+        <f>N($H12)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N12" s="398">
+        <f>$L12+$M12</f>
+        <v/>
+      </c>
+      <c r="O12" s="401">
+        <f>IF($I12="","nog te plannen",IFERROR(LOOKUP($I12,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5034,23 +5165,34 @@
       <c r="G13" s="391" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="H13" s="417" t="n">
+      <c r="H13" s="391" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="I13" s="417" t="n">
         <v>45310</v>
       </c>
-      <c r="I13" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C13,'SAERTEX-prijstabel'!$B$2:$B$496,$D13,'SAERTEX-prijstabel'!$C$2:$C$496,$E13,'SAERTEX-prijstabel'!$D$2:$D$496,$F13),0)</f>
-        <v/>
-      </c>
-      <c r="J13" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G13="","",IF($G13&lt;15,0.25,IF($G13&lt;=50,0.035,IF($G13&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K13" s="392">
-        <f>IF($I13=0,0,$G13*$I13*(1+N($J13)))</f>
-        <v/>
-      </c>
-      <c r="L13" s="401">
-        <f>IF($H13="","nog te plannen",IFERROR(LOOKUP($H13,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J13" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C13,'SAERTEX-prijstabel'!$B$2:$B$496,$D13,'SAERTEX-prijstabel'!$C$2:$C$496,$E13,'SAERTEX-prijstabel'!$D$2:$D$496,$F13),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K13" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G13)+N($H13))=0,0,IF((N($G13)+N($H13))&lt;15,0.25,IF((N($G13)+N($H13))&lt;=50,0.035,IF((N($G13)+N($H13))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L13" s="392">
+        <f>IF($J13=0,0,$G13*$J13*(1+$K13))</f>
+        <v/>
+      </c>
+      <c r="M13" s="392">
+        <f>N($H13)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N13" s="398">
+        <f>$L13+$M13</f>
+        <v/>
+      </c>
+      <c r="O13" s="401">
+        <f>IF($I13="","nog te plannen",IFERROR(LOOKUP($I13,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5084,23 +5226,34 @@
       <c r="G14" s="391" t="n">
         <v>133.9</v>
       </c>
-      <c r="H14" s="417" t="n">
+      <c r="H14" s="391" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I14" s="417" t="n">
         <v>45321</v>
       </c>
-      <c r="I14" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C14,'SAERTEX-prijstabel'!$B$2:$B$496,$D14,'SAERTEX-prijstabel'!$C$2:$C$496,$E14,'SAERTEX-prijstabel'!$D$2:$D$496,$F14),0)</f>
-        <v/>
-      </c>
-      <c r="J14" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G14="","",IF($G14&lt;15,0.25,IF($G14&lt;=50,0.035,IF($G14&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K14" s="392">
-        <f>IF($I14=0,0,$G14*$I14*(1+N($J14)))</f>
-        <v/>
-      </c>
-      <c r="L14" s="401">
-        <f>IF($H14="","nog te plannen",IFERROR(LOOKUP($H14,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J14" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C14,'SAERTEX-prijstabel'!$B$2:$B$496,$D14,'SAERTEX-prijstabel'!$C$2:$C$496,$E14,'SAERTEX-prijstabel'!$D$2:$D$496,$F14),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K14" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G14)+N($H14))=0,0,IF((N($G14)+N($H14))&lt;15,0.25,IF((N($G14)+N($H14))&lt;=50,0.035,IF((N($G14)+N($H14))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L14" s="392">
+        <f>IF($J14=0,0,$G14*$J14*(1+$K14))</f>
+        <v/>
+      </c>
+      <c r="M14" s="392">
+        <f>N($H14)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N14" s="398">
+        <f>$L14+$M14</f>
+        <v/>
+      </c>
+      <c r="O14" s="401">
+        <f>IF($I14="","nog te plannen",IFERROR(LOOKUP($I14,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5134,23 +5287,34 @@
       <c r="G15" s="391" t="n">
         <v>92.3</v>
       </c>
-      <c r="H15" s="417" t="n">
+      <c r="H15" s="391" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="I15" s="417" t="n">
         <v>45324</v>
       </c>
-      <c r="I15" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C15,'SAERTEX-prijstabel'!$B$2:$B$496,$D15,'SAERTEX-prijstabel'!$C$2:$C$496,$E15,'SAERTEX-prijstabel'!$D$2:$D$496,$F15),0)</f>
-        <v/>
-      </c>
-      <c r="J15" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G15="","",IF($G15&lt;15,0.25,IF($G15&lt;=50,0.035,IF($G15&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K15" s="392">
-        <f>IF($I15=0,0,$G15*$I15*(1+N($J15)))</f>
-        <v/>
-      </c>
-      <c r="L15" s="401">
-        <f>IF($H15="","nog te plannen",IFERROR(LOOKUP($H15,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J15" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C15,'SAERTEX-prijstabel'!$B$2:$B$496,$D15,'SAERTEX-prijstabel'!$C$2:$C$496,$E15,'SAERTEX-prijstabel'!$D$2:$D$496,$F15),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K15" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G15)+N($H15))=0,0,IF((N($G15)+N($H15))&lt;15,0.25,IF((N($G15)+N($H15))&lt;=50,0.035,IF((N($G15)+N($H15))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L15" s="392">
+        <f>IF($J15=0,0,$G15*$J15*(1+$K15))</f>
+        <v/>
+      </c>
+      <c r="M15" s="392">
+        <f>N($H15)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N15" s="398">
+        <f>$L15+$M15</f>
+        <v/>
+      </c>
+      <c r="O15" s="401">
+        <f>IF($I15="","nog te plannen",IFERROR(LOOKUP($I15,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5184,23 +5348,34 @@
       <c r="G16" s="391" t="n">
         <v>124.6</v>
       </c>
-      <c r="H16" s="417" t="n">
+      <c r="H16" s="391" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I16" s="417" t="n">
         <v>45327</v>
       </c>
-      <c r="I16" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C16,'SAERTEX-prijstabel'!$B$2:$B$496,$D16,'SAERTEX-prijstabel'!$C$2:$C$496,$E16,'SAERTEX-prijstabel'!$D$2:$D$496,$F16),0)</f>
-        <v/>
-      </c>
-      <c r="J16" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G16="","",IF($G16&lt;15,0.25,IF($G16&lt;=50,0.035,IF($G16&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K16" s="392">
-        <f>IF($I16=0,0,$G16*$I16*(1+N($J16)))</f>
-        <v/>
-      </c>
-      <c r="L16" s="401">
-        <f>IF($H16="","nog te plannen",IFERROR(LOOKUP($H16,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J16" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C16,'SAERTEX-prijstabel'!$B$2:$B$496,$D16,'SAERTEX-prijstabel'!$C$2:$C$496,$E16,'SAERTEX-prijstabel'!$D$2:$D$496,$F16),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K16" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G16)+N($H16))=0,0,IF((N($G16)+N($H16))&lt;15,0.25,IF((N($G16)+N($H16))&lt;=50,0.035,IF((N($G16)+N($H16))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L16" s="392">
+        <f>IF($J16=0,0,$G16*$J16*(1+$K16))</f>
+        <v/>
+      </c>
+      <c r="M16" s="392">
+        <f>N($H16)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N16" s="398">
+        <f>$L16+$M16</f>
+        <v/>
+      </c>
+      <c r="O16" s="401">
+        <f>IF($I16="","nog te plannen",IFERROR(LOOKUP($I16,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5234,23 +5409,34 @@
       <c r="G17" s="391" t="n">
         <v>67</v>
       </c>
-      <c r="H17" s="417" t="n">
+      <c r="H17" s="391" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="I17" s="417" t="n">
         <v>45330</v>
       </c>
-      <c r="I17" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C17,'SAERTEX-prijstabel'!$B$2:$B$496,$D17,'SAERTEX-prijstabel'!$C$2:$C$496,$E17,'SAERTEX-prijstabel'!$D$2:$D$496,$F17),0)</f>
-        <v/>
-      </c>
-      <c r="J17" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G17="","",IF($G17&lt;15,0.25,IF($G17&lt;=50,0.035,IF($G17&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K17" s="392">
-        <f>IF($I17=0,0,$G17*$I17*(1+N($J17)))</f>
-        <v/>
-      </c>
-      <c r="L17" s="401">
-        <f>IF($H17="","nog te plannen",IFERROR(LOOKUP($H17,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J17" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C17,'SAERTEX-prijstabel'!$B$2:$B$496,$D17,'SAERTEX-prijstabel'!$C$2:$C$496,$E17,'SAERTEX-prijstabel'!$D$2:$D$496,$F17),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K17" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G17)+N($H17))=0,0,IF((N($G17)+N($H17))&lt;15,0.25,IF((N($G17)+N($H17))&lt;=50,0.035,IF((N($G17)+N($H17))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L17" s="392">
+        <f>IF($J17=0,0,$G17*$J17*(1+$K17))</f>
+        <v/>
+      </c>
+      <c r="M17" s="392">
+        <f>N($H17)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N17" s="398">
+        <f>$L17+$M17</f>
+        <v/>
+      </c>
+      <c r="O17" s="401">
+        <f>IF($I17="","nog te plannen",IFERROR(LOOKUP($I17,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5284,23 +5470,34 @@
       <c r="G18" s="391" t="n">
         <v>120</v>
       </c>
-      <c r="H18" s="417" t="n">
+      <c r="H18" s="391" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="I18" s="417" t="n">
         <v>45333</v>
       </c>
-      <c r="I18" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C18,'SAERTEX-prijstabel'!$B$2:$B$496,$D18,'SAERTEX-prijstabel'!$C$2:$C$496,$E18,'SAERTEX-prijstabel'!$D$2:$D$496,$F18),0)</f>
-        <v/>
-      </c>
-      <c r="J18" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G18="","",IF($G18&lt;15,0.25,IF($G18&lt;=50,0.035,IF($G18&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K18" s="392">
-        <f>IF($I18=0,0,$G18*$I18*(1+N($J18)))</f>
-        <v/>
-      </c>
-      <c r="L18" s="401">
-        <f>IF($H18="","nog te plannen",IFERROR(LOOKUP($H18,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J18" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C18,'SAERTEX-prijstabel'!$B$2:$B$496,$D18,'SAERTEX-prijstabel'!$C$2:$C$496,$E18,'SAERTEX-prijstabel'!$D$2:$D$496,$F18),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K18" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G18)+N($H18))=0,0,IF((N($G18)+N($H18))&lt;15,0.25,IF((N($G18)+N($H18))&lt;=50,0.035,IF((N($G18)+N($H18))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L18" s="392">
+        <f>IF($J18=0,0,$G18*$J18*(1+$K18))</f>
+        <v/>
+      </c>
+      <c r="M18" s="392">
+        <f>N($H18)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N18" s="398">
+        <f>$L18+$M18</f>
+        <v/>
+      </c>
+      <c r="O18" s="401">
+        <f>IF($I18="","nog te plannen",IFERROR(LOOKUP($I18,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5334,23 +5531,34 @@
       <c r="G19" s="391" t="n">
         <v>66.09999999999999</v>
       </c>
-      <c r="H19" s="417" t="n">
+      <c r="H19" s="391" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="I19" s="417" t="n">
         <v>45336</v>
       </c>
-      <c r="I19" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C19,'SAERTEX-prijstabel'!$B$2:$B$496,$D19,'SAERTEX-prijstabel'!$C$2:$C$496,$E19,'SAERTEX-prijstabel'!$D$2:$D$496,$F19),0)</f>
-        <v/>
-      </c>
-      <c r="J19" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G19="","",IF($G19&lt;15,0.25,IF($G19&lt;=50,0.035,IF($G19&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K19" s="392">
-        <f>IF($I19=0,0,$G19*$I19*(1+N($J19)))</f>
-        <v/>
-      </c>
-      <c r="L19" s="401">
-        <f>IF($H19="","nog te plannen",IFERROR(LOOKUP($H19,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J19" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C19,'SAERTEX-prijstabel'!$B$2:$B$496,$D19,'SAERTEX-prijstabel'!$C$2:$C$496,$E19,'SAERTEX-prijstabel'!$D$2:$D$496,$F19),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K19" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G19)+N($H19))=0,0,IF((N($G19)+N($H19))&lt;15,0.25,IF((N($G19)+N($H19))&lt;=50,0.035,IF((N($G19)+N($H19))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L19" s="392">
+        <f>IF($J19=0,0,$G19*$J19*(1+$K19))</f>
+        <v/>
+      </c>
+      <c r="M19" s="392">
+        <f>N($H19)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N19" s="398">
+        <f>$L19+$M19</f>
+        <v/>
+      </c>
+      <c r="O19" s="401">
+        <f>IF($I19="","nog te plannen",IFERROR(LOOKUP($I19,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5384,23 +5592,34 @@
       <c r="G20" s="391" t="n">
         <v>14.2</v>
       </c>
-      <c r="H20" s="417" t="n">
+      <c r="H20" s="391" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="I20" s="417" t="n">
         <v>45339</v>
       </c>
-      <c r="I20" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C20,'SAERTEX-prijstabel'!$B$2:$B$496,$D20,'SAERTEX-prijstabel'!$C$2:$C$496,$E20,'SAERTEX-prijstabel'!$D$2:$D$496,$F20),0)</f>
-        <v/>
-      </c>
-      <c r="J20" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G20="","",IF($G20&lt;15,0.25,IF($G20&lt;=50,0.035,IF($G20&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K20" s="392">
-        <f>IF($I20=0,0,$G20*$I20*(1+N($J20)))</f>
-        <v/>
-      </c>
-      <c r="L20" s="401">
-        <f>IF($H20="","nog te plannen",IFERROR(LOOKUP($H20,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J20" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C20,'SAERTEX-prijstabel'!$B$2:$B$496,$D20,'SAERTEX-prijstabel'!$C$2:$C$496,$E20,'SAERTEX-prijstabel'!$D$2:$D$496,$F20),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K20" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G20)+N($H20))=0,0,IF((N($G20)+N($H20))&lt;15,0.25,IF((N($G20)+N($H20))&lt;=50,0.035,IF((N($G20)+N($H20))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L20" s="392">
+        <f>IF($J20=0,0,$G20*$J20*(1+$K20))</f>
+        <v/>
+      </c>
+      <c r="M20" s="392">
+        <f>N($H20)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N20" s="398">
+        <f>$L20+$M20</f>
+        <v/>
+      </c>
+      <c r="O20" s="401">
+        <f>IF($I20="","nog te plannen",IFERROR(LOOKUP($I20,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5434,23 +5653,34 @@
       <c r="G21" s="391" t="n">
         <v>49.2</v>
       </c>
-      <c r="H21" s="417" t="n">
+      <c r="H21" s="391" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="I21" s="417" t="n">
         <v>45342</v>
       </c>
-      <c r="I21" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C21,'SAERTEX-prijstabel'!$B$2:$B$496,$D21,'SAERTEX-prijstabel'!$C$2:$C$496,$E21,'SAERTEX-prijstabel'!$D$2:$D$496,$F21),0)</f>
-        <v/>
-      </c>
-      <c r="J21" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G21="","",IF($G21&lt;15,0.25,IF($G21&lt;=50,0.035,IF($G21&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K21" s="392">
-        <f>IF($I21=0,0,$G21*$I21*(1+N($J21)))</f>
-        <v/>
-      </c>
-      <c r="L21" s="401">
-        <f>IF($H21="","nog te plannen",IFERROR(LOOKUP($H21,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J21" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C21,'SAERTEX-prijstabel'!$B$2:$B$496,$D21,'SAERTEX-prijstabel'!$C$2:$C$496,$E21,'SAERTEX-prijstabel'!$D$2:$D$496,$F21),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K21" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G21)+N($H21))=0,0,IF((N($G21)+N($H21))&lt;15,0.25,IF((N($G21)+N($H21))&lt;=50,0.035,IF((N($G21)+N($H21))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L21" s="392">
+        <f>IF($J21=0,0,$G21*$J21*(1+$K21))</f>
+        <v/>
+      </c>
+      <c r="M21" s="392">
+        <f>N($H21)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N21" s="398">
+        <f>$L21+$M21</f>
+        <v/>
+      </c>
+      <c r="O21" s="401">
+        <f>IF($I21="","nog te plannen",IFERROR(LOOKUP($I21,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5476,7 +5706,7 @@
         </is>
       </c>
       <c r="E22" s="306" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="F22" s="306" t="n">
         <v>6</v>
@@ -5484,23 +5714,34 @@
       <c r="G22" s="391" t="n">
         <v>54.3</v>
       </c>
-      <c r="H22" s="417" t="n">
+      <c r="H22" s="391" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="I22" s="417" t="n">
         <v>45349</v>
       </c>
-      <c r="I22" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C22,'SAERTEX-prijstabel'!$B$2:$B$496,$D22,'SAERTEX-prijstabel'!$C$2:$C$496,$E22,'SAERTEX-prijstabel'!$D$2:$D$496,$F22),0)</f>
-        <v/>
-      </c>
-      <c r="J22" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G22="","",IF($G22&lt;15,0.25,IF($G22&lt;=50,0.035,IF($G22&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K22" s="392">
-        <f>IF($I22=0,0,$G22*$I22*(1+N($J22)))</f>
-        <v/>
-      </c>
-      <c r="L22" s="401">
-        <f>IF($H22="","nog te plannen",IFERROR(LOOKUP($H22,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J22" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C22,'SAERTEX-prijstabel'!$B$2:$B$496,$D22,'SAERTEX-prijstabel'!$C$2:$C$496,$E22,'SAERTEX-prijstabel'!$D$2:$D$496,$F22),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K22" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G22)+N($H22))=0,0,IF((N($G22)+N($H22))&lt;15,0.25,IF((N($G22)+N($H22))&lt;=50,0.035,IF((N($G22)+N($H22))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L22" s="392">
+        <f>IF($J22=0,0,$G22*$J22*(1+$K22))</f>
+        <v/>
+      </c>
+      <c r="M22" s="392">
+        <f>N($H22)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N22" s="398">
+        <f>$L22+$M22</f>
+        <v/>
+      </c>
+      <c r="O22" s="401">
+        <f>IF($I22="","nog te plannen",IFERROR(LOOKUP($I22,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5534,23 +5775,34 @@
       <c r="G23" s="391" t="n">
         <v>123.6</v>
       </c>
-      <c r="H23" s="417" t="n">
+      <c r="H23" s="391" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="I23" s="417" t="n">
         <v>45352</v>
       </c>
-      <c r="I23" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C23,'SAERTEX-prijstabel'!$B$2:$B$496,$D23,'SAERTEX-prijstabel'!$C$2:$C$496,$E23,'SAERTEX-prijstabel'!$D$2:$D$496,$F23),0)</f>
-        <v/>
-      </c>
-      <c r="J23" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G23="","",IF($G23&lt;15,0.25,IF($G23&lt;=50,0.035,IF($G23&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K23" s="392">
-        <f>IF($I23=0,0,$G23*$I23*(1+N($J23)))</f>
-        <v/>
-      </c>
-      <c r="L23" s="401">
-        <f>IF($H23="","nog te plannen",IFERROR(LOOKUP($H23,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J23" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C23,'SAERTEX-prijstabel'!$B$2:$B$496,$D23,'SAERTEX-prijstabel'!$C$2:$C$496,$E23,'SAERTEX-prijstabel'!$D$2:$D$496,$F23),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K23" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G23)+N($H23))=0,0,IF((N($G23)+N($H23))&lt;15,0.25,IF((N($G23)+N($H23))&lt;=50,0.035,IF((N($G23)+N($H23))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L23" s="392">
+        <f>IF($J23=0,0,$G23*$J23*(1+$K23))</f>
+        <v/>
+      </c>
+      <c r="M23" s="392">
+        <f>N($H23)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N23" s="398">
+        <f>$L23+$M23</f>
+        <v/>
+      </c>
+      <c r="O23" s="401">
+        <f>IF($I23="","nog te plannen",IFERROR(LOOKUP($I23,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5584,23 +5836,34 @@
       <c r="G24" s="391" t="n">
         <v>87.59999999999999</v>
       </c>
-      <c r="H24" s="417" t="n">
+      <c r="H24" s="391" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I24" s="417" t="n">
         <v>45355</v>
       </c>
-      <c r="I24" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C24,'SAERTEX-prijstabel'!$B$2:$B$496,$D24,'SAERTEX-prijstabel'!$C$2:$C$496,$E24,'SAERTEX-prijstabel'!$D$2:$D$496,$F24),0)</f>
-        <v/>
-      </c>
-      <c r="J24" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G24="","",IF($G24&lt;15,0.25,IF($G24&lt;=50,0.035,IF($G24&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K24" s="392">
-        <f>IF($I24=0,0,$G24*$I24*(1+N($J24)))</f>
-        <v/>
-      </c>
-      <c r="L24" s="401">
-        <f>IF($H24="","nog te plannen",IFERROR(LOOKUP($H24,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J24" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C24,'SAERTEX-prijstabel'!$B$2:$B$496,$D24,'SAERTEX-prijstabel'!$C$2:$C$496,$E24,'SAERTEX-prijstabel'!$D$2:$D$496,$F24),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K24" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G24)+N($H24))=0,0,IF((N($G24)+N($H24))&lt;15,0.25,IF((N($G24)+N($H24))&lt;=50,0.035,IF((N($G24)+N($H24))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L24" s="392">
+        <f>IF($J24=0,0,$G24*$J24*(1+$K24))</f>
+        <v/>
+      </c>
+      <c r="M24" s="392">
+        <f>N($H24)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N24" s="398">
+        <f>$L24+$M24</f>
+        <v/>
+      </c>
+      <c r="O24" s="401">
+        <f>IF($I24="","nog te plannen",IFERROR(LOOKUP($I24,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5634,23 +5897,34 @@
       <c r="G25" s="391" t="n">
         <v>121.4</v>
       </c>
-      <c r="H25" s="417" t="n">
+      <c r="H25" s="391" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="I25" s="417" t="n">
         <v>45358</v>
       </c>
-      <c r="I25" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C25,'SAERTEX-prijstabel'!$B$2:$B$496,$D25,'SAERTEX-prijstabel'!$C$2:$C$496,$E25,'SAERTEX-prijstabel'!$D$2:$D$496,$F25),0)</f>
-        <v/>
-      </c>
-      <c r="J25" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G25="","",IF($G25&lt;15,0.25,IF($G25&lt;=50,0.035,IF($G25&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K25" s="392">
-        <f>IF($I25=0,0,$G25*$I25*(1+N($J25)))</f>
-        <v/>
-      </c>
-      <c r="L25" s="401">
-        <f>IF($H25="","nog te plannen",IFERROR(LOOKUP($H25,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J25" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C25,'SAERTEX-prijstabel'!$B$2:$B$496,$D25,'SAERTEX-prijstabel'!$C$2:$C$496,$E25,'SAERTEX-prijstabel'!$D$2:$D$496,$F25),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K25" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G25)+N($H25))=0,0,IF((N($G25)+N($H25))&lt;15,0.25,IF((N($G25)+N($H25))&lt;=50,0.035,IF((N($G25)+N($H25))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L25" s="392">
+        <f>IF($J25=0,0,$G25*$J25*(1+$K25))</f>
+        <v/>
+      </c>
+      <c r="M25" s="392">
+        <f>N($H25)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N25" s="398">
+        <f>$L25+$M25</f>
+        <v/>
+      </c>
+      <c r="O25" s="401">
+        <f>IF($I25="","nog te plannen",IFERROR(LOOKUP($I25,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5684,23 +5958,34 @@
       <c r="G26" s="391" t="n">
         <v>93.8</v>
       </c>
-      <c r="H26" s="417" t="n">
+      <c r="H26" s="391" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="I26" s="417" t="n">
         <v>45361</v>
       </c>
-      <c r="I26" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C26,'SAERTEX-prijstabel'!$B$2:$B$496,$D26,'SAERTEX-prijstabel'!$C$2:$C$496,$E26,'SAERTEX-prijstabel'!$D$2:$D$496,$F26),0)</f>
-        <v/>
-      </c>
-      <c r="J26" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G26="","",IF($G26&lt;15,0.25,IF($G26&lt;=50,0.035,IF($G26&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K26" s="392">
-        <f>IF($I26=0,0,$G26*$I26*(1+N($J26)))</f>
-        <v/>
-      </c>
-      <c r="L26" s="401">
-        <f>IF($H26="","nog te plannen",IFERROR(LOOKUP($H26,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J26" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C26,'SAERTEX-prijstabel'!$B$2:$B$496,$D26,'SAERTEX-prijstabel'!$C$2:$C$496,$E26,'SAERTEX-prijstabel'!$D$2:$D$496,$F26),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K26" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G26)+N($H26))=0,0,IF((N($G26)+N($H26))&lt;15,0.25,IF((N($G26)+N($H26))&lt;=50,0.035,IF((N($G26)+N($H26))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L26" s="392">
+        <f>IF($J26=0,0,$G26*$J26*(1+$K26))</f>
+        <v/>
+      </c>
+      <c r="M26" s="392">
+        <f>N($H26)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N26" s="398">
+        <f>$L26+$M26</f>
+        <v/>
+      </c>
+      <c r="O26" s="401">
+        <f>IF($I26="","nog te plannen",IFERROR(LOOKUP($I26,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5734,23 +6019,34 @@
       <c r="G27" s="391" t="n">
         <v>60.9</v>
       </c>
-      <c r="H27" s="417" t="n">
+      <c r="H27" s="391" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="I27" s="417" t="n">
         <v>45364</v>
       </c>
-      <c r="I27" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C27,'SAERTEX-prijstabel'!$B$2:$B$496,$D27,'SAERTEX-prijstabel'!$C$2:$C$496,$E27,'SAERTEX-prijstabel'!$D$2:$D$496,$F27),0)</f>
-        <v/>
-      </c>
-      <c r="J27" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G27="","",IF($G27&lt;15,0.25,IF($G27&lt;=50,0.035,IF($G27&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K27" s="392">
-        <f>IF($I27=0,0,$G27*$I27*(1+N($J27)))</f>
-        <v/>
-      </c>
-      <c r="L27" s="401">
-        <f>IF($H27="","nog te plannen",IFERROR(LOOKUP($H27,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J27" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C27,'SAERTEX-prijstabel'!$B$2:$B$496,$D27,'SAERTEX-prijstabel'!$C$2:$C$496,$E27,'SAERTEX-prijstabel'!$D$2:$D$496,$F27),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K27" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G27)+N($H27))=0,0,IF((N($G27)+N($H27))&lt;15,0.25,IF((N($G27)+N($H27))&lt;=50,0.035,IF((N($G27)+N($H27))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L27" s="392">
+        <f>IF($J27=0,0,$G27*$J27*(1+$K27))</f>
+        <v/>
+      </c>
+      <c r="M27" s="392">
+        <f>N($H27)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N27" s="398">
+        <f>$L27+$M27</f>
+        <v/>
+      </c>
+      <c r="O27" s="401">
+        <f>IF($I27="","nog te plannen",IFERROR(LOOKUP($I27,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5784,23 +6080,34 @@
       <c r="G28" s="391" t="n">
         <v>49.2</v>
       </c>
-      <c r="H28" s="417" t="n">
+      <c r="H28" s="391" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I28" s="417" t="n">
         <v>45367</v>
       </c>
-      <c r="I28" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C28,'SAERTEX-prijstabel'!$B$2:$B$496,$D28,'SAERTEX-prijstabel'!$C$2:$C$496,$E28,'SAERTEX-prijstabel'!$D$2:$D$496,$F28),0)</f>
-        <v/>
-      </c>
-      <c r="J28" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G28="","",IF($G28&lt;15,0.25,IF($G28&lt;=50,0.035,IF($G28&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K28" s="392">
-        <f>IF($I28=0,0,$G28*$I28*(1+N($J28)))</f>
-        <v/>
-      </c>
-      <c r="L28" s="401">
-        <f>IF($H28="","nog te plannen",IFERROR(LOOKUP($H28,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J28" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C28,'SAERTEX-prijstabel'!$B$2:$B$496,$D28,'SAERTEX-prijstabel'!$C$2:$C$496,$E28,'SAERTEX-prijstabel'!$D$2:$D$496,$F28),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K28" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G28)+N($H28))=0,0,IF((N($G28)+N($H28))&lt;15,0.25,IF((N($G28)+N($H28))&lt;=50,0.035,IF((N($G28)+N($H28))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L28" s="392">
+        <f>IF($J28=0,0,$G28*$J28*(1+$K28))</f>
+        <v/>
+      </c>
+      <c r="M28" s="392">
+        <f>N($H28)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N28" s="398">
+        <f>$L28+$M28</f>
+        <v/>
+      </c>
+      <c r="O28" s="401">
+        <f>IF($I28="","nog te plannen",IFERROR(LOOKUP($I28,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5834,23 +6141,34 @@
       <c r="G29" s="391" t="n">
         <v>106.1</v>
       </c>
-      <c r="H29" s="417" t="n">
+      <c r="H29" s="391" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I29" s="417" t="n">
         <v>45370</v>
       </c>
-      <c r="I29" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C29,'SAERTEX-prijstabel'!$B$2:$B$496,$D29,'SAERTEX-prijstabel'!$C$2:$C$496,$E29,'SAERTEX-prijstabel'!$D$2:$D$496,$F29),0)</f>
-        <v/>
-      </c>
-      <c r="J29" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G29="","",IF($G29&lt;15,0.25,IF($G29&lt;=50,0.035,IF($G29&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K29" s="392">
-        <f>IF($I29=0,0,$G29*$I29*(1+N($J29)))</f>
-        <v/>
-      </c>
-      <c r="L29" s="401">
-        <f>IF($H29="","nog te plannen",IFERROR(LOOKUP($H29,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J29" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C29,'SAERTEX-prijstabel'!$B$2:$B$496,$D29,'SAERTEX-prijstabel'!$C$2:$C$496,$E29,'SAERTEX-prijstabel'!$D$2:$D$496,$F29),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K29" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G29)+N($H29))=0,0,IF((N($G29)+N($H29))&lt;15,0.25,IF((N($G29)+N($H29))&lt;=50,0.035,IF((N($G29)+N($H29))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L29" s="392">
+        <f>IF($J29=0,0,$G29*$J29*(1+$K29))</f>
+        <v/>
+      </c>
+      <c r="M29" s="392">
+        <f>N($H29)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N29" s="398">
+        <f>$L29+$M29</f>
+        <v/>
+      </c>
+      <c r="O29" s="401">
+        <f>IF($I29="","nog te plannen",IFERROR(LOOKUP($I29,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5862,21 +6180,30 @@
       <c r="E30" s="306" t="n"/>
       <c r="F30" s="306" t="n"/>
       <c r="G30" s="391" t="n"/>
-      <c r="H30" s="388" t="n"/>
-      <c r="I30" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C30,'SAERTEX-prijstabel'!$B$2:$B$496,$D30,'SAERTEX-prijstabel'!$C$2:$C$496,$E30,'SAERTEX-prijstabel'!$D$2:$D$496,$F30),0)</f>
-        <v/>
-      </c>
-      <c r="J30" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G30="","",IF($G30&lt;15,0.25,IF($G30&lt;=50,0.035,IF($G30&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K30" s="392">
-        <f>IF($I30=0,0,$G30*$I30*(1+N($J30)))</f>
-        <v/>
-      </c>
-      <c r="L30" s="401">
-        <f>IF($H30="","nog te plannen",IFERROR(LOOKUP($H30,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H30" s="391" t="n"/>
+      <c r="I30" s="388" t="n"/>
+      <c r="J30" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C30,'SAERTEX-prijstabel'!$B$2:$B$496,$D30,'SAERTEX-prijstabel'!$C$2:$C$496,$E30,'SAERTEX-prijstabel'!$D$2:$D$496,$F30),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K30" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G30)+N($H30))=0,0,IF((N($G30)+N($H30))&lt;15,0.25,IF((N($G30)+N($H30))&lt;=50,0.035,IF((N($G30)+N($H30))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L30" s="392">
+        <f>IF($J30=0,0,$G30*$J30*(1+$K30))</f>
+        <v/>
+      </c>
+      <c r="M30" s="392">
+        <f>N($H30)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N30" s="398">
+        <f>$L30+$M30</f>
+        <v/>
+      </c>
+      <c r="O30" s="401">
+        <f>IF($I30="","nog te plannen",IFERROR(LOOKUP($I30,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5888,21 +6215,30 @@
       <c r="E31" s="306" t="n"/>
       <c r="F31" s="306" t="n"/>
       <c r="G31" s="391" t="n"/>
-      <c r="H31" s="388" t="n"/>
-      <c r="I31" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C31,'SAERTEX-prijstabel'!$B$2:$B$496,$D31,'SAERTEX-prijstabel'!$C$2:$C$496,$E31,'SAERTEX-prijstabel'!$D$2:$D$496,$F31),0)</f>
-        <v/>
-      </c>
-      <c r="J31" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G31="","",IF($G31&lt;15,0.25,IF($G31&lt;=50,0.035,IF($G31&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K31" s="392">
-        <f>IF($I31=0,0,$G31*$I31*(1+N($J31)))</f>
-        <v/>
-      </c>
-      <c r="L31" s="401">
-        <f>IF($H31="","nog te plannen",IFERROR(LOOKUP($H31,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H31" s="391" t="n"/>
+      <c r="I31" s="388" t="n"/>
+      <c r="J31" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C31,'SAERTEX-prijstabel'!$B$2:$B$496,$D31,'SAERTEX-prijstabel'!$C$2:$C$496,$E31,'SAERTEX-prijstabel'!$D$2:$D$496,$F31),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K31" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G31)+N($H31))=0,0,IF((N($G31)+N($H31))&lt;15,0.25,IF((N($G31)+N($H31))&lt;=50,0.035,IF((N($G31)+N($H31))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L31" s="392">
+        <f>IF($J31=0,0,$G31*$J31*(1+$K31))</f>
+        <v/>
+      </c>
+      <c r="M31" s="392">
+        <f>N($H31)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N31" s="398">
+        <f>$L31+$M31</f>
+        <v/>
+      </c>
+      <c r="O31" s="401">
+        <f>IF($I31="","nog te plannen",IFERROR(LOOKUP($I31,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5914,21 +6250,30 @@
       <c r="E32" s="306" t="n"/>
       <c r="F32" s="306" t="n"/>
       <c r="G32" s="391" t="n"/>
-      <c r="H32" s="388" t="n"/>
-      <c r="I32" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C32,'SAERTEX-prijstabel'!$B$2:$B$496,$D32,'SAERTEX-prijstabel'!$C$2:$C$496,$E32,'SAERTEX-prijstabel'!$D$2:$D$496,$F32),0)</f>
-        <v/>
-      </c>
-      <c r="J32" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G32="","",IF($G32&lt;15,0.25,IF($G32&lt;=50,0.035,IF($G32&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K32" s="392">
-        <f>IF($I32=0,0,$G32*$I32*(1+N($J32)))</f>
-        <v/>
-      </c>
-      <c r="L32" s="401">
-        <f>IF($H32="","nog te plannen",IFERROR(LOOKUP($H32,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H32" s="391" t="n"/>
+      <c r="I32" s="388" t="n"/>
+      <c r="J32" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C32,'SAERTEX-prijstabel'!$B$2:$B$496,$D32,'SAERTEX-prijstabel'!$C$2:$C$496,$E32,'SAERTEX-prijstabel'!$D$2:$D$496,$F32),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K32" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G32)+N($H32))=0,0,IF((N($G32)+N($H32))&lt;15,0.25,IF((N($G32)+N($H32))&lt;=50,0.035,IF((N($G32)+N($H32))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L32" s="392">
+        <f>IF($J32=0,0,$G32*$J32*(1+$K32))</f>
+        <v/>
+      </c>
+      <c r="M32" s="392">
+        <f>N($H32)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N32" s="398">
+        <f>$L32+$M32</f>
+        <v/>
+      </c>
+      <c r="O32" s="401">
+        <f>IF($I32="","nog te plannen",IFERROR(LOOKUP($I32,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5940,21 +6285,30 @@
       <c r="E33" s="306" t="n"/>
       <c r="F33" s="306" t="n"/>
       <c r="G33" s="391" t="n"/>
-      <c r="H33" s="388" t="n"/>
-      <c r="I33" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C33,'SAERTEX-prijstabel'!$B$2:$B$496,$D33,'SAERTEX-prijstabel'!$C$2:$C$496,$E33,'SAERTEX-prijstabel'!$D$2:$D$496,$F33),0)</f>
-        <v/>
-      </c>
-      <c r="J33" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G33="","",IF($G33&lt;15,0.25,IF($G33&lt;=50,0.035,IF($G33&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K33" s="392">
-        <f>IF($I33=0,0,$G33*$I33*(1+N($J33)))</f>
-        <v/>
-      </c>
-      <c r="L33" s="401">
-        <f>IF($H33="","nog te plannen",IFERROR(LOOKUP($H33,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H33" s="391" t="n"/>
+      <c r="I33" s="388" t="n"/>
+      <c r="J33" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C33,'SAERTEX-prijstabel'!$B$2:$B$496,$D33,'SAERTEX-prijstabel'!$C$2:$C$496,$E33,'SAERTEX-prijstabel'!$D$2:$D$496,$F33),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K33" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G33)+N($H33))=0,0,IF((N($G33)+N($H33))&lt;15,0.25,IF((N($G33)+N($H33))&lt;=50,0.035,IF((N($G33)+N($H33))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L33" s="392">
+        <f>IF($J33=0,0,$G33*$J33*(1+$K33))</f>
+        <v/>
+      </c>
+      <c r="M33" s="392">
+        <f>N($H33)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N33" s="398">
+        <f>$L33+$M33</f>
+        <v/>
+      </c>
+      <c r="O33" s="401">
+        <f>IF($I33="","nog te plannen",IFERROR(LOOKUP($I33,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5966,21 +6320,30 @@
       <c r="E34" s="306" t="n"/>
       <c r="F34" s="306" t="n"/>
       <c r="G34" s="391" t="n"/>
-      <c r="H34" s="388" t="n"/>
-      <c r="I34" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C34,'SAERTEX-prijstabel'!$B$2:$B$496,$D34,'SAERTEX-prijstabel'!$C$2:$C$496,$E34,'SAERTEX-prijstabel'!$D$2:$D$496,$F34),0)</f>
-        <v/>
-      </c>
-      <c r="J34" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G34="","",IF($G34&lt;15,0.25,IF($G34&lt;=50,0.035,IF($G34&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K34" s="392">
-        <f>IF($I34=0,0,$G34*$I34*(1+N($J34)))</f>
-        <v/>
-      </c>
-      <c r="L34" s="401">
-        <f>IF($H34="","nog te plannen",IFERROR(LOOKUP($H34,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H34" s="391" t="n"/>
+      <c r="I34" s="388" t="n"/>
+      <c r="J34" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C34,'SAERTEX-prijstabel'!$B$2:$B$496,$D34,'SAERTEX-prijstabel'!$C$2:$C$496,$E34,'SAERTEX-prijstabel'!$D$2:$D$496,$F34),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K34" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G34)+N($H34))=0,0,IF((N($G34)+N($H34))&lt;15,0.25,IF((N($G34)+N($H34))&lt;=50,0.035,IF((N($G34)+N($H34))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L34" s="392">
+        <f>IF($J34=0,0,$G34*$J34*(1+$K34))</f>
+        <v/>
+      </c>
+      <c r="M34" s="392">
+        <f>N($H34)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N34" s="398">
+        <f>$L34+$M34</f>
+        <v/>
+      </c>
+      <c r="O34" s="401">
+        <f>IF($I34="","nog te plannen",IFERROR(LOOKUP($I34,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5992,21 +6355,30 @@
       <c r="E35" s="306" t="n"/>
       <c r="F35" s="306" t="n"/>
       <c r="G35" s="391" t="n"/>
-      <c r="H35" s="388" t="n"/>
-      <c r="I35" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C35,'SAERTEX-prijstabel'!$B$2:$B$496,$D35,'SAERTEX-prijstabel'!$C$2:$C$496,$E35,'SAERTEX-prijstabel'!$D$2:$D$496,$F35),0)</f>
-        <v/>
-      </c>
-      <c r="J35" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G35="","",IF($G35&lt;15,0.25,IF($G35&lt;=50,0.035,IF($G35&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K35" s="392">
-        <f>IF($I35=0,0,$G35*$I35*(1+N($J35)))</f>
-        <v/>
-      </c>
-      <c r="L35" s="401">
-        <f>IF($H35="","nog te plannen",IFERROR(LOOKUP($H35,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H35" s="391" t="n"/>
+      <c r="I35" s="388" t="n"/>
+      <c r="J35" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C35,'SAERTEX-prijstabel'!$B$2:$B$496,$D35,'SAERTEX-prijstabel'!$C$2:$C$496,$E35,'SAERTEX-prijstabel'!$D$2:$D$496,$F35),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K35" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G35)+N($H35))=0,0,IF((N($G35)+N($H35))&lt;15,0.25,IF((N($G35)+N($H35))&lt;=50,0.035,IF((N($G35)+N($H35))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L35" s="392">
+        <f>IF($J35=0,0,$G35*$J35*(1+$K35))</f>
+        <v/>
+      </c>
+      <c r="M35" s="392">
+        <f>N($H35)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N35" s="398">
+        <f>$L35+$M35</f>
+        <v/>
+      </c>
+      <c r="O35" s="401">
+        <f>IF($I35="","nog te plannen",IFERROR(LOOKUP($I35,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6018,21 +6390,30 @@
       <c r="E36" s="306" t="n"/>
       <c r="F36" s="306" t="n"/>
       <c r="G36" s="391" t="n"/>
-      <c r="H36" s="388" t="n"/>
-      <c r="I36" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C36,'SAERTEX-prijstabel'!$B$2:$B$496,$D36,'SAERTEX-prijstabel'!$C$2:$C$496,$E36,'SAERTEX-prijstabel'!$D$2:$D$496,$F36),0)</f>
-        <v/>
-      </c>
-      <c r="J36" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G36="","",IF($G36&lt;15,0.25,IF($G36&lt;=50,0.035,IF($G36&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K36" s="392">
-        <f>IF($I36=0,0,$G36*$I36*(1+N($J36)))</f>
-        <v/>
-      </c>
-      <c r="L36" s="401">
-        <f>IF($H36="","nog te plannen",IFERROR(LOOKUP($H36,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H36" s="391" t="n"/>
+      <c r="I36" s="388" t="n"/>
+      <c r="J36" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C36,'SAERTEX-prijstabel'!$B$2:$B$496,$D36,'SAERTEX-prijstabel'!$C$2:$C$496,$E36,'SAERTEX-prijstabel'!$D$2:$D$496,$F36),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K36" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G36)+N($H36))=0,0,IF((N($G36)+N($H36))&lt;15,0.25,IF((N($G36)+N($H36))&lt;=50,0.035,IF((N($G36)+N($H36))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L36" s="392">
+        <f>IF($J36=0,0,$G36*$J36*(1+$K36))</f>
+        <v/>
+      </c>
+      <c r="M36" s="392">
+        <f>N($H36)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N36" s="398">
+        <f>$L36+$M36</f>
+        <v/>
+      </c>
+      <c r="O36" s="401">
+        <f>IF($I36="","nog te plannen",IFERROR(LOOKUP($I36,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6044,21 +6425,30 @@
       <c r="E37" s="306" t="n"/>
       <c r="F37" s="306" t="n"/>
       <c r="G37" s="391" t="n"/>
-      <c r="H37" s="388" t="n"/>
-      <c r="I37" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C37,'SAERTEX-prijstabel'!$B$2:$B$496,$D37,'SAERTEX-prijstabel'!$C$2:$C$496,$E37,'SAERTEX-prijstabel'!$D$2:$D$496,$F37),0)</f>
-        <v/>
-      </c>
-      <c r="J37" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G37="","",IF($G37&lt;15,0.25,IF($G37&lt;=50,0.035,IF($G37&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K37" s="392">
-        <f>IF($I37=0,0,$G37*$I37*(1+N($J37)))</f>
-        <v/>
-      </c>
-      <c r="L37" s="401">
-        <f>IF($H37="","nog te plannen",IFERROR(LOOKUP($H37,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H37" s="391" t="n"/>
+      <c r="I37" s="388" t="n"/>
+      <c r="J37" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C37,'SAERTEX-prijstabel'!$B$2:$B$496,$D37,'SAERTEX-prijstabel'!$C$2:$C$496,$E37,'SAERTEX-prijstabel'!$D$2:$D$496,$F37),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K37" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G37)+N($H37))=0,0,IF((N($G37)+N($H37))&lt;15,0.25,IF((N($G37)+N($H37))&lt;=50,0.035,IF((N($G37)+N($H37))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L37" s="392">
+        <f>IF($J37=0,0,$G37*$J37*(1+$K37))</f>
+        <v/>
+      </c>
+      <c r="M37" s="392">
+        <f>N($H37)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N37" s="398">
+        <f>$L37+$M37</f>
+        <v/>
+      </c>
+      <c r="O37" s="401">
+        <f>IF($I37="","nog te plannen",IFERROR(LOOKUP($I37,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6070,21 +6460,30 @@
       <c r="E38" s="306" t="n"/>
       <c r="F38" s="306" t="n"/>
       <c r="G38" s="391" t="n"/>
-      <c r="H38" s="388" t="n"/>
-      <c r="I38" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C38,'SAERTEX-prijstabel'!$B$2:$B$496,$D38,'SAERTEX-prijstabel'!$C$2:$C$496,$E38,'SAERTEX-prijstabel'!$D$2:$D$496,$F38),0)</f>
-        <v/>
-      </c>
-      <c r="J38" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G38="","",IF($G38&lt;15,0.25,IF($G38&lt;=50,0.035,IF($G38&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K38" s="392">
-        <f>IF($I38=0,0,$G38*$I38*(1+N($J38)))</f>
-        <v/>
-      </c>
-      <c r="L38" s="401">
-        <f>IF($H38="","nog te plannen",IFERROR(LOOKUP($H38,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H38" s="391" t="n"/>
+      <c r="I38" s="388" t="n"/>
+      <c r="J38" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C38,'SAERTEX-prijstabel'!$B$2:$B$496,$D38,'SAERTEX-prijstabel'!$C$2:$C$496,$E38,'SAERTEX-prijstabel'!$D$2:$D$496,$F38),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K38" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G38)+N($H38))=0,0,IF((N($G38)+N($H38))&lt;15,0.25,IF((N($G38)+N($H38))&lt;=50,0.035,IF((N($G38)+N($H38))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L38" s="392">
+        <f>IF($J38=0,0,$G38*$J38*(1+$K38))</f>
+        <v/>
+      </c>
+      <c r="M38" s="392">
+        <f>N($H38)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N38" s="398">
+        <f>$L38+$M38</f>
+        <v/>
+      </c>
+      <c r="O38" s="401">
+        <f>IF($I38="","nog te plannen",IFERROR(LOOKUP($I38,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6096,21 +6495,30 @@
       <c r="E39" s="306" t="n"/>
       <c r="F39" s="306" t="n"/>
       <c r="G39" s="391" t="n"/>
-      <c r="H39" s="388" t="n"/>
-      <c r="I39" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C39,'SAERTEX-prijstabel'!$B$2:$B$496,$D39,'SAERTEX-prijstabel'!$C$2:$C$496,$E39,'SAERTEX-prijstabel'!$D$2:$D$496,$F39),0)</f>
-        <v/>
-      </c>
-      <c r="J39" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G39="","",IF($G39&lt;15,0.25,IF($G39&lt;=50,0.035,IF($G39&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K39" s="392">
-        <f>IF($I39=0,0,$G39*$I39*(1+N($J39)))</f>
-        <v/>
-      </c>
-      <c r="L39" s="401">
-        <f>IF($H39="","nog te plannen",IFERROR(LOOKUP($H39,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H39" s="391" t="n"/>
+      <c r="I39" s="388" t="n"/>
+      <c r="J39" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C39,'SAERTEX-prijstabel'!$B$2:$B$496,$D39,'SAERTEX-prijstabel'!$C$2:$C$496,$E39,'SAERTEX-prijstabel'!$D$2:$D$496,$F39),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K39" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G39)+N($H39))=0,0,IF((N($G39)+N($H39))&lt;15,0.25,IF((N($G39)+N($H39))&lt;=50,0.035,IF((N($G39)+N($H39))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L39" s="392">
+        <f>IF($J39=0,0,$G39*$J39*(1+$K39))</f>
+        <v/>
+      </c>
+      <c r="M39" s="392">
+        <f>N($H39)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N39" s="398">
+        <f>$L39+$M39</f>
+        <v/>
+      </c>
+      <c r="O39" s="401">
+        <f>IF($I39="","nog te plannen",IFERROR(LOOKUP($I39,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6122,21 +6530,30 @@
       <c r="E40" s="306" t="n"/>
       <c r="F40" s="306" t="n"/>
       <c r="G40" s="391" t="n"/>
-      <c r="H40" s="388" t="n"/>
-      <c r="I40" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C40,'SAERTEX-prijstabel'!$B$2:$B$496,$D40,'SAERTEX-prijstabel'!$C$2:$C$496,$E40,'SAERTEX-prijstabel'!$D$2:$D$496,$F40),0)</f>
-        <v/>
-      </c>
-      <c r="J40" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G40="","",IF($G40&lt;15,0.25,IF($G40&lt;=50,0.035,IF($G40&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K40" s="392">
-        <f>IF($I40=0,0,$G40*$I40*(1+N($J40)))</f>
-        <v/>
-      </c>
-      <c r="L40" s="401">
-        <f>IF($H40="","nog te plannen",IFERROR(LOOKUP($H40,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H40" s="391" t="n"/>
+      <c r="I40" s="388" t="n"/>
+      <c r="J40" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C40,'SAERTEX-prijstabel'!$B$2:$B$496,$D40,'SAERTEX-prijstabel'!$C$2:$C$496,$E40,'SAERTEX-prijstabel'!$D$2:$D$496,$F40),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K40" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G40)+N($H40))=0,0,IF((N($G40)+N($H40))&lt;15,0.25,IF((N($G40)+N($H40))&lt;=50,0.035,IF((N($G40)+N($H40))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L40" s="392">
+        <f>IF($J40=0,0,$G40*$J40*(1+$K40))</f>
+        <v/>
+      </c>
+      <c r="M40" s="392">
+        <f>N($H40)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N40" s="398">
+        <f>$L40+$M40</f>
+        <v/>
+      </c>
+      <c r="O40" s="401">
+        <f>IF($I40="","nog te plannen",IFERROR(LOOKUP($I40,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6148,21 +6565,30 @@
       <c r="E41" s="306" t="n"/>
       <c r="F41" s="306" t="n"/>
       <c r="G41" s="391" t="n"/>
-      <c r="H41" s="388" t="n"/>
-      <c r="I41" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C41,'SAERTEX-prijstabel'!$B$2:$B$496,$D41,'SAERTEX-prijstabel'!$C$2:$C$496,$E41,'SAERTEX-prijstabel'!$D$2:$D$496,$F41),0)</f>
-        <v/>
-      </c>
-      <c r="J41" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G41="","",IF($G41&lt;15,0.25,IF($G41&lt;=50,0.035,IF($G41&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K41" s="392">
-        <f>IF($I41=0,0,$G41*$I41*(1+N($J41)))</f>
-        <v/>
-      </c>
-      <c r="L41" s="401">
-        <f>IF($H41="","nog te plannen",IFERROR(LOOKUP($H41,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H41" s="391" t="n"/>
+      <c r="I41" s="388" t="n"/>
+      <c r="J41" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C41,'SAERTEX-prijstabel'!$B$2:$B$496,$D41,'SAERTEX-prijstabel'!$C$2:$C$496,$E41,'SAERTEX-prijstabel'!$D$2:$D$496,$F41),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K41" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G41)+N($H41))=0,0,IF((N($G41)+N($H41))&lt;15,0.25,IF((N($G41)+N($H41))&lt;=50,0.035,IF((N($G41)+N($H41))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L41" s="392">
+        <f>IF($J41=0,0,$G41*$J41*(1+$K41))</f>
+        <v/>
+      </c>
+      <c r="M41" s="392">
+        <f>N($H41)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N41" s="398">
+        <f>$L41+$M41</f>
+        <v/>
+      </c>
+      <c r="O41" s="401">
+        <f>IF($I41="","nog te plannen",IFERROR(LOOKUP($I41,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6174,21 +6600,30 @@
       <c r="E42" s="306" t="n"/>
       <c r="F42" s="306" t="n"/>
       <c r="G42" s="391" t="n"/>
-      <c r="H42" s="388" t="n"/>
-      <c r="I42" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C42,'SAERTEX-prijstabel'!$B$2:$B$496,$D42,'SAERTEX-prijstabel'!$C$2:$C$496,$E42,'SAERTEX-prijstabel'!$D$2:$D$496,$F42),0)</f>
-        <v/>
-      </c>
-      <c r="J42" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G42="","",IF($G42&lt;15,0.25,IF($G42&lt;=50,0.035,IF($G42&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K42" s="392">
-        <f>IF($I42=0,0,$G42*$I42*(1+N($J42)))</f>
-        <v/>
-      </c>
-      <c r="L42" s="401">
-        <f>IF($H42="","nog te plannen",IFERROR(LOOKUP($H42,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H42" s="391" t="n"/>
+      <c r="I42" s="388" t="n"/>
+      <c r="J42" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C42,'SAERTEX-prijstabel'!$B$2:$B$496,$D42,'SAERTEX-prijstabel'!$C$2:$C$496,$E42,'SAERTEX-prijstabel'!$D$2:$D$496,$F42),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K42" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G42)+N($H42))=0,0,IF((N($G42)+N($H42))&lt;15,0.25,IF((N($G42)+N($H42))&lt;=50,0.035,IF((N($G42)+N($H42))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L42" s="392">
+        <f>IF($J42=0,0,$G42*$J42*(1+$K42))</f>
+        <v/>
+      </c>
+      <c r="M42" s="392">
+        <f>N($H42)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N42" s="398">
+        <f>$L42+$M42</f>
+        <v/>
+      </c>
+      <c r="O42" s="401">
+        <f>IF($I42="","nog te plannen",IFERROR(LOOKUP($I42,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6200,21 +6635,30 @@
       <c r="E43" s="306" t="n"/>
       <c r="F43" s="306" t="n"/>
       <c r="G43" s="391" t="n"/>
-      <c r="H43" s="388" t="n"/>
-      <c r="I43" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C43,'SAERTEX-prijstabel'!$B$2:$B$496,$D43,'SAERTEX-prijstabel'!$C$2:$C$496,$E43,'SAERTEX-prijstabel'!$D$2:$D$496,$F43),0)</f>
-        <v/>
-      </c>
-      <c r="J43" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G43="","",IF($G43&lt;15,0.25,IF($G43&lt;=50,0.035,IF($G43&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K43" s="392">
-        <f>IF($I43=0,0,$G43*$I43*(1+N($J43)))</f>
-        <v/>
-      </c>
-      <c r="L43" s="401">
-        <f>IF($H43="","nog te plannen",IFERROR(LOOKUP($H43,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H43" s="391" t="n"/>
+      <c r="I43" s="388" t="n"/>
+      <c r="J43" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C43,'SAERTEX-prijstabel'!$B$2:$B$496,$D43,'SAERTEX-prijstabel'!$C$2:$C$496,$E43,'SAERTEX-prijstabel'!$D$2:$D$496,$F43),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K43" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G43)+N($H43))=0,0,IF((N($G43)+N($H43))&lt;15,0.25,IF((N($G43)+N($H43))&lt;=50,0.035,IF((N($G43)+N($H43))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L43" s="392">
+        <f>IF($J43=0,0,$G43*$J43*(1+$K43))</f>
+        <v/>
+      </c>
+      <c r="M43" s="392">
+        <f>N($H43)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N43" s="398">
+        <f>$L43+$M43</f>
+        <v/>
+      </c>
+      <c r="O43" s="401">
+        <f>IF($I43="","nog te plannen",IFERROR(LOOKUP($I43,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6226,21 +6670,30 @@
       <c r="E44" s="306" t="n"/>
       <c r="F44" s="306" t="n"/>
       <c r="G44" s="391" t="n"/>
-      <c r="H44" s="388" t="n"/>
-      <c r="I44" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C44,'SAERTEX-prijstabel'!$B$2:$B$496,$D44,'SAERTEX-prijstabel'!$C$2:$C$496,$E44,'SAERTEX-prijstabel'!$D$2:$D$496,$F44),0)</f>
-        <v/>
-      </c>
-      <c r="J44" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G44="","",IF($G44&lt;15,0.25,IF($G44&lt;=50,0.035,IF($G44&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K44" s="392">
-        <f>IF($I44=0,0,$G44*$I44*(1+N($J44)))</f>
-        <v/>
-      </c>
-      <c r="L44" s="401">
-        <f>IF($H44="","nog te plannen",IFERROR(LOOKUP($H44,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H44" s="391" t="n"/>
+      <c r="I44" s="388" t="n"/>
+      <c r="J44" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C44,'SAERTEX-prijstabel'!$B$2:$B$496,$D44,'SAERTEX-prijstabel'!$C$2:$C$496,$E44,'SAERTEX-prijstabel'!$D$2:$D$496,$F44),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K44" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G44)+N($H44))=0,0,IF((N($G44)+N($H44))&lt;15,0.25,IF((N($G44)+N($H44))&lt;=50,0.035,IF((N($G44)+N($H44))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L44" s="392">
+        <f>IF($J44=0,0,$G44*$J44*(1+$K44))</f>
+        <v/>
+      </c>
+      <c r="M44" s="392">
+        <f>N($H44)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N44" s="398">
+        <f>$L44+$M44</f>
+        <v/>
+      </c>
+      <c r="O44" s="401">
+        <f>IF($I44="","nog te plannen",IFERROR(LOOKUP($I44,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6252,21 +6705,30 @@
       <c r="E45" s="306" t="n"/>
       <c r="F45" s="306" t="n"/>
       <c r="G45" s="391" t="n"/>
-      <c r="H45" s="388" t="n"/>
-      <c r="I45" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C45,'SAERTEX-prijstabel'!$B$2:$B$496,$D45,'SAERTEX-prijstabel'!$C$2:$C$496,$E45,'SAERTEX-prijstabel'!$D$2:$D$496,$F45),0)</f>
-        <v/>
-      </c>
-      <c r="J45" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G45="","",IF($G45&lt;15,0.25,IF($G45&lt;=50,0.035,IF($G45&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K45" s="392">
-        <f>IF($I45=0,0,$G45*$I45*(1+N($J45)))</f>
-        <v/>
-      </c>
-      <c r="L45" s="401">
-        <f>IF($H45="","nog te plannen",IFERROR(LOOKUP($H45,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H45" s="391" t="n"/>
+      <c r="I45" s="388" t="n"/>
+      <c r="J45" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C45,'SAERTEX-prijstabel'!$B$2:$B$496,$D45,'SAERTEX-prijstabel'!$C$2:$C$496,$E45,'SAERTEX-prijstabel'!$D$2:$D$496,$F45),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K45" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G45)+N($H45))=0,0,IF((N($G45)+N($H45))&lt;15,0.25,IF((N($G45)+N($H45))&lt;=50,0.035,IF((N($G45)+N($H45))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L45" s="392">
+        <f>IF($J45=0,0,$G45*$J45*(1+$K45))</f>
+        <v/>
+      </c>
+      <c r="M45" s="392">
+        <f>N($H45)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N45" s="398">
+        <f>$L45+$M45</f>
+        <v/>
+      </c>
+      <c r="O45" s="401">
+        <f>IF($I45="","nog te plannen",IFERROR(LOOKUP($I45,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6278,21 +6740,30 @@
       <c r="E46" s="306" t="n"/>
       <c r="F46" s="306" t="n"/>
       <c r="G46" s="391" t="n"/>
-      <c r="H46" s="388" t="n"/>
-      <c r="I46" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C46,'SAERTEX-prijstabel'!$B$2:$B$496,$D46,'SAERTEX-prijstabel'!$C$2:$C$496,$E46,'SAERTEX-prijstabel'!$D$2:$D$496,$F46),0)</f>
-        <v/>
-      </c>
-      <c r="J46" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G46="","",IF($G46&lt;15,0.25,IF($G46&lt;=50,0.035,IF($G46&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K46" s="392">
-        <f>IF($I46=0,0,$G46*$I46*(1+N($J46)))</f>
-        <v/>
-      </c>
-      <c r="L46" s="401">
-        <f>IF($H46="","nog te plannen",IFERROR(LOOKUP($H46,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H46" s="391" t="n"/>
+      <c r="I46" s="388" t="n"/>
+      <c r="J46" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C46,'SAERTEX-prijstabel'!$B$2:$B$496,$D46,'SAERTEX-prijstabel'!$C$2:$C$496,$E46,'SAERTEX-prijstabel'!$D$2:$D$496,$F46),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K46" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G46)+N($H46))=0,0,IF((N($G46)+N($H46))&lt;15,0.25,IF((N($G46)+N($H46))&lt;=50,0.035,IF((N($G46)+N($H46))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L46" s="392">
+        <f>IF($J46=0,0,$G46*$J46*(1+$K46))</f>
+        <v/>
+      </c>
+      <c r="M46" s="392">
+        <f>N($H46)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N46" s="398">
+        <f>$L46+$M46</f>
+        <v/>
+      </c>
+      <c r="O46" s="401">
+        <f>IF($I46="","nog te plannen",IFERROR(LOOKUP($I46,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6304,21 +6775,30 @@
       <c r="E47" s="306" t="n"/>
       <c r="F47" s="306" t="n"/>
       <c r="G47" s="391" t="n"/>
-      <c r="H47" s="388" t="n"/>
-      <c r="I47" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C47,'SAERTEX-prijstabel'!$B$2:$B$496,$D47,'SAERTEX-prijstabel'!$C$2:$C$496,$E47,'SAERTEX-prijstabel'!$D$2:$D$496,$F47),0)</f>
-        <v/>
-      </c>
-      <c r="J47" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G47="","",IF($G47&lt;15,0.25,IF($G47&lt;=50,0.035,IF($G47&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K47" s="392">
-        <f>IF($I47=0,0,$G47*$I47*(1+N($J47)))</f>
-        <v/>
-      </c>
-      <c r="L47" s="401">
-        <f>IF($H47="","nog te plannen",IFERROR(LOOKUP($H47,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H47" s="391" t="n"/>
+      <c r="I47" s="388" t="n"/>
+      <c r="J47" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C47,'SAERTEX-prijstabel'!$B$2:$B$496,$D47,'SAERTEX-prijstabel'!$C$2:$C$496,$E47,'SAERTEX-prijstabel'!$D$2:$D$496,$F47),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K47" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G47)+N($H47))=0,0,IF((N($G47)+N($H47))&lt;15,0.25,IF((N($G47)+N($H47))&lt;=50,0.035,IF((N($G47)+N($H47))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L47" s="392">
+        <f>IF($J47=0,0,$G47*$J47*(1+$K47))</f>
+        <v/>
+      </c>
+      <c r="M47" s="392">
+        <f>N($H47)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N47" s="398">
+        <f>$L47+$M47</f>
+        <v/>
+      </c>
+      <c r="O47" s="401">
+        <f>IF($I47="","nog te plannen",IFERROR(LOOKUP($I47,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6330,21 +6810,30 @@
       <c r="E48" s="306" t="n"/>
       <c r="F48" s="306" t="n"/>
       <c r="G48" s="391" t="n"/>
-      <c r="H48" s="388" t="n"/>
-      <c r="I48" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C48,'SAERTEX-prijstabel'!$B$2:$B$496,$D48,'SAERTEX-prijstabel'!$C$2:$C$496,$E48,'SAERTEX-prijstabel'!$D$2:$D$496,$F48),0)</f>
-        <v/>
-      </c>
-      <c r="J48" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G48="","",IF($G48&lt;15,0.25,IF($G48&lt;=50,0.035,IF($G48&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K48" s="392">
-        <f>IF($I48=0,0,$G48*$I48*(1+N($J48)))</f>
-        <v/>
-      </c>
-      <c r="L48" s="401">
-        <f>IF($H48="","nog te plannen",IFERROR(LOOKUP($H48,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H48" s="391" t="n"/>
+      <c r="I48" s="388" t="n"/>
+      <c r="J48" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C48,'SAERTEX-prijstabel'!$B$2:$B$496,$D48,'SAERTEX-prijstabel'!$C$2:$C$496,$E48,'SAERTEX-prijstabel'!$D$2:$D$496,$F48),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K48" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G48)+N($H48))=0,0,IF((N($G48)+N($H48))&lt;15,0.25,IF((N($G48)+N($H48))&lt;=50,0.035,IF((N($G48)+N($H48))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L48" s="392">
+        <f>IF($J48=0,0,$G48*$J48*(1+$K48))</f>
+        <v/>
+      </c>
+      <c r="M48" s="392">
+        <f>N($H48)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N48" s="398">
+        <f>$L48+$M48</f>
+        <v/>
+      </c>
+      <c r="O48" s="401">
+        <f>IF($I48="","nog te plannen",IFERROR(LOOKUP($I48,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6356,21 +6845,30 @@
       <c r="E49" s="306" t="n"/>
       <c r="F49" s="306" t="n"/>
       <c r="G49" s="391" t="n"/>
-      <c r="H49" s="388" t="n"/>
-      <c r="I49" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C49,'SAERTEX-prijstabel'!$B$2:$B$496,$D49,'SAERTEX-prijstabel'!$C$2:$C$496,$E49,'SAERTEX-prijstabel'!$D$2:$D$496,$F49),0)</f>
-        <v/>
-      </c>
-      <c r="J49" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G49="","",IF($G49&lt;15,0.25,IF($G49&lt;=50,0.035,IF($G49&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K49" s="392">
-        <f>IF($I49=0,0,$G49*$I49*(1+N($J49)))</f>
-        <v/>
-      </c>
-      <c r="L49" s="401">
-        <f>IF($H49="","nog te plannen",IFERROR(LOOKUP($H49,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H49" s="391" t="n"/>
+      <c r="I49" s="388" t="n"/>
+      <c r="J49" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C49,'SAERTEX-prijstabel'!$B$2:$B$496,$D49,'SAERTEX-prijstabel'!$C$2:$C$496,$E49,'SAERTEX-prijstabel'!$D$2:$D$496,$F49),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K49" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G49)+N($H49))=0,0,IF((N($G49)+N($H49))&lt;15,0.25,IF((N($G49)+N($H49))&lt;=50,0.035,IF((N($G49)+N($H49))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L49" s="392">
+        <f>IF($J49=0,0,$G49*$J49*(1+$K49))</f>
+        <v/>
+      </c>
+      <c r="M49" s="392">
+        <f>N($H49)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N49" s="398">
+        <f>$L49+$M49</f>
+        <v/>
+      </c>
+      <c r="O49" s="401">
+        <f>IF($I49="","nog te plannen",IFERROR(LOOKUP($I49,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6382,21 +6880,30 @@
       <c r="E50" s="306" t="n"/>
       <c r="F50" s="306" t="n"/>
       <c r="G50" s="391" t="n"/>
-      <c r="H50" s="388" t="n"/>
-      <c r="I50" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C50,'SAERTEX-prijstabel'!$B$2:$B$496,$D50,'SAERTEX-prijstabel'!$C$2:$C$496,$E50,'SAERTEX-prijstabel'!$D$2:$D$496,$F50),0)</f>
-        <v/>
-      </c>
-      <c r="J50" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G50="","",IF($G50&lt;15,0.25,IF($G50&lt;=50,0.035,IF($G50&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K50" s="392">
-        <f>IF($I50=0,0,$G50*$I50*(1+N($J50)))</f>
-        <v/>
-      </c>
-      <c r="L50" s="401">
-        <f>IF($H50="","nog te plannen",IFERROR(LOOKUP($H50,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H50" s="391" t="n"/>
+      <c r="I50" s="388" t="n"/>
+      <c r="J50" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C50,'SAERTEX-prijstabel'!$B$2:$B$496,$D50,'SAERTEX-prijstabel'!$C$2:$C$496,$E50,'SAERTEX-prijstabel'!$D$2:$D$496,$F50),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K50" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G50)+N($H50))=0,0,IF((N($G50)+N($H50))&lt;15,0.25,IF((N($G50)+N($H50))&lt;=50,0.035,IF((N($G50)+N($H50))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L50" s="392">
+        <f>IF($J50=0,0,$G50*$J50*(1+$K50))</f>
+        <v/>
+      </c>
+      <c r="M50" s="392">
+        <f>N($H50)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N50" s="398">
+        <f>$L50+$M50</f>
+        <v/>
+      </c>
+      <c r="O50" s="401">
+        <f>IF($I50="","nog te plannen",IFERROR(LOOKUP($I50,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6408,21 +6915,30 @@
       <c r="E51" s="306" t="n"/>
       <c r="F51" s="306" t="n"/>
       <c r="G51" s="391" t="n"/>
-      <c r="H51" s="388" t="n"/>
-      <c r="I51" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C51,'SAERTEX-prijstabel'!$B$2:$B$496,$D51,'SAERTEX-prijstabel'!$C$2:$C$496,$E51,'SAERTEX-prijstabel'!$D$2:$D$496,$F51),0)</f>
-        <v/>
-      </c>
-      <c r="J51" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G51="","",IF($G51&lt;15,0.25,IF($G51&lt;=50,0.035,IF($G51&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K51" s="392">
-        <f>IF($I51=0,0,$G51*$I51*(1+N($J51)))</f>
-        <v/>
-      </c>
-      <c r="L51" s="401">
-        <f>IF($H51="","nog te plannen",IFERROR(LOOKUP($H51,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H51" s="391" t="n"/>
+      <c r="I51" s="388" t="n"/>
+      <c r="J51" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C51,'SAERTEX-prijstabel'!$B$2:$B$496,$D51,'SAERTEX-prijstabel'!$C$2:$C$496,$E51,'SAERTEX-prijstabel'!$D$2:$D$496,$F51),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K51" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G51)+N($H51))=0,0,IF((N($G51)+N($H51))&lt;15,0.25,IF((N($G51)+N($H51))&lt;=50,0.035,IF((N($G51)+N($H51))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L51" s="392">
+        <f>IF($J51=0,0,$G51*$J51*(1+$K51))</f>
+        <v/>
+      </c>
+      <c r="M51" s="392">
+        <f>N($H51)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N51" s="398">
+        <f>$L51+$M51</f>
+        <v/>
+      </c>
+      <c r="O51" s="401">
+        <f>IF($I51="","nog te plannen",IFERROR(LOOKUP($I51,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6434,21 +6950,30 @@
       <c r="E52" s="306" t="n"/>
       <c r="F52" s="306" t="n"/>
       <c r="G52" s="391" t="n"/>
-      <c r="H52" s="388" t="n"/>
-      <c r="I52" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C52,'SAERTEX-prijstabel'!$B$2:$B$496,$D52,'SAERTEX-prijstabel'!$C$2:$C$496,$E52,'SAERTEX-prijstabel'!$D$2:$D$496,$F52),0)</f>
-        <v/>
-      </c>
-      <c r="J52" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G52="","",IF($G52&lt;15,0.25,IF($G52&lt;=50,0.035,IF($G52&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K52" s="392">
-        <f>IF($I52=0,0,$G52*$I52*(1+N($J52)))</f>
-        <v/>
-      </c>
-      <c r="L52" s="401">
-        <f>IF($H52="","nog te plannen",IFERROR(LOOKUP($H52,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H52" s="391" t="n"/>
+      <c r="I52" s="388" t="n"/>
+      <c r="J52" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C52,'SAERTEX-prijstabel'!$B$2:$B$496,$D52,'SAERTEX-prijstabel'!$C$2:$C$496,$E52,'SAERTEX-prijstabel'!$D$2:$D$496,$F52),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K52" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G52)+N($H52))=0,0,IF((N($G52)+N($H52))&lt;15,0.25,IF((N($G52)+N($H52))&lt;=50,0.035,IF((N($G52)+N($H52))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L52" s="392">
+        <f>IF($J52=0,0,$G52*$J52*(1+$K52))</f>
+        <v/>
+      </c>
+      <c r="M52" s="392">
+        <f>N($H52)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N52" s="398">
+        <f>$L52+$M52</f>
+        <v/>
+      </c>
+      <c r="O52" s="401">
+        <f>IF($I52="","nog te plannen",IFERROR(LOOKUP($I52,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6460,21 +6985,30 @@
       <c r="E53" s="306" t="n"/>
       <c r="F53" s="306" t="n"/>
       <c r="G53" s="391" t="n"/>
-      <c r="H53" s="388" t="n"/>
-      <c r="I53" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C53,'SAERTEX-prijstabel'!$B$2:$B$496,$D53,'SAERTEX-prijstabel'!$C$2:$C$496,$E53,'SAERTEX-prijstabel'!$D$2:$D$496,$F53),0)</f>
-        <v/>
-      </c>
-      <c r="J53" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G53="","",IF($G53&lt;15,0.25,IF($G53&lt;=50,0.035,IF($G53&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K53" s="392">
-        <f>IF($I53=0,0,$G53*$I53*(1+N($J53)))</f>
-        <v/>
-      </c>
-      <c r="L53" s="401">
-        <f>IF($H53="","nog te plannen",IFERROR(LOOKUP($H53,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H53" s="391" t="n"/>
+      <c r="I53" s="388" t="n"/>
+      <c r="J53" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C53,'SAERTEX-prijstabel'!$B$2:$B$496,$D53,'SAERTEX-prijstabel'!$C$2:$C$496,$E53,'SAERTEX-prijstabel'!$D$2:$D$496,$F53),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K53" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G53)+N($H53))=0,0,IF((N($G53)+N($H53))&lt;15,0.25,IF((N($G53)+N($H53))&lt;=50,0.035,IF((N($G53)+N($H53))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L53" s="392">
+        <f>IF($J53=0,0,$G53*$J53*(1+$K53))</f>
+        <v/>
+      </c>
+      <c r="M53" s="392">
+        <f>N($H53)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N53" s="398">
+        <f>$L53+$M53</f>
+        <v/>
+      </c>
+      <c r="O53" s="401">
+        <f>IF($I53="","nog te plannen",IFERROR(LOOKUP($I53,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6486,21 +7020,30 @@
       <c r="E54" s="306" t="n"/>
       <c r="F54" s="306" t="n"/>
       <c r="G54" s="391" t="n"/>
-      <c r="H54" s="388" t="n"/>
-      <c r="I54" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C54,'SAERTEX-prijstabel'!$B$2:$B$496,$D54,'SAERTEX-prijstabel'!$C$2:$C$496,$E54,'SAERTEX-prijstabel'!$D$2:$D$496,$F54),0)</f>
-        <v/>
-      </c>
-      <c r="J54" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G54="","",IF($G54&lt;15,0.25,IF($G54&lt;=50,0.035,IF($G54&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K54" s="392">
-        <f>IF($I54=0,0,$G54*$I54*(1+N($J54)))</f>
-        <v/>
-      </c>
-      <c r="L54" s="401">
-        <f>IF($H54="","nog te plannen",IFERROR(LOOKUP($H54,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H54" s="391" t="n"/>
+      <c r="I54" s="388" t="n"/>
+      <c r="J54" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C54,'SAERTEX-prijstabel'!$B$2:$B$496,$D54,'SAERTEX-prijstabel'!$C$2:$C$496,$E54,'SAERTEX-prijstabel'!$D$2:$D$496,$F54),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K54" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G54)+N($H54))=0,0,IF((N($G54)+N($H54))&lt;15,0.25,IF((N($G54)+N($H54))&lt;=50,0.035,IF((N($G54)+N($H54))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L54" s="392">
+        <f>IF($J54=0,0,$G54*$J54*(1+$K54))</f>
+        <v/>
+      </c>
+      <c r="M54" s="392">
+        <f>N($H54)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N54" s="398">
+        <f>$L54+$M54</f>
+        <v/>
+      </c>
+      <c r="O54" s="401">
+        <f>IF($I54="","nog te plannen",IFERROR(LOOKUP($I54,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6512,21 +7055,30 @@
       <c r="E55" s="306" t="n"/>
       <c r="F55" s="306" t="n"/>
       <c r="G55" s="391" t="n"/>
-      <c r="H55" s="388" t="n"/>
-      <c r="I55" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C55,'SAERTEX-prijstabel'!$B$2:$B$496,$D55,'SAERTEX-prijstabel'!$C$2:$C$496,$E55,'SAERTEX-prijstabel'!$D$2:$D$496,$F55),0)</f>
-        <v/>
-      </c>
-      <c r="J55" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G55="","",IF($G55&lt;15,0.25,IF($G55&lt;=50,0.035,IF($G55&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K55" s="392">
-        <f>IF($I55=0,0,$G55*$I55*(1+N($J55)))</f>
-        <v/>
-      </c>
-      <c r="L55" s="401">
-        <f>IF($H55="","nog te plannen",IFERROR(LOOKUP($H55,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H55" s="391" t="n"/>
+      <c r="I55" s="388" t="n"/>
+      <c r="J55" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C55,'SAERTEX-prijstabel'!$B$2:$B$496,$D55,'SAERTEX-prijstabel'!$C$2:$C$496,$E55,'SAERTEX-prijstabel'!$D$2:$D$496,$F55),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K55" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G55)+N($H55))=0,0,IF((N($G55)+N($H55))&lt;15,0.25,IF((N($G55)+N($H55))&lt;=50,0.035,IF((N($G55)+N($H55))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L55" s="392">
+        <f>IF($J55=0,0,$G55*$J55*(1+$K55))</f>
+        <v/>
+      </c>
+      <c r="M55" s="392">
+        <f>N($H55)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N55" s="398">
+        <f>$L55+$M55</f>
+        <v/>
+      </c>
+      <c r="O55" s="401">
+        <f>IF($I55="","nog te plannen",IFERROR(LOOKUP($I55,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6538,21 +7090,30 @@
       <c r="E56" s="306" t="n"/>
       <c r="F56" s="306" t="n"/>
       <c r="G56" s="391" t="n"/>
-      <c r="H56" s="388" t="n"/>
-      <c r="I56" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C56,'SAERTEX-prijstabel'!$B$2:$B$496,$D56,'SAERTEX-prijstabel'!$C$2:$C$496,$E56,'SAERTEX-prijstabel'!$D$2:$D$496,$F56),0)</f>
-        <v/>
-      </c>
-      <c r="J56" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G56="","",IF($G56&lt;15,0.25,IF($G56&lt;=50,0.035,IF($G56&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K56" s="392">
-        <f>IF($I56=0,0,$G56*$I56*(1+N($J56)))</f>
-        <v/>
-      </c>
-      <c r="L56" s="401">
-        <f>IF($H56="","nog te plannen",IFERROR(LOOKUP($H56,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H56" s="391" t="n"/>
+      <c r="I56" s="388" t="n"/>
+      <c r="J56" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C56,'SAERTEX-prijstabel'!$B$2:$B$496,$D56,'SAERTEX-prijstabel'!$C$2:$C$496,$E56,'SAERTEX-prijstabel'!$D$2:$D$496,$F56),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K56" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G56)+N($H56))=0,0,IF((N($G56)+N($H56))&lt;15,0.25,IF((N($G56)+N($H56))&lt;=50,0.035,IF((N($G56)+N($H56))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L56" s="392">
+        <f>IF($J56=0,0,$G56*$J56*(1+$K56))</f>
+        <v/>
+      </c>
+      <c r="M56" s="392">
+        <f>N($H56)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N56" s="398">
+        <f>$L56+$M56</f>
+        <v/>
+      </c>
+      <c r="O56" s="401">
+        <f>IF($I56="","nog te plannen",IFERROR(LOOKUP($I56,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6564,21 +7125,30 @@
       <c r="E57" s="306" t="n"/>
       <c r="F57" s="306" t="n"/>
       <c r="G57" s="391" t="n"/>
-      <c r="H57" s="388" t="n"/>
-      <c r="I57" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C57,'SAERTEX-prijstabel'!$B$2:$B$496,$D57,'SAERTEX-prijstabel'!$C$2:$C$496,$E57,'SAERTEX-prijstabel'!$D$2:$D$496,$F57),0)</f>
-        <v/>
-      </c>
-      <c r="J57" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G57="","",IF($G57&lt;15,0.25,IF($G57&lt;=50,0.035,IF($G57&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K57" s="392">
-        <f>IF($I57=0,0,$G57*$I57*(1+N($J57)))</f>
-        <v/>
-      </c>
-      <c r="L57" s="401">
-        <f>IF($H57="","nog te plannen",IFERROR(LOOKUP($H57,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H57" s="391" t="n"/>
+      <c r="I57" s="388" t="n"/>
+      <c r="J57" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C57,'SAERTEX-prijstabel'!$B$2:$B$496,$D57,'SAERTEX-prijstabel'!$C$2:$C$496,$E57,'SAERTEX-prijstabel'!$D$2:$D$496,$F57),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K57" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G57)+N($H57))=0,0,IF((N($G57)+N($H57))&lt;15,0.25,IF((N($G57)+N($H57))&lt;=50,0.035,IF((N($G57)+N($H57))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L57" s="392">
+        <f>IF($J57=0,0,$G57*$J57*(1+$K57))</f>
+        <v/>
+      </c>
+      <c r="M57" s="392">
+        <f>N($H57)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N57" s="398">
+        <f>$L57+$M57</f>
+        <v/>
+      </c>
+      <c r="O57" s="401">
+        <f>IF($I57="","nog te plannen",IFERROR(LOOKUP($I57,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6590,21 +7160,30 @@
       <c r="E58" s="306" t="n"/>
       <c r="F58" s="306" t="n"/>
       <c r="G58" s="391" t="n"/>
-      <c r="H58" s="388" t="n"/>
-      <c r="I58" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C58,'SAERTEX-prijstabel'!$B$2:$B$496,$D58,'SAERTEX-prijstabel'!$C$2:$C$496,$E58,'SAERTEX-prijstabel'!$D$2:$D$496,$F58),0)</f>
-        <v/>
-      </c>
-      <c r="J58" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G58="","",IF($G58&lt;15,0.25,IF($G58&lt;=50,0.035,IF($G58&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K58" s="392">
-        <f>IF($I58=0,0,$G58*$I58*(1+N($J58)))</f>
-        <v/>
-      </c>
-      <c r="L58" s="401">
-        <f>IF($H58="","nog te plannen",IFERROR(LOOKUP($H58,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H58" s="391" t="n"/>
+      <c r="I58" s="388" t="n"/>
+      <c r="J58" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C58,'SAERTEX-prijstabel'!$B$2:$B$496,$D58,'SAERTEX-prijstabel'!$C$2:$C$496,$E58,'SAERTEX-prijstabel'!$D$2:$D$496,$F58),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K58" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G58)+N($H58))=0,0,IF((N($G58)+N($H58))&lt;15,0.25,IF((N($G58)+N($H58))&lt;=50,0.035,IF((N($G58)+N($H58))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L58" s="392">
+        <f>IF($J58=0,0,$G58*$J58*(1+$K58))</f>
+        <v/>
+      </c>
+      <c r="M58" s="392">
+        <f>N($H58)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N58" s="398">
+        <f>$L58+$M58</f>
+        <v/>
+      </c>
+      <c r="O58" s="401">
+        <f>IF($I58="","nog te plannen",IFERROR(LOOKUP($I58,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6616,21 +7195,30 @@
       <c r="E59" s="306" t="n"/>
       <c r="F59" s="306" t="n"/>
       <c r="G59" s="391" t="n"/>
-      <c r="H59" s="388" t="n"/>
-      <c r="I59" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C59,'SAERTEX-prijstabel'!$B$2:$B$496,$D59,'SAERTEX-prijstabel'!$C$2:$C$496,$E59,'SAERTEX-prijstabel'!$D$2:$D$496,$F59),0)</f>
-        <v/>
-      </c>
-      <c r="J59" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G59="","",IF($G59&lt;15,0.25,IF($G59&lt;=50,0.035,IF($G59&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K59" s="392">
-        <f>IF($I59=0,0,$G59*$I59*(1+N($J59)))</f>
-        <v/>
-      </c>
-      <c r="L59" s="401">
-        <f>IF($H59="","nog te plannen",IFERROR(LOOKUP($H59,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H59" s="391" t="n"/>
+      <c r="I59" s="388" t="n"/>
+      <c r="J59" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C59,'SAERTEX-prijstabel'!$B$2:$B$496,$D59,'SAERTEX-prijstabel'!$C$2:$C$496,$E59,'SAERTEX-prijstabel'!$D$2:$D$496,$F59),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K59" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G59)+N($H59))=0,0,IF((N($G59)+N($H59))&lt;15,0.25,IF((N($G59)+N($H59))&lt;=50,0.035,IF((N($G59)+N($H59))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L59" s="392">
+        <f>IF($J59=0,0,$G59*$J59*(1+$K59))</f>
+        <v/>
+      </c>
+      <c r="M59" s="392">
+        <f>N($H59)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N59" s="398">
+        <f>$L59+$M59</f>
+        <v/>
+      </c>
+      <c r="O59" s="401">
+        <f>IF($I59="","nog te plannen",IFERROR(LOOKUP($I59,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6642,21 +7230,30 @@
       <c r="E60" s="306" t="n"/>
       <c r="F60" s="306" t="n"/>
       <c r="G60" s="391" t="n"/>
-      <c r="H60" s="388" t="n"/>
-      <c r="I60" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C60,'SAERTEX-prijstabel'!$B$2:$B$496,$D60,'SAERTEX-prijstabel'!$C$2:$C$496,$E60,'SAERTEX-prijstabel'!$D$2:$D$496,$F60),0)</f>
-        <v/>
-      </c>
-      <c r="J60" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G60="","",IF($G60&lt;15,0.25,IF($G60&lt;=50,0.035,IF($G60&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K60" s="392">
-        <f>IF($I60=0,0,$G60*$I60*(1+N($J60)))</f>
-        <v/>
-      </c>
-      <c r="L60" s="401">
-        <f>IF($H60="","nog te plannen",IFERROR(LOOKUP($H60,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H60" s="391" t="n"/>
+      <c r="I60" s="388" t="n"/>
+      <c r="J60" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C60,'SAERTEX-prijstabel'!$B$2:$B$496,$D60,'SAERTEX-prijstabel'!$C$2:$C$496,$E60,'SAERTEX-prijstabel'!$D$2:$D$496,$F60),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K60" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G60)+N($H60))=0,0,IF((N($G60)+N($H60))&lt;15,0.25,IF((N($G60)+N($H60))&lt;=50,0.035,IF((N($G60)+N($H60))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L60" s="392">
+        <f>IF($J60=0,0,$G60*$J60*(1+$K60))</f>
+        <v/>
+      </c>
+      <c r="M60" s="392">
+        <f>N($H60)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N60" s="398">
+        <f>$L60+$M60</f>
+        <v/>
+      </c>
+      <c r="O60" s="401">
+        <f>IF($I60="","nog te plannen",IFERROR(LOOKUP($I60,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6668,21 +7265,30 @@
       <c r="E61" s="306" t="n"/>
       <c r="F61" s="306" t="n"/>
       <c r="G61" s="391" t="n"/>
-      <c r="H61" s="388" t="n"/>
-      <c r="I61" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C61,'SAERTEX-prijstabel'!$B$2:$B$496,$D61,'SAERTEX-prijstabel'!$C$2:$C$496,$E61,'SAERTEX-prijstabel'!$D$2:$D$496,$F61),0)</f>
-        <v/>
-      </c>
-      <c r="J61" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G61="","",IF($G61&lt;15,0.25,IF($G61&lt;=50,0.035,IF($G61&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K61" s="392">
-        <f>IF($I61=0,0,$G61*$I61*(1+N($J61)))</f>
-        <v/>
-      </c>
-      <c r="L61" s="401">
-        <f>IF($H61="","nog te plannen",IFERROR(LOOKUP($H61,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H61" s="391" t="n"/>
+      <c r="I61" s="388" t="n"/>
+      <c r="J61" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C61,'SAERTEX-prijstabel'!$B$2:$B$496,$D61,'SAERTEX-prijstabel'!$C$2:$C$496,$E61,'SAERTEX-prijstabel'!$D$2:$D$496,$F61),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K61" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G61)+N($H61))=0,0,IF((N($G61)+N($H61))&lt;15,0.25,IF((N($G61)+N($H61))&lt;=50,0.035,IF((N($G61)+N($H61))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L61" s="392">
+        <f>IF($J61=0,0,$G61*$J61*(1+$K61))</f>
+        <v/>
+      </c>
+      <c r="M61" s="392">
+        <f>N($H61)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N61" s="398">
+        <f>$L61+$M61</f>
+        <v/>
+      </c>
+      <c r="O61" s="401">
+        <f>IF($I61="","nog te plannen",IFERROR(LOOKUP($I61,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6694,21 +7300,30 @@
       <c r="E62" s="306" t="n"/>
       <c r="F62" s="306" t="n"/>
       <c r="G62" s="391" t="n"/>
-      <c r="H62" s="388" t="n"/>
-      <c r="I62" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C62,'SAERTEX-prijstabel'!$B$2:$B$496,$D62,'SAERTEX-prijstabel'!$C$2:$C$496,$E62,'SAERTEX-prijstabel'!$D$2:$D$496,$F62),0)</f>
-        <v/>
-      </c>
-      <c r="J62" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G62="","",IF($G62&lt;15,0.25,IF($G62&lt;=50,0.035,IF($G62&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K62" s="392">
-        <f>IF($I62=0,0,$G62*$I62*(1+N($J62)))</f>
-        <v/>
-      </c>
-      <c r="L62" s="401">
-        <f>IF($H62="","nog te plannen",IFERROR(LOOKUP($H62,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H62" s="391" t="n"/>
+      <c r="I62" s="388" t="n"/>
+      <c r="J62" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C62,'SAERTEX-prijstabel'!$B$2:$B$496,$D62,'SAERTEX-prijstabel'!$C$2:$C$496,$E62,'SAERTEX-prijstabel'!$D$2:$D$496,$F62),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K62" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G62)+N($H62))=0,0,IF((N($G62)+N($H62))&lt;15,0.25,IF((N($G62)+N($H62))&lt;=50,0.035,IF((N($G62)+N($H62))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L62" s="392">
+        <f>IF($J62=0,0,$G62*$J62*(1+$K62))</f>
+        <v/>
+      </c>
+      <c r="M62" s="392">
+        <f>N($H62)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N62" s="398">
+        <f>$L62+$M62</f>
+        <v/>
+      </c>
+      <c r="O62" s="401">
+        <f>IF($I62="","nog te plannen",IFERROR(LOOKUP($I62,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6720,21 +7335,30 @@
       <c r="E63" s="306" t="n"/>
       <c r="F63" s="306" t="n"/>
       <c r="G63" s="391" t="n"/>
-      <c r="H63" s="388" t="n"/>
-      <c r="I63" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C63,'SAERTEX-prijstabel'!$B$2:$B$496,$D63,'SAERTEX-prijstabel'!$C$2:$C$496,$E63,'SAERTEX-prijstabel'!$D$2:$D$496,$F63),0)</f>
-        <v/>
-      </c>
-      <c r="J63" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G63="","",IF($G63&lt;15,0.25,IF($G63&lt;=50,0.035,IF($G63&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K63" s="392">
-        <f>IF($I63=0,0,$G63*$I63*(1+N($J63)))</f>
-        <v/>
-      </c>
-      <c r="L63" s="401">
-        <f>IF($H63="","nog te plannen",IFERROR(LOOKUP($H63,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H63" s="391" t="n"/>
+      <c r="I63" s="388" t="n"/>
+      <c r="J63" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C63,'SAERTEX-prijstabel'!$B$2:$B$496,$D63,'SAERTEX-prijstabel'!$C$2:$C$496,$E63,'SAERTEX-prijstabel'!$D$2:$D$496,$F63),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K63" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G63)+N($H63))=0,0,IF((N($G63)+N($H63))&lt;15,0.25,IF((N($G63)+N($H63))&lt;=50,0.035,IF((N($G63)+N($H63))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L63" s="392">
+        <f>IF($J63=0,0,$G63*$J63*(1+$K63))</f>
+        <v/>
+      </c>
+      <c r="M63" s="392">
+        <f>N($H63)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N63" s="398">
+        <f>$L63+$M63</f>
+        <v/>
+      </c>
+      <c r="O63" s="401">
+        <f>IF($I63="","nog te plannen",IFERROR(LOOKUP($I63,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6746,21 +7370,30 @@
       <c r="E64" s="306" t="n"/>
       <c r="F64" s="306" t="n"/>
       <c r="G64" s="391" t="n"/>
-      <c r="H64" s="388" t="n"/>
-      <c r="I64" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C64,'SAERTEX-prijstabel'!$B$2:$B$496,$D64,'SAERTEX-prijstabel'!$C$2:$C$496,$E64,'SAERTEX-prijstabel'!$D$2:$D$496,$F64),0)</f>
-        <v/>
-      </c>
-      <c r="J64" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G64="","",IF($G64&lt;15,0.25,IF($G64&lt;=50,0.035,IF($G64&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K64" s="392">
-        <f>IF($I64=0,0,$G64*$I64*(1+N($J64)))</f>
-        <v/>
-      </c>
-      <c r="L64" s="401">
-        <f>IF($H64="","nog te plannen",IFERROR(LOOKUP($H64,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H64" s="391" t="n"/>
+      <c r="I64" s="388" t="n"/>
+      <c r="J64" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C64,'SAERTEX-prijstabel'!$B$2:$B$496,$D64,'SAERTEX-prijstabel'!$C$2:$C$496,$E64,'SAERTEX-prijstabel'!$D$2:$D$496,$F64),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K64" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G64)+N($H64))=0,0,IF((N($G64)+N($H64))&lt;15,0.25,IF((N($G64)+N($H64))&lt;=50,0.035,IF((N($G64)+N($H64))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L64" s="392">
+        <f>IF($J64=0,0,$G64*$J64*(1+$K64))</f>
+        <v/>
+      </c>
+      <c r="M64" s="392">
+        <f>N($H64)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N64" s="398">
+        <f>$L64+$M64</f>
+        <v/>
+      </c>
+      <c r="O64" s="401">
+        <f>IF($I64="","nog te plannen",IFERROR(LOOKUP($I64,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6772,21 +7405,30 @@
       <c r="E65" s="306" t="n"/>
       <c r="F65" s="306" t="n"/>
       <c r="G65" s="391" t="n"/>
-      <c r="H65" s="388" t="n"/>
-      <c r="I65" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C65,'SAERTEX-prijstabel'!$B$2:$B$496,$D65,'SAERTEX-prijstabel'!$C$2:$C$496,$E65,'SAERTEX-prijstabel'!$D$2:$D$496,$F65),0)</f>
-        <v/>
-      </c>
-      <c r="J65" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G65="","",IF($G65&lt;15,0.25,IF($G65&lt;=50,0.035,IF($G65&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K65" s="392">
-        <f>IF($I65=0,0,$G65*$I65*(1+N($J65)))</f>
-        <v/>
-      </c>
-      <c r="L65" s="401">
-        <f>IF($H65="","nog te plannen",IFERROR(LOOKUP($H65,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H65" s="391" t="n"/>
+      <c r="I65" s="388" t="n"/>
+      <c r="J65" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C65,'SAERTEX-prijstabel'!$B$2:$B$496,$D65,'SAERTEX-prijstabel'!$C$2:$C$496,$E65,'SAERTEX-prijstabel'!$D$2:$D$496,$F65),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K65" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G65)+N($H65))=0,0,IF((N($G65)+N($H65))&lt;15,0.25,IF((N($G65)+N($H65))&lt;=50,0.035,IF((N($G65)+N($H65))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L65" s="392">
+        <f>IF($J65=0,0,$G65*$J65*(1+$K65))</f>
+        <v/>
+      </c>
+      <c r="M65" s="392">
+        <f>N($H65)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N65" s="398">
+        <f>$L65+$M65</f>
+        <v/>
+      </c>
+      <c r="O65" s="401">
+        <f>IF($I65="","nog te plannen",IFERROR(LOOKUP($I65,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6798,21 +7440,30 @@
       <c r="E66" s="306" t="n"/>
       <c r="F66" s="306" t="n"/>
       <c r="G66" s="391" t="n"/>
-      <c r="H66" s="388" t="n"/>
-      <c r="I66" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C66,'SAERTEX-prijstabel'!$B$2:$B$496,$D66,'SAERTEX-prijstabel'!$C$2:$C$496,$E66,'SAERTEX-prijstabel'!$D$2:$D$496,$F66),0)</f>
-        <v/>
-      </c>
-      <c r="J66" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G66="","",IF($G66&lt;15,0.25,IF($G66&lt;=50,0.035,IF($G66&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K66" s="392">
-        <f>IF($I66=0,0,$G66*$I66*(1+N($J66)))</f>
-        <v/>
-      </c>
-      <c r="L66" s="401">
-        <f>IF($H66="","nog te plannen",IFERROR(LOOKUP($H66,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H66" s="391" t="n"/>
+      <c r="I66" s="388" t="n"/>
+      <c r="J66" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C66,'SAERTEX-prijstabel'!$B$2:$B$496,$D66,'SAERTEX-prijstabel'!$C$2:$C$496,$E66,'SAERTEX-prijstabel'!$D$2:$D$496,$F66),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K66" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G66)+N($H66))=0,0,IF((N($G66)+N($H66))&lt;15,0.25,IF((N($G66)+N($H66))&lt;=50,0.035,IF((N($G66)+N($H66))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L66" s="392">
+        <f>IF($J66=0,0,$G66*$J66*(1+$K66))</f>
+        <v/>
+      </c>
+      <c r="M66" s="392">
+        <f>N($H66)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N66" s="398">
+        <f>$L66+$M66</f>
+        <v/>
+      </c>
+      <c r="O66" s="401">
+        <f>IF($I66="","nog te plannen",IFERROR(LOOKUP($I66,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6824,21 +7475,30 @@
       <c r="E67" s="306" t="n"/>
       <c r="F67" s="306" t="n"/>
       <c r="G67" s="391" t="n"/>
-      <c r="H67" s="388" t="n"/>
-      <c r="I67" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C67,'SAERTEX-prijstabel'!$B$2:$B$496,$D67,'SAERTEX-prijstabel'!$C$2:$C$496,$E67,'SAERTEX-prijstabel'!$D$2:$D$496,$F67),0)</f>
-        <v/>
-      </c>
-      <c r="J67" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G67="","",IF($G67&lt;15,0.25,IF($G67&lt;=50,0.035,IF($G67&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K67" s="392">
-        <f>IF($I67=0,0,$G67*$I67*(1+N($J67)))</f>
-        <v/>
-      </c>
-      <c r="L67" s="401">
-        <f>IF($H67="","nog te plannen",IFERROR(LOOKUP($H67,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H67" s="391" t="n"/>
+      <c r="I67" s="388" t="n"/>
+      <c r="J67" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C67,'SAERTEX-prijstabel'!$B$2:$B$496,$D67,'SAERTEX-prijstabel'!$C$2:$C$496,$E67,'SAERTEX-prijstabel'!$D$2:$D$496,$F67),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K67" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G67)+N($H67))=0,0,IF((N($G67)+N($H67))&lt;15,0.25,IF((N($G67)+N($H67))&lt;=50,0.035,IF((N($G67)+N($H67))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L67" s="392">
+        <f>IF($J67=0,0,$G67*$J67*(1+$K67))</f>
+        <v/>
+      </c>
+      <c r="M67" s="392">
+        <f>N($H67)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N67" s="398">
+        <f>$L67+$M67</f>
+        <v/>
+      </c>
+      <c r="O67" s="401">
+        <f>IF($I67="","nog te plannen",IFERROR(LOOKUP($I67,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6850,21 +7510,30 @@
       <c r="E68" s="306" t="n"/>
       <c r="F68" s="306" t="n"/>
       <c r="G68" s="391" t="n"/>
-      <c r="H68" s="388" t="n"/>
-      <c r="I68" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C68,'SAERTEX-prijstabel'!$B$2:$B$496,$D68,'SAERTEX-prijstabel'!$C$2:$C$496,$E68,'SAERTEX-prijstabel'!$D$2:$D$496,$F68),0)</f>
-        <v/>
-      </c>
-      <c r="J68" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G68="","",IF($G68&lt;15,0.25,IF($G68&lt;=50,0.035,IF($G68&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K68" s="392">
-        <f>IF($I68=0,0,$G68*$I68*(1+N($J68)))</f>
-        <v/>
-      </c>
-      <c r="L68" s="401">
-        <f>IF($H68="","nog te plannen",IFERROR(LOOKUP($H68,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H68" s="391" t="n"/>
+      <c r="I68" s="388" t="n"/>
+      <c r="J68" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C68,'SAERTEX-prijstabel'!$B$2:$B$496,$D68,'SAERTEX-prijstabel'!$C$2:$C$496,$E68,'SAERTEX-prijstabel'!$D$2:$D$496,$F68),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K68" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G68)+N($H68))=0,0,IF((N($G68)+N($H68))&lt;15,0.25,IF((N($G68)+N($H68))&lt;=50,0.035,IF((N($G68)+N($H68))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L68" s="392">
+        <f>IF($J68=0,0,$G68*$J68*(1+$K68))</f>
+        <v/>
+      </c>
+      <c r="M68" s="392">
+        <f>N($H68)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N68" s="398">
+        <f>$L68+$M68</f>
+        <v/>
+      </c>
+      <c r="O68" s="401">
+        <f>IF($I68="","nog te plannen",IFERROR(LOOKUP($I68,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6876,21 +7545,30 @@
       <c r="E69" s="306" t="n"/>
       <c r="F69" s="306" t="n"/>
       <c r="G69" s="391" t="n"/>
-      <c r="H69" s="388" t="n"/>
-      <c r="I69" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C69,'SAERTEX-prijstabel'!$B$2:$B$496,$D69,'SAERTEX-prijstabel'!$C$2:$C$496,$E69,'SAERTEX-prijstabel'!$D$2:$D$496,$F69),0)</f>
-        <v/>
-      </c>
-      <c r="J69" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G69="","",IF($G69&lt;15,0.25,IF($G69&lt;=50,0.035,IF($G69&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K69" s="392">
-        <f>IF($I69=0,0,$G69*$I69*(1+N($J69)))</f>
-        <v/>
-      </c>
-      <c r="L69" s="401">
-        <f>IF($H69="","nog te plannen",IFERROR(LOOKUP($H69,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H69" s="391" t="n"/>
+      <c r="I69" s="388" t="n"/>
+      <c r="J69" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C69,'SAERTEX-prijstabel'!$B$2:$B$496,$D69,'SAERTEX-prijstabel'!$C$2:$C$496,$E69,'SAERTEX-prijstabel'!$D$2:$D$496,$F69),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K69" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G69)+N($H69))=0,0,IF((N($G69)+N($H69))&lt;15,0.25,IF((N($G69)+N($H69))&lt;=50,0.035,IF((N($G69)+N($H69))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L69" s="392">
+        <f>IF($J69=0,0,$G69*$J69*(1+$K69))</f>
+        <v/>
+      </c>
+      <c r="M69" s="392">
+        <f>N($H69)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N69" s="398">
+        <f>$L69+$M69</f>
+        <v/>
+      </c>
+      <c r="O69" s="401">
+        <f>IF($I69="","nog te plannen",IFERROR(LOOKUP($I69,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6902,21 +7580,30 @@
       <c r="E70" s="306" t="n"/>
       <c r="F70" s="306" t="n"/>
       <c r="G70" s="391" t="n"/>
-      <c r="H70" s="388" t="n"/>
-      <c r="I70" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C70,'SAERTEX-prijstabel'!$B$2:$B$496,$D70,'SAERTEX-prijstabel'!$C$2:$C$496,$E70,'SAERTEX-prijstabel'!$D$2:$D$496,$F70),0)</f>
-        <v/>
-      </c>
-      <c r="J70" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G70="","",IF($G70&lt;15,0.25,IF($G70&lt;=50,0.035,IF($G70&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K70" s="392">
-        <f>IF($I70=0,0,$G70*$I70*(1+N($J70)))</f>
-        <v/>
-      </c>
-      <c r="L70" s="401">
-        <f>IF($H70="","nog te plannen",IFERROR(LOOKUP($H70,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H70" s="391" t="n"/>
+      <c r="I70" s="388" t="n"/>
+      <c r="J70" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C70,'SAERTEX-prijstabel'!$B$2:$B$496,$D70,'SAERTEX-prijstabel'!$C$2:$C$496,$E70,'SAERTEX-prijstabel'!$D$2:$D$496,$F70),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K70" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G70)+N($H70))=0,0,IF((N($G70)+N($H70))&lt;15,0.25,IF((N($G70)+N($H70))&lt;=50,0.035,IF((N($G70)+N($H70))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L70" s="392">
+        <f>IF($J70=0,0,$G70*$J70*(1+$K70))</f>
+        <v/>
+      </c>
+      <c r="M70" s="392">
+        <f>N($H70)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N70" s="398">
+        <f>$L70+$M70</f>
+        <v/>
+      </c>
+      <c r="O70" s="401">
+        <f>IF($I70="","nog te plannen",IFERROR(LOOKUP($I70,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6928,21 +7615,30 @@
       <c r="E71" s="306" t="n"/>
       <c r="F71" s="306" t="n"/>
       <c r="G71" s="391" t="n"/>
-      <c r="H71" s="388" t="n"/>
-      <c r="I71" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C71,'SAERTEX-prijstabel'!$B$2:$B$496,$D71,'SAERTEX-prijstabel'!$C$2:$C$496,$E71,'SAERTEX-prijstabel'!$D$2:$D$496,$F71),0)</f>
-        <v/>
-      </c>
-      <c r="J71" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G71="","",IF($G71&lt;15,0.25,IF($G71&lt;=50,0.035,IF($G71&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K71" s="392">
-        <f>IF($I71=0,0,$G71*$I71*(1+N($J71)))</f>
-        <v/>
-      </c>
-      <c r="L71" s="401">
-        <f>IF($H71="","nog te plannen",IFERROR(LOOKUP($H71,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H71" s="391" t="n"/>
+      <c r="I71" s="388" t="n"/>
+      <c r="J71" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C71,'SAERTEX-prijstabel'!$B$2:$B$496,$D71,'SAERTEX-prijstabel'!$C$2:$C$496,$E71,'SAERTEX-prijstabel'!$D$2:$D$496,$F71),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K71" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G71)+N($H71))=0,0,IF((N($G71)+N($H71))&lt;15,0.25,IF((N($G71)+N($H71))&lt;=50,0.035,IF((N($G71)+N($H71))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L71" s="392">
+        <f>IF($J71=0,0,$G71*$J71*(1+$K71))</f>
+        <v/>
+      </c>
+      <c r="M71" s="392">
+        <f>N($H71)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N71" s="398">
+        <f>$L71+$M71</f>
+        <v/>
+      </c>
+      <c r="O71" s="401">
+        <f>IF($I71="","nog te plannen",IFERROR(LOOKUP($I71,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6954,21 +7650,30 @@
       <c r="E72" s="306" t="n"/>
       <c r="F72" s="306" t="n"/>
       <c r="G72" s="391" t="n"/>
-      <c r="H72" s="388" t="n"/>
-      <c r="I72" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C72,'SAERTEX-prijstabel'!$B$2:$B$496,$D72,'SAERTEX-prijstabel'!$C$2:$C$496,$E72,'SAERTEX-prijstabel'!$D$2:$D$496,$F72),0)</f>
-        <v/>
-      </c>
-      <c r="J72" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G72="","",IF($G72&lt;15,0.25,IF($G72&lt;=50,0.035,IF($G72&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K72" s="392">
-        <f>IF($I72=0,0,$G72*$I72*(1+N($J72)))</f>
-        <v/>
-      </c>
-      <c r="L72" s="401">
-        <f>IF($H72="","nog te plannen",IFERROR(LOOKUP($H72,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H72" s="391" t="n"/>
+      <c r="I72" s="388" t="n"/>
+      <c r="J72" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C72,'SAERTEX-prijstabel'!$B$2:$B$496,$D72,'SAERTEX-prijstabel'!$C$2:$C$496,$E72,'SAERTEX-prijstabel'!$D$2:$D$496,$F72),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K72" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G72)+N($H72))=0,0,IF((N($G72)+N($H72))&lt;15,0.25,IF((N($G72)+N($H72))&lt;=50,0.035,IF((N($G72)+N($H72))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L72" s="392">
+        <f>IF($J72=0,0,$G72*$J72*(1+$K72))</f>
+        <v/>
+      </c>
+      <c r="M72" s="392">
+        <f>N($H72)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N72" s="398">
+        <f>$L72+$M72</f>
+        <v/>
+      </c>
+      <c r="O72" s="401">
+        <f>IF($I72="","nog te plannen",IFERROR(LOOKUP($I72,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6980,21 +7685,30 @@
       <c r="E73" s="306" t="n"/>
       <c r="F73" s="306" t="n"/>
       <c r="G73" s="391" t="n"/>
-      <c r="H73" s="388" t="n"/>
-      <c r="I73" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C73,'SAERTEX-prijstabel'!$B$2:$B$496,$D73,'SAERTEX-prijstabel'!$C$2:$C$496,$E73,'SAERTEX-prijstabel'!$D$2:$D$496,$F73),0)</f>
-        <v/>
-      </c>
-      <c r="J73" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G73="","",IF($G73&lt;15,0.25,IF($G73&lt;=50,0.035,IF($G73&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K73" s="392">
-        <f>IF($I73=0,0,$G73*$I73*(1+N($J73)))</f>
-        <v/>
-      </c>
-      <c r="L73" s="401">
-        <f>IF($H73="","nog te plannen",IFERROR(LOOKUP($H73,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H73" s="391" t="n"/>
+      <c r="I73" s="388" t="n"/>
+      <c r="J73" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C73,'SAERTEX-prijstabel'!$B$2:$B$496,$D73,'SAERTEX-prijstabel'!$C$2:$C$496,$E73,'SAERTEX-prijstabel'!$D$2:$D$496,$F73),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K73" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G73)+N($H73))=0,0,IF((N($G73)+N($H73))&lt;15,0.25,IF((N($G73)+N($H73))&lt;=50,0.035,IF((N($G73)+N($H73))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L73" s="392">
+        <f>IF($J73=0,0,$G73*$J73*(1+$K73))</f>
+        <v/>
+      </c>
+      <c r="M73" s="392">
+        <f>N($H73)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N73" s="398">
+        <f>$L73+$M73</f>
+        <v/>
+      </c>
+      <c r="O73" s="401">
+        <f>IF($I73="","nog te plannen",IFERROR(LOOKUP($I73,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7006,21 +7720,30 @@
       <c r="E74" s="306" t="n"/>
       <c r="F74" s="306" t="n"/>
       <c r="G74" s="391" t="n"/>
-      <c r="H74" s="388" t="n"/>
-      <c r="I74" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C74,'SAERTEX-prijstabel'!$B$2:$B$496,$D74,'SAERTEX-prijstabel'!$C$2:$C$496,$E74,'SAERTEX-prijstabel'!$D$2:$D$496,$F74),0)</f>
-        <v/>
-      </c>
-      <c r="J74" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G74="","",IF($G74&lt;15,0.25,IF($G74&lt;=50,0.035,IF($G74&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K74" s="392">
-        <f>IF($I74=0,0,$G74*$I74*(1+N($J74)))</f>
-        <v/>
-      </c>
-      <c r="L74" s="401">
-        <f>IF($H74="","nog te plannen",IFERROR(LOOKUP($H74,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H74" s="391" t="n"/>
+      <c r="I74" s="388" t="n"/>
+      <c r="J74" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C74,'SAERTEX-prijstabel'!$B$2:$B$496,$D74,'SAERTEX-prijstabel'!$C$2:$C$496,$E74,'SAERTEX-prijstabel'!$D$2:$D$496,$F74),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K74" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G74)+N($H74))=0,0,IF((N($G74)+N($H74))&lt;15,0.25,IF((N($G74)+N($H74))&lt;=50,0.035,IF((N($G74)+N($H74))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L74" s="392">
+        <f>IF($J74=0,0,$G74*$J74*(1+$K74))</f>
+        <v/>
+      </c>
+      <c r="M74" s="392">
+        <f>N($H74)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N74" s="398">
+        <f>$L74+$M74</f>
+        <v/>
+      </c>
+      <c r="O74" s="401">
+        <f>IF($I74="","nog te plannen",IFERROR(LOOKUP($I74,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7032,21 +7755,30 @@
       <c r="E75" s="306" t="n"/>
       <c r="F75" s="306" t="n"/>
       <c r="G75" s="391" t="n"/>
-      <c r="H75" s="388" t="n"/>
-      <c r="I75" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C75,'SAERTEX-prijstabel'!$B$2:$B$496,$D75,'SAERTEX-prijstabel'!$C$2:$C$496,$E75,'SAERTEX-prijstabel'!$D$2:$D$496,$F75),0)</f>
-        <v/>
-      </c>
-      <c r="J75" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G75="","",IF($G75&lt;15,0.25,IF($G75&lt;=50,0.035,IF($G75&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K75" s="392">
-        <f>IF($I75=0,0,$G75*$I75*(1+N($J75)))</f>
-        <v/>
-      </c>
-      <c r="L75" s="401">
-        <f>IF($H75="","nog te plannen",IFERROR(LOOKUP($H75,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H75" s="391" t="n"/>
+      <c r="I75" s="388" t="n"/>
+      <c r="J75" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C75,'SAERTEX-prijstabel'!$B$2:$B$496,$D75,'SAERTEX-prijstabel'!$C$2:$C$496,$E75,'SAERTEX-prijstabel'!$D$2:$D$496,$F75),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K75" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G75)+N($H75))=0,0,IF((N($G75)+N($H75))&lt;15,0.25,IF((N($G75)+N($H75))&lt;=50,0.035,IF((N($G75)+N($H75))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L75" s="392">
+        <f>IF($J75=0,0,$G75*$J75*(1+$K75))</f>
+        <v/>
+      </c>
+      <c r="M75" s="392">
+        <f>N($H75)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N75" s="398">
+        <f>$L75+$M75</f>
+        <v/>
+      </c>
+      <c r="O75" s="401">
+        <f>IF($I75="","nog te plannen",IFERROR(LOOKUP($I75,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7058,21 +7790,30 @@
       <c r="E76" s="306" t="n"/>
       <c r="F76" s="306" t="n"/>
       <c r="G76" s="391" t="n"/>
-      <c r="H76" s="388" t="n"/>
-      <c r="I76" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C76,'SAERTEX-prijstabel'!$B$2:$B$496,$D76,'SAERTEX-prijstabel'!$C$2:$C$496,$E76,'SAERTEX-prijstabel'!$D$2:$D$496,$F76),0)</f>
-        <v/>
-      </c>
-      <c r="J76" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G76="","",IF($G76&lt;15,0.25,IF($G76&lt;=50,0.035,IF($G76&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K76" s="392">
-        <f>IF($I76=0,0,$G76*$I76*(1+N($J76)))</f>
-        <v/>
-      </c>
-      <c r="L76" s="401">
-        <f>IF($H76="","nog te plannen",IFERROR(LOOKUP($H76,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H76" s="391" t="n"/>
+      <c r="I76" s="388" t="n"/>
+      <c r="J76" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C76,'SAERTEX-prijstabel'!$B$2:$B$496,$D76,'SAERTEX-prijstabel'!$C$2:$C$496,$E76,'SAERTEX-prijstabel'!$D$2:$D$496,$F76),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K76" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G76)+N($H76))=0,0,IF((N($G76)+N($H76))&lt;15,0.25,IF((N($G76)+N($H76))&lt;=50,0.035,IF((N($G76)+N($H76))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L76" s="392">
+        <f>IF($J76=0,0,$G76*$J76*(1+$K76))</f>
+        <v/>
+      </c>
+      <c r="M76" s="392">
+        <f>N($H76)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N76" s="398">
+        <f>$L76+$M76</f>
+        <v/>
+      </c>
+      <c r="O76" s="401">
+        <f>IF($I76="","nog te plannen",IFERROR(LOOKUP($I76,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7084,21 +7825,30 @@
       <c r="E77" s="306" t="n"/>
       <c r="F77" s="306" t="n"/>
       <c r="G77" s="391" t="n"/>
-      <c r="H77" s="388" t="n"/>
-      <c r="I77" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C77,'SAERTEX-prijstabel'!$B$2:$B$496,$D77,'SAERTEX-prijstabel'!$C$2:$C$496,$E77,'SAERTEX-prijstabel'!$D$2:$D$496,$F77),0)</f>
-        <v/>
-      </c>
-      <c r="J77" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G77="","",IF($G77&lt;15,0.25,IF($G77&lt;=50,0.035,IF($G77&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K77" s="392">
-        <f>IF($I77=0,0,$G77*$I77*(1+N($J77)))</f>
-        <v/>
-      </c>
-      <c r="L77" s="401">
-        <f>IF($H77="","nog te plannen",IFERROR(LOOKUP($H77,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H77" s="391" t="n"/>
+      <c r="I77" s="388" t="n"/>
+      <c r="J77" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C77,'SAERTEX-prijstabel'!$B$2:$B$496,$D77,'SAERTEX-prijstabel'!$C$2:$C$496,$E77,'SAERTEX-prijstabel'!$D$2:$D$496,$F77),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K77" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G77)+N($H77))=0,0,IF((N($G77)+N($H77))&lt;15,0.25,IF((N($G77)+N($H77))&lt;=50,0.035,IF((N($G77)+N($H77))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L77" s="392">
+        <f>IF($J77=0,0,$G77*$J77*(1+$K77))</f>
+        <v/>
+      </c>
+      <c r="M77" s="392">
+        <f>N($H77)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N77" s="398">
+        <f>$L77+$M77</f>
+        <v/>
+      </c>
+      <c r="O77" s="401">
+        <f>IF($I77="","nog te plannen",IFERROR(LOOKUP($I77,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7110,21 +7860,30 @@
       <c r="E78" s="306" t="n"/>
       <c r="F78" s="306" t="n"/>
       <c r="G78" s="391" t="n"/>
-      <c r="H78" s="388" t="n"/>
-      <c r="I78" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C78,'SAERTEX-prijstabel'!$B$2:$B$496,$D78,'SAERTEX-prijstabel'!$C$2:$C$496,$E78,'SAERTEX-prijstabel'!$D$2:$D$496,$F78),0)</f>
-        <v/>
-      </c>
-      <c r="J78" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G78="","",IF($G78&lt;15,0.25,IF($G78&lt;=50,0.035,IF($G78&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K78" s="392">
-        <f>IF($I78=0,0,$G78*$I78*(1+N($J78)))</f>
-        <v/>
-      </c>
-      <c r="L78" s="401">
-        <f>IF($H78="","nog te plannen",IFERROR(LOOKUP($H78,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H78" s="391" t="n"/>
+      <c r="I78" s="388" t="n"/>
+      <c r="J78" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C78,'SAERTEX-prijstabel'!$B$2:$B$496,$D78,'SAERTEX-prijstabel'!$C$2:$C$496,$E78,'SAERTEX-prijstabel'!$D$2:$D$496,$F78),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K78" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G78)+N($H78))=0,0,IF((N($G78)+N($H78))&lt;15,0.25,IF((N($G78)+N($H78))&lt;=50,0.035,IF((N($G78)+N($H78))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L78" s="392">
+        <f>IF($J78=0,0,$G78*$J78*(1+$K78))</f>
+        <v/>
+      </c>
+      <c r="M78" s="392">
+        <f>N($H78)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N78" s="398">
+        <f>$L78+$M78</f>
+        <v/>
+      </c>
+      <c r="O78" s="401">
+        <f>IF($I78="","nog te plannen",IFERROR(LOOKUP($I78,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7136,21 +7895,30 @@
       <c r="E79" s="306" t="n"/>
       <c r="F79" s="306" t="n"/>
       <c r="G79" s="391" t="n"/>
-      <c r="H79" s="388" t="n"/>
-      <c r="I79" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C79,'SAERTEX-prijstabel'!$B$2:$B$496,$D79,'SAERTEX-prijstabel'!$C$2:$C$496,$E79,'SAERTEX-prijstabel'!$D$2:$D$496,$F79),0)</f>
-        <v/>
-      </c>
-      <c r="J79" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G79="","",IF($G79&lt;15,0.25,IF($G79&lt;=50,0.035,IF($G79&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K79" s="392">
-        <f>IF($I79=0,0,$G79*$I79*(1+N($J79)))</f>
-        <v/>
-      </c>
-      <c r="L79" s="401">
-        <f>IF($H79="","nog te plannen",IFERROR(LOOKUP($H79,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H79" s="391" t="n"/>
+      <c r="I79" s="388" t="n"/>
+      <c r="J79" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C79,'SAERTEX-prijstabel'!$B$2:$B$496,$D79,'SAERTEX-prijstabel'!$C$2:$C$496,$E79,'SAERTEX-prijstabel'!$D$2:$D$496,$F79),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K79" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G79)+N($H79))=0,0,IF((N($G79)+N($H79))&lt;15,0.25,IF((N($G79)+N($H79))&lt;=50,0.035,IF((N($G79)+N($H79))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L79" s="392">
+        <f>IF($J79=0,0,$G79*$J79*(1+$K79))</f>
+        <v/>
+      </c>
+      <c r="M79" s="392">
+        <f>N($H79)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N79" s="398">
+        <f>$L79+$M79</f>
+        <v/>
+      </c>
+      <c r="O79" s="401">
+        <f>IF($I79="","nog te plannen",IFERROR(LOOKUP($I79,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7162,32 +7930,41 @@
       <c r="E80" s="306" t="n"/>
       <c r="F80" s="306" t="n"/>
       <c r="G80" s="391" t="n"/>
-      <c r="H80" s="388" t="n"/>
-      <c r="I80" s="392">
-        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C80,'SAERTEX-prijstabel'!$B$2:$B$496,$D80,'SAERTEX-prijstabel'!$C$2:$C$496,$E80,'SAERTEX-prijstabel'!$D$2:$D$496,$F80),0)</f>
-        <v/>
-      </c>
-      <c r="J80" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF($G80="","",IF($G80&lt;15,0.25,IF($G80&lt;=50,0.035,IF($G80&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="K80" s="392">
-        <f>IF($I80=0,0,$G80*$I80*(1+N($J80)))</f>
-        <v/>
-      </c>
-      <c r="L80" s="401">
-        <f>IF($H80="","nog te plannen",IFERROR(LOOKUP($H80,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="H80" s="391" t="n"/>
+      <c r="I80" s="388" t="n"/>
+      <c r="J80" s="392">
+        <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C80,'SAERTEX-prijstabel'!$B$2:$B$496,$D80,'SAERTEX-prijstabel'!$C$2:$C$496,$E80,'SAERTEX-prijstabel'!$D$2:$D$496,$F80),0)*(1+'SAERTEX 2026'!$B$3)</f>
+        <v/>
+      </c>
+      <c r="K80" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G80)+N($H80))=0,0,IF((N($G80)+N($H80))&lt;15,0.25,IF((N($G80)+N($H80))&lt;=50,0.035,IF((N($G80)+N($H80))&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="L80" s="392">
+        <f>IF($J80=0,0,$G80*$J80*(1+$K80))</f>
+        <v/>
+      </c>
+      <c r="M80" s="392">
+        <f>N($H80)*$E$3</f>
+        <v/>
+      </c>
+      <c r="N80" s="398">
+        <f>$L80+$M80</f>
+        <v/>
+      </c>
+      <c r="O80" s="401">
+        <f>IF($I80="","nog te plannen",IFERROR(LOOKUP($I80,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="J81" s="402" t="inlineStr">
+      <c r="M81" s="402" t="inlineStr">
         <is>
           <t>TOTAAL</t>
         </is>
       </c>
-      <c r="K81" s="403">
-        <f>SUM(K5:K80)</f>
+      <c r="N81" s="403">
+        <f>SUM(N5:N80)</f>
         <v/>
       </c>
     </row>
@@ -7399,7 +8176,7 @@
       <c r="D14" s="306" t="n"/>
       <c r="E14" s="410" t="n"/>
       <c r="F14" s="411">
-        <f>'Kousen'!K81</f>
+        <f>'Kousen'!N81</f>
         <v/>
       </c>
       <c r="G14" s="410" t="n"/>
@@ -15479,6 +16256,21 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="442" t="inlineStr">
+        <is>
+          <t>Indexering op deze prijslijst:</t>
+        </is>
+      </c>
+      <c r="B3" s="443" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="422" t="inlineStr">
+        <is>
+          <t>(bijv. 3,5% = prijzen +3,5% t.o.v. lijst 9-5-2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="419" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Kousen terug naar één geïmpregneerde lengte; indexering op 0%
- SAERTEX kent geen dry-lengte: dry-liner-kolommen verwijderd, weer één
  Lengte -> één Kostprijs (lengte x €/m x (1+handling))
- Indexering staat op 0% zodat de 2026-prijzen gelden (instelbaar op SAERTEX 2026)
- Totalen weer doorgekoppeld (Periode-overzicht, Prognose, Overzicht)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5wVhvLcrmmgSCsGwdMWTF
</commit_message>
<xml_diff>
--- a/Kostencalculatie_Compleet.xlsx
+++ b/Kostencalculatie_Compleet.xlsx
@@ -3649,7 +3649,7 @@
       </c>
       <c r="C26" s="244" t="n"/>
       <c r="D26" s="245">
-        <f>'Kousen'!N81</f>
+        <f>'Kousen'!K81</f>
         <v/>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="B17" s="437">
-        <f>SUM(Kousen!$N$5:$N$80)</f>
+        <f>SUM(Kousen!$K$5:$K$80)</f>
         <v/>
       </c>
     </row>
@@ -4064,11 +4064,11 @@
         <v/>
       </c>
       <c r="D25" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C25)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C25)</f>
         <v/>
       </c>
       <c r="E25" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D25</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D25</f>
         <v/>
       </c>
       <c r="F25" s="385" t="n"/>
@@ -4097,11 +4097,11 @@
         <v/>
       </c>
       <c r="D26" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C26)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C26)</f>
         <v/>
       </c>
       <c r="E26" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D26</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D26</f>
         <v/>
       </c>
       <c r="F26" s="385" t="n"/>
@@ -4130,11 +4130,11 @@
         <v/>
       </c>
       <c r="D27" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C27)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C27)</f>
         <v/>
       </c>
       <c r="E27" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D27</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D27</f>
         <v/>
       </c>
       <c r="F27" s="385" t="n"/>
@@ -4163,11 +4163,11 @@
         <v/>
       </c>
       <c r="D28" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C28)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C28)</f>
         <v/>
       </c>
       <c r="E28" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D28</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D28</f>
         <v/>
       </c>
       <c r="F28" s="385" t="n"/>
@@ -4196,11 +4196,11 @@
         <v/>
       </c>
       <c r="D29" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C29)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C29)</f>
         <v/>
       </c>
       <c r="E29" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D29</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D29</f>
         <v/>
       </c>
       <c r="F29" s="385" t="n"/>
@@ -4229,11 +4229,11 @@
         <v/>
       </c>
       <c r="D30" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C30)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C30)</f>
         <v/>
       </c>
       <c r="E30" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D30</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D30</f>
         <v/>
       </c>
       <c r="F30" s="385" t="n"/>
@@ -4262,11 +4262,11 @@
         <v/>
       </c>
       <c r="D31" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C31)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C31)</f>
         <v/>
       </c>
       <c r="E31" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D31</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D31</f>
         <v/>
       </c>
       <c r="F31" s="385" t="n"/>
@@ -4295,11 +4295,11 @@
         <v/>
       </c>
       <c r="D32" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C32)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C32)</f>
         <v/>
       </c>
       <c r="E32" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D32</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D32</f>
         <v/>
       </c>
       <c r="F32" s="385" t="n"/>
@@ -4328,11 +4328,11 @@
         <v/>
       </c>
       <c r="D33" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C33)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C33)</f>
         <v/>
       </c>
       <c r="E33" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D33</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D33</f>
         <v/>
       </c>
       <c r="F33" s="385" t="n"/>
@@ -4361,11 +4361,11 @@
         <v/>
       </c>
       <c r="D34" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C34)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C34)</f>
         <v/>
       </c>
       <c r="E34" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D34</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D34</f>
         <v/>
       </c>
       <c r="F34" s="385" t="n"/>
@@ -4394,11 +4394,11 @@
         <v/>
       </c>
       <c r="D35" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C35)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C35)</f>
         <v/>
       </c>
       <c r="E35" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D35</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D35</f>
         <v/>
       </c>
       <c r="F35" s="385" t="n"/>
@@ -4427,11 +4427,11 @@
         <v/>
       </c>
       <c r="D36" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C36)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C36)</f>
         <v/>
       </c>
       <c r="E36" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D36</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D36</f>
         <v/>
       </c>
       <c r="F36" s="385" t="n"/>
@@ -4460,11 +4460,11 @@
         <v/>
       </c>
       <c r="D37" s="392">
-        <f>SUMIFS(Kousen!$N$5:$N$80,Kousen!$I$5:$I$80,"&lt;="&amp;$C37)</f>
+        <f>SUMIFS(Kousen!$K$5:$K$80,Kousen!$H$5:$H$80,"&lt;="&amp;$C37)</f>
         <v/>
       </c>
       <c r="E37" s="392">
-        <f>SUM(Kousen!$N$5:$N$80)-$D37</f>
+        <f>SUM(Kousen!$K$5:$K$80)-$D37</f>
         <v/>
       </c>
       <c r="F37" s="385" t="n"/>
@@ -4494,24 +4494,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4524,7 +4521,7 @@
     <row r="2">
       <c r="A2" s="386" t="inlineStr">
         <is>
-          <t>Geel = invoer. €/m (incl. indexering), handling, kosten en periode rekenen automatisch.</t>
+          <t>Geel = invoer. Lengte = totale geïmpregneerde lengte. €/m, handling, kostprijs en periode rekenen automatisch.</t>
         </is>
       </c>
     </row>
@@ -4541,26 +4538,20 @@
       </c>
       <c r="D3" s="421" t="inlineStr">
         <is>
-          <t>Dry-liner €/m:</t>
-        </is>
-      </c>
-      <c r="E3" s="385" t="n"/>
-      <c r="F3" s="421" t="inlineStr">
-        <is>
           <t>Indexering SAERTEX:</t>
         </is>
       </c>
-      <c r="G3" s="441">
+      <c r="E3" s="441">
         <f>'SAERTEX 2026'!$B$3</f>
         <v/>
       </c>
-      <c r="I3" s="422" t="inlineStr">
-        <is>
-          <t>(dry-€/m = tarief voor omslag/eindstuk; indexering stel je in op SAERTEX 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+      <c r="F3" s="422" t="inlineStr">
+        <is>
+          <t>(indexering = 0% → 2026-prijzen; aanpassen op blad SAERTEX 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="315" t="inlineStr">
         <is>
           <t>Kousnr</t>
@@ -4594,53 +4585,35 @@
       </c>
       <c r="G4" s="315" t="inlineStr">
         <is>
-          <t>Geïmpreg.
-lengte (m)</t>
+          <t>Lengte
+(m)</t>
         </is>
       </c>
       <c r="H4" s="315" t="inlineStr">
-        <is>
-          <t>Dry/omslag
-lengte (m)</t>
-        </is>
-      </c>
-      <c r="I4" s="315" t="inlineStr">
         <is>
           <t>Inbreng-
 datum</t>
         </is>
       </c>
-      <c r="J4" s="315" t="inlineStr">
+      <c r="I4" s="315" t="inlineStr">
         <is>
           <t>€/m
 (basis)</t>
         </is>
       </c>
-      <c r="K4" s="315" t="inlineStr">
+      <c r="J4" s="315" t="inlineStr">
         <is>
           <t>Handling
 %</t>
         </is>
       </c>
+      <c r="K4" s="315" t="inlineStr">
+        <is>
+          <t>Kostprijs
+(€)</t>
+        </is>
+      </c>
       <c r="L4" s="315" t="inlineStr">
-        <is>
-          <t>Kosten
-geïmpreg.</t>
-        </is>
-      </c>
-      <c r="M4" s="315" t="inlineStr">
-        <is>
-          <t>Kosten
-dry-liner</t>
-        </is>
-      </c>
-      <c r="N4" s="315" t="inlineStr">
-        <is>
-          <t>Kostprijs
-totaal (€)</t>
-        </is>
-      </c>
-      <c r="O4" s="315" t="inlineStr">
         <is>
           <t>Periode
 (auto)</t>
@@ -4677,34 +4650,23 @@
       <c r="G5" s="391" t="n">
         <v>121.8</v>
       </c>
-      <c r="H5" s="391" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="I5" s="417" t="n">
+      <c r="H5" s="417" t="n">
         <v>45294</v>
       </c>
-      <c r="J5" s="392">
+      <c r="I5" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C5,'SAERTEX-prijstabel'!$B$2:$B$496,$D5,'SAERTEX-prijstabel'!$C$2:$C$496,$E5,'SAERTEX-prijstabel'!$D$2:$D$496,$F5),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K5" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G5)+N($H5))=0,0,IF((N($G5)+N($H5))&lt;15,0.25,IF((N($G5)+N($H5))&lt;=50,0.035,IF((N($G5)+N($H5))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L5" s="392">
-        <f>IF($J5=0,0,$G5*$J5*(1+$K5))</f>
-        <v/>
-      </c>
-      <c r="M5" s="392">
-        <f>N($H5)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N5" s="398">
-        <f>$L5+$M5</f>
-        <v/>
-      </c>
-      <c r="O5" s="401">
-        <f>IF($I5="","nog te plannen",IFERROR(LOOKUP($I5,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J5" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G5)=0,0,IF($G5&lt;15,0.25,IF($G5&lt;=50,0.035,IF($G5&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K5" s="398">
+        <f>IF($I5=0,0,$G5*$I5*(1+$J5))</f>
+        <v/>
+      </c>
+      <c r="L5" s="401">
+        <f>IF($H5="","nog te plannen",IFERROR(LOOKUP($H5,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4738,34 +4700,23 @@
       <c r="G6" s="391" t="n">
         <v>30.6</v>
       </c>
-      <c r="H6" s="391" t="n">
-        <v>4.34</v>
-      </c>
-      <c r="I6" s="417" t="n">
+      <c r="H6" s="417" t="n">
         <v>45296</v>
       </c>
-      <c r="J6" s="392">
+      <c r="I6" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C6,'SAERTEX-prijstabel'!$B$2:$B$496,$D6,'SAERTEX-prijstabel'!$C$2:$C$496,$E6,'SAERTEX-prijstabel'!$D$2:$D$496,$F6),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K6" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G6)+N($H6))=0,0,IF((N($G6)+N($H6))&lt;15,0.25,IF((N($G6)+N($H6))&lt;=50,0.035,IF((N($G6)+N($H6))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L6" s="392">
-        <f>IF($J6=0,0,$G6*$J6*(1+$K6))</f>
-        <v/>
-      </c>
-      <c r="M6" s="392">
-        <f>N($H6)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N6" s="398">
-        <f>$L6+$M6</f>
-        <v/>
-      </c>
-      <c r="O6" s="401">
-        <f>IF($I6="","nog te plannen",IFERROR(LOOKUP($I6,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J6" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G6)=0,0,IF($G6&lt;15,0.25,IF($G6&lt;=50,0.035,IF($G6&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K6" s="398">
+        <f>IF($I6=0,0,$G6*$I6*(1+$J6))</f>
+        <v/>
+      </c>
+      <c r="L6" s="401">
+        <f>IF($H6="","nog te plannen",IFERROR(LOOKUP($H6,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4799,34 +4750,23 @@
       <c r="G7" s="391" t="n">
         <v>60</v>
       </c>
-      <c r="H7" s="391" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="I7" s="417" t="n">
+      <c r="H7" s="417" t="n">
         <v>45298</v>
       </c>
-      <c r="J7" s="392">
+      <c r="I7" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C7,'SAERTEX-prijstabel'!$B$2:$B$496,$D7,'SAERTEX-prijstabel'!$C$2:$C$496,$E7,'SAERTEX-prijstabel'!$D$2:$D$496,$F7),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K7" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G7)+N($H7))=0,0,IF((N($G7)+N($H7))&lt;15,0.25,IF((N($G7)+N($H7))&lt;=50,0.035,IF((N($G7)+N($H7))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L7" s="392">
-        <f>IF($J7=0,0,$G7*$J7*(1+$K7))</f>
-        <v/>
-      </c>
-      <c r="M7" s="392">
-        <f>N($H7)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N7" s="398">
-        <f>$L7+$M7</f>
-        <v/>
-      </c>
-      <c r="O7" s="401">
-        <f>IF($I7="","nog te plannen",IFERROR(LOOKUP($I7,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J7" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G7)=0,0,IF($G7&lt;15,0.25,IF($G7&lt;=50,0.035,IF($G7&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K7" s="398">
+        <f>IF($I7=0,0,$G7*$I7*(1+$J7))</f>
+        <v/>
+      </c>
+      <c r="L7" s="401">
+        <f>IF($H7="","nog te plannen",IFERROR(LOOKUP($H7,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4860,34 +4800,23 @@
       <c r="G8" s="391" t="n">
         <v>104.7</v>
       </c>
-      <c r="H8" s="391" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="I8" s="417" t="n">
+      <c r="H8" s="417" t="n">
         <v>45300</v>
       </c>
-      <c r="J8" s="392">
+      <c r="I8" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C8,'SAERTEX-prijstabel'!$B$2:$B$496,$D8,'SAERTEX-prijstabel'!$C$2:$C$496,$E8,'SAERTEX-prijstabel'!$D$2:$D$496,$F8),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K8" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G8)+N($H8))=0,0,IF((N($G8)+N($H8))&lt;15,0.25,IF((N($G8)+N($H8))&lt;=50,0.035,IF((N($G8)+N($H8))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L8" s="392">
-        <f>IF($J8=0,0,$G8*$J8*(1+$K8))</f>
-        <v/>
-      </c>
-      <c r="M8" s="392">
-        <f>N($H8)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N8" s="398">
-        <f>$L8+$M8</f>
-        <v/>
-      </c>
-      <c r="O8" s="401">
-        <f>IF($I8="","nog te plannen",IFERROR(LOOKUP($I8,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J8" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G8)=0,0,IF($G8&lt;15,0.25,IF($G8&lt;=50,0.035,IF($G8&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K8" s="398">
+        <f>IF($I8=0,0,$G8*$I8*(1+$J8))</f>
+        <v/>
+      </c>
+      <c r="L8" s="401">
+        <f>IF($H8="","nog te plannen",IFERROR(LOOKUP($H8,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4921,34 +4850,23 @@
       <c r="G9" s="391" t="n">
         <v>67.3</v>
       </c>
-      <c r="H9" s="391" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="I9" s="417" t="n">
+      <c r="H9" s="417" t="n">
         <v>45302</v>
       </c>
-      <c r="J9" s="392">
+      <c r="I9" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C9,'SAERTEX-prijstabel'!$B$2:$B$496,$D9,'SAERTEX-prijstabel'!$C$2:$C$496,$E9,'SAERTEX-prijstabel'!$D$2:$D$496,$F9),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K9" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G9)+N($H9))=0,0,IF((N($G9)+N($H9))&lt;15,0.25,IF((N($G9)+N($H9))&lt;=50,0.035,IF((N($G9)+N($H9))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L9" s="392">
-        <f>IF($J9=0,0,$G9*$J9*(1+$K9))</f>
-        <v/>
-      </c>
-      <c r="M9" s="392">
-        <f>N($H9)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N9" s="398">
-        <f>$L9+$M9</f>
-        <v/>
-      </c>
-      <c r="O9" s="401">
-        <f>IF($I9="","nog te plannen",IFERROR(LOOKUP($I9,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J9" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G9)=0,0,IF($G9&lt;15,0.25,IF($G9&lt;=50,0.035,IF($G9&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K9" s="398">
+        <f>IF($I9=0,0,$G9*$I9*(1+$J9))</f>
+        <v/>
+      </c>
+      <c r="L9" s="401">
+        <f>IF($H9="","nog te plannen",IFERROR(LOOKUP($H9,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -4982,34 +4900,23 @@
       <c r="G10" s="391" t="n">
         <v>42.1</v>
       </c>
-      <c r="H10" s="391" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="I10" s="417" t="n">
+      <c r="H10" s="417" t="n">
         <v>45304</v>
       </c>
-      <c r="J10" s="392">
+      <c r="I10" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C10,'SAERTEX-prijstabel'!$B$2:$B$496,$D10,'SAERTEX-prijstabel'!$C$2:$C$496,$E10,'SAERTEX-prijstabel'!$D$2:$D$496,$F10),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K10" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G10)+N($H10))=0,0,IF((N($G10)+N($H10))&lt;15,0.25,IF((N($G10)+N($H10))&lt;=50,0.035,IF((N($G10)+N($H10))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L10" s="392">
-        <f>IF($J10=0,0,$G10*$J10*(1+$K10))</f>
-        <v/>
-      </c>
-      <c r="M10" s="392">
-        <f>N($H10)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N10" s="398">
-        <f>$L10+$M10</f>
-        <v/>
-      </c>
-      <c r="O10" s="401">
-        <f>IF($I10="","nog te plannen",IFERROR(LOOKUP($I10,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J10" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G10)=0,0,IF($G10&lt;15,0.25,IF($G10&lt;=50,0.035,IF($G10&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K10" s="398">
+        <f>IF($I10=0,0,$G10*$I10*(1+$J10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="401">
+        <f>IF($H10="","nog te plannen",IFERROR(LOOKUP($H10,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5043,34 +4950,23 @@
       <c r="G11" s="391" t="n">
         <v>35.4</v>
       </c>
-      <c r="H11" s="391" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="I11" s="417" t="n">
+      <c r="H11" s="417" t="n">
         <v>45306</v>
       </c>
-      <c r="J11" s="392">
+      <c r="I11" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C11,'SAERTEX-prijstabel'!$B$2:$B$496,$D11,'SAERTEX-prijstabel'!$C$2:$C$496,$E11,'SAERTEX-prijstabel'!$D$2:$D$496,$F11),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K11" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G11)+N($H11))=0,0,IF((N($G11)+N($H11))&lt;15,0.25,IF((N($G11)+N($H11))&lt;=50,0.035,IF((N($G11)+N($H11))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L11" s="392">
-        <f>IF($J11=0,0,$G11*$J11*(1+$K11))</f>
-        <v/>
-      </c>
-      <c r="M11" s="392">
-        <f>N($H11)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N11" s="398">
-        <f>$L11+$M11</f>
-        <v/>
-      </c>
-      <c r="O11" s="401">
-        <f>IF($I11="","nog te plannen",IFERROR(LOOKUP($I11,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J11" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G11)=0,0,IF($G11&lt;15,0.25,IF($G11&lt;=50,0.035,IF($G11&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K11" s="398">
+        <f>IF($I11=0,0,$G11*$I11*(1+$J11))</f>
+        <v/>
+      </c>
+      <c r="L11" s="401">
+        <f>IF($H11="","nog te plannen",IFERROR(LOOKUP($H11,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5104,34 +5000,23 @@
       <c r="G12" s="391" t="n">
         <v>41.1</v>
       </c>
-      <c r="H12" s="391" t="n">
-        <v>4.29</v>
-      </c>
-      <c r="I12" s="417" t="n">
+      <c r="H12" s="417" t="n">
         <v>45308</v>
       </c>
-      <c r="J12" s="392">
+      <c r="I12" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C12,'SAERTEX-prijstabel'!$B$2:$B$496,$D12,'SAERTEX-prijstabel'!$C$2:$C$496,$E12,'SAERTEX-prijstabel'!$D$2:$D$496,$F12),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K12" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G12)+N($H12))=0,0,IF((N($G12)+N($H12))&lt;15,0.25,IF((N($G12)+N($H12))&lt;=50,0.035,IF((N($G12)+N($H12))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L12" s="392">
-        <f>IF($J12=0,0,$G12*$J12*(1+$K12))</f>
-        <v/>
-      </c>
-      <c r="M12" s="392">
-        <f>N($H12)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N12" s="398">
-        <f>$L12+$M12</f>
-        <v/>
-      </c>
-      <c r="O12" s="401">
-        <f>IF($I12="","nog te plannen",IFERROR(LOOKUP($I12,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J12" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G12)=0,0,IF($G12&lt;15,0.25,IF($G12&lt;=50,0.035,IF($G12&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K12" s="398">
+        <f>IF($I12=0,0,$G12*$I12*(1+$J12))</f>
+        <v/>
+      </c>
+      <c r="L12" s="401">
+        <f>IF($H12="","nog te plannen",IFERROR(LOOKUP($H12,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5165,34 +5050,23 @@
       <c r="G13" s="391" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="H13" s="391" t="n">
-        <v>4.47</v>
-      </c>
-      <c r="I13" s="417" t="n">
+      <c r="H13" s="417" t="n">
         <v>45310</v>
       </c>
-      <c r="J13" s="392">
+      <c r="I13" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C13,'SAERTEX-prijstabel'!$B$2:$B$496,$D13,'SAERTEX-prijstabel'!$C$2:$C$496,$E13,'SAERTEX-prijstabel'!$D$2:$D$496,$F13),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K13" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G13)+N($H13))=0,0,IF((N($G13)+N($H13))&lt;15,0.25,IF((N($G13)+N($H13))&lt;=50,0.035,IF((N($G13)+N($H13))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L13" s="392">
-        <f>IF($J13=0,0,$G13*$J13*(1+$K13))</f>
-        <v/>
-      </c>
-      <c r="M13" s="392">
-        <f>N($H13)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N13" s="398">
-        <f>$L13+$M13</f>
-        <v/>
-      </c>
-      <c r="O13" s="401">
-        <f>IF($I13="","nog te plannen",IFERROR(LOOKUP($I13,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J13" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G13)=0,0,IF($G13&lt;15,0.25,IF($G13&lt;=50,0.035,IF($G13&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K13" s="398">
+        <f>IF($I13=0,0,$G13*$I13*(1+$J13))</f>
+        <v/>
+      </c>
+      <c r="L13" s="401">
+        <f>IF($H13="","nog te plannen",IFERROR(LOOKUP($H13,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5226,34 +5100,23 @@
       <c r="G14" s="391" t="n">
         <v>133.9</v>
       </c>
-      <c r="H14" s="391" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="I14" s="417" t="n">
+      <c r="H14" s="417" t="n">
         <v>45321</v>
       </c>
-      <c r="J14" s="392">
+      <c r="I14" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C14,'SAERTEX-prijstabel'!$B$2:$B$496,$D14,'SAERTEX-prijstabel'!$C$2:$C$496,$E14,'SAERTEX-prijstabel'!$D$2:$D$496,$F14),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K14" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G14)+N($H14))=0,0,IF((N($G14)+N($H14))&lt;15,0.25,IF((N($G14)+N($H14))&lt;=50,0.035,IF((N($G14)+N($H14))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L14" s="392">
-        <f>IF($J14=0,0,$G14*$J14*(1+$K14))</f>
-        <v/>
-      </c>
-      <c r="M14" s="392">
-        <f>N($H14)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N14" s="398">
-        <f>$L14+$M14</f>
-        <v/>
-      </c>
-      <c r="O14" s="401">
-        <f>IF($I14="","nog te plannen",IFERROR(LOOKUP($I14,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J14" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G14)=0,0,IF($G14&lt;15,0.25,IF($G14&lt;=50,0.035,IF($G14&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K14" s="398">
+        <f>IF($I14=0,0,$G14*$I14*(1+$J14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="401">
+        <f>IF($H14="","nog te plannen",IFERROR(LOOKUP($H14,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5287,34 +5150,23 @@
       <c r="G15" s="391" t="n">
         <v>92.3</v>
       </c>
-      <c r="H15" s="391" t="n">
-        <v>4.36</v>
-      </c>
-      <c r="I15" s="417" t="n">
+      <c r="H15" s="417" t="n">
         <v>45324</v>
       </c>
-      <c r="J15" s="392">
+      <c r="I15" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C15,'SAERTEX-prijstabel'!$B$2:$B$496,$D15,'SAERTEX-prijstabel'!$C$2:$C$496,$E15,'SAERTEX-prijstabel'!$D$2:$D$496,$F15),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K15" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G15)+N($H15))=0,0,IF((N($G15)+N($H15))&lt;15,0.25,IF((N($G15)+N($H15))&lt;=50,0.035,IF((N($G15)+N($H15))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L15" s="392">
-        <f>IF($J15=0,0,$G15*$J15*(1+$K15))</f>
-        <v/>
-      </c>
-      <c r="M15" s="392">
-        <f>N($H15)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N15" s="398">
-        <f>$L15+$M15</f>
-        <v/>
-      </c>
-      <c r="O15" s="401">
-        <f>IF($I15="","nog te plannen",IFERROR(LOOKUP($I15,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J15" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G15)=0,0,IF($G15&lt;15,0.25,IF($G15&lt;=50,0.035,IF($G15&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K15" s="398">
+        <f>IF($I15=0,0,$G15*$I15*(1+$J15))</f>
+        <v/>
+      </c>
+      <c r="L15" s="401">
+        <f>IF($H15="","nog te plannen",IFERROR(LOOKUP($H15,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5348,34 +5200,23 @@
       <c r="G16" s="391" t="n">
         <v>124.6</v>
       </c>
-      <c r="H16" s="391" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="I16" s="417" t="n">
+      <c r="H16" s="417" t="n">
         <v>45327</v>
       </c>
-      <c r="J16" s="392">
+      <c r="I16" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C16,'SAERTEX-prijstabel'!$B$2:$B$496,$D16,'SAERTEX-prijstabel'!$C$2:$C$496,$E16,'SAERTEX-prijstabel'!$D$2:$D$496,$F16),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K16" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G16)+N($H16))=0,0,IF((N($G16)+N($H16))&lt;15,0.25,IF((N($G16)+N($H16))&lt;=50,0.035,IF((N($G16)+N($H16))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L16" s="392">
-        <f>IF($J16=0,0,$G16*$J16*(1+$K16))</f>
-        <v/>
-      </c>
-      <c r="M16" s="392">
-        <f>N($H16)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N16" s="398">
-        <f>$L16+$M16</f>
-        <v/>
-      </c>
-      <c r="O16" s="401">
-        <f>IF($I16="","nog te plannen",IFERROR(LOOKUP($I16,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J16" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G16)=0,0,IF($G16&lt;15,0.25,IF($G16&lt;=50,0.035,IF($G16&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K16" s="398">
+        <f>IF($I16=0,0,$G16*$I16*(1+$J16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="401">
+        <f>IF($H16="","nog te plannen",IFERROR(LOOKUP($H16,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5409,34 +5250,23 @@
       <c r="G17" s="391" t="n">
         <v>67</v>
       </c>
-      <c r="H17" s="391" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="I17" s="417" t="n">
+      <c r="H17" s="417" t="n">
         <v>45330</v>
       </c>
-      <c r="J17" s="392">
+      <c r="I17" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C17,'SAERTEX-prijstabel'!$B$2:$B$496,$D17,'SAERTEX-prijstabel'!$C$2:$C$496,$E17,'SAERTEX-prijstabel'!$D$2:$D$496,$F17),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K17" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G17)+N($H17))=0,0,IF((N($G17)+N($H17))&lt;15,0.25,IF((N($G17)+N($H17))&lt;=50,0.035,IF((N($G17)+N($H17))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L17" s="392">
-        <f>IF($J17=0,0,$G17*$J17*(1+$K17))</f>
-        <v/>
-      </c>
-      <c r="M17" s="392">
-        <f>N($H17)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N17" s="398">
-        <f>$L17+$M17</f>
-        <v/>
-      </c>
-      <c r="O17" s="401">
-        <f>IF($I17="","nog te plannen",IFERROR(LOOKUP($I17,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J17" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G17)=0,0,IF($G17&lt;15,0.25,IF($G17&lt;=50,0.035,IF($G17&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K17" s="398">
+        <f>IF($I17=0,0,$G17*$I17*(1+$J17))</f>
+        <v/>
+      </c>
+      <c r="L17" s="401">
+        <f>IF($H17="","nog te plannen",IFERROR(LOOKUP($H17,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5470,34 +5300,23 @@
       <c r="G18" s="391" t="n">
         <v>120</v>
       </c>
-      <c r="H18" s="391" t="n">
-        <v>4.92</v>
-      </c>
-      <c r="I18" s="417" t="n">
+      <c r="H18" s="417" t="n">
         <v>45333</v>
       </c>
-      <c r="J18" s="392">
+      <c r="I18" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C18,'SAERTEX-prijstabel'!$B$2:$B$496,$D18,'SAERTEX-prijstabel'!$C$2:$C$496,$E18,'SAERTEX-prijstabel'!$D$2:$D$496,$F18),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K18" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G18)+N($H18))=0,0,IF((N($G18)+N($H18))&lt;15,0.25,IF((N($G18)+N($H18))&lt;=50,0.035,IF((N($G18)+N($H18))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L18" s="392">
-        <f>IF($J18=0,0,$G18*$J18*(1+$K18))</f>
-        <v/>
-      </c>
-      <c r="M18" s="392">
-        <f>N($H18)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N18" s="398">
-        <f>$L18+$M18</f>
-        <v/>
-      </c>
-      <c r="O18" s="401">
-        <f>IF($I18="","nog te plannen",IFERROR(LOOKUP($I18,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J18" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G18)=0,0,IF($G18&lt;15,0.25,IF($G18&lt;=50,0.035,IF($G18&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K18" s="398">
+        <f>IF($I18=0,0,$G18*$I18*(1+$J18))</f>
+        <v/>
+      </c>
+      <c r="L18" s="401">
+        <f>IF($H18="","nog te plannen",IFERROR(LOOKUP($H18,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5531,34 +5350,23 @@
       <c r="G19" s="391" t="n">
         <v>66.09999999999999</v>
       </c>
-      <c r="H19" s="391" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="I19" s="417" t="n">
+      <c r="H19" s="417" t="n">
         <v>45336</v>
       </c>
-      <c r="J19" s="392">
+      <c r="I19" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C19,'SAERTEX-prijstabel'!$B$2:$B$496,$D19,'SAERTEX-prijstabel'!$C$2:$C$496,$E19,'SAERTEX-prijstabel'!$D$2:$D$496,$F19),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K19" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G19)+N($H19))=0,0,IF((N($G19)+N($H19))&lt;15,0.25,IF((N($G19)+N($H19))&lt;=50,0.035,IF((N($G19)+N($H19))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L19" s="392">
-        <f>IF($J19=0,0,$G19*$J19*(1+$K19))</f>
-        <v/>
-      </c>
-      <c r="M19" s="392">
-        <f>N($H19)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N19" s="398">
-        <f>$L19+$M19</f>
-        <v/>
-      </c>
-      <c r="O19" s="401">
-        <f>IF($I19="","nog te plannen",IFERROR(LOOKUP($I19,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J19" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G19)=0,0,IF($G19&lt;15,0.25,IF($G19&lt;=50,0.035,IF($G19&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K19" s="398">
+        <f>IF($I19=0,0,$G19*$I19*(1+$J19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="401">
+        <f>IF($H19="","nog te plannen",IFERROR(LOOKUP($H19,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5592,34 +5400,23 @@
       <c r="G20" s="391" t="n">
         <v>14.2</v>
       </c>
-      <c r="H20" s="391" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="I20" s="417" t="n">
+      <c r="H20" s="417" t="n">
         <v>45339</v>
       </c>
-      <c r="J20" s="392">
+      <c r="I20" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C20,'SAERTEX-prijstabel'!$B$2:$B$496,$D20,'SAERTEX-prijstabel'!$C$2:$C$496,$E20,'SAERTEX-prijstabel'!$D$2:$D$496,$F20),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K20" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G20)+N($H20))=0,0,IF((N($G20)+N($H20))&lt;15,0.25,IF((N($G20)+N($H20))&lt;=50,0.035,IF((N($G20)+N($H20))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L20" s="392">
-        <f>IF($J20=0,0,$G20*$J20*(1+$K20))</f>
-        <v/>
-      </c>
-      <c r="M20" s="392">
-        <f>N($H20)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N20" s="398">
-        <f>$L20+$M20</f>
-        <v/>
-      </c>
-      <c r="O20" s="401">
-        <f>IF($I20="","nog te plannen",IFERROR(LOOKUP($I20,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J20" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G20)=0,0,IF($G20&lt;15,0.25,IF($G20&lt;=50,0.035,IF($G20&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K20" s="398">
+        <f>IF($I20=0,0,$G20*$I20*(1+$J20))</f>
+        <v/>
+      </c>
+      <c r="L20" s="401">
+        <f>IF($H20="","nog te plannen",IFERROR(LOOKUP($H20,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5653,34 +5450,23 @@
       <c r="G21" s="391" t="n">
         <v>49.2</v>
       </c>
-      <c r="H21" s="391" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="I21" s="417" t="n">
+      <c r="H21" s="417" t="n">
         <v>45342</v>
       </c>
-      <c r="J21" s="392">
+      <c r="I21" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C21,'SAERTEX-prijstabel'!$B$2:$B$496,$D21,'SAERTEX-prijstabel'!$C$2:$C$496,$E21,'SAERTEX-prijstabel'!$D$2:$D$496,$F21),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K21" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G21)+N($H21))=0,0,IF((N($G21)+N($H21))&lt;15,0.25,IF((N($G21)+N($H21))&lt;=50,0.035,IF((N($G21)+N($H21))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L21" s="392">
-        <f>IF($J21=0,0,$G21*$J21*(1+$K21))</f>
-        <v/>
-      </c>
-      <c r="M21" s="392">
-        <f>N($H21)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N21" s="398">
-        <f>$L21+$M21</f>
-        <v/>
-      </c>
-      <c r="O21" s="401">
-        <f>IF($I21="","nog te plannen",IFERROR(LOOKUP($I21,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J21" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G21)=0,0,IF($G21&lt;15,0.25,IF($G21&lt;=50,0.035,IF($G21&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K21" s="398">
+        <f>IF($I21=0,0,$G21*$I21*(1+$J21))</f>
+        <v/>
+      </c>
+      <c r="L21" s="401">
+        <f>IF($H21="","nog te plannen",IFERROR(LOOKUP($H21,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5714,34 +5500,23 @@
       <c r="G22" s="391" t="n">
         <v>54.3</v>
       </c>
-      <c r="H22" s="391" t="n">
-        <v>6.31</v>
-      </c>
-      <c r="I22" s="417" t="n">
+      <c r="H22" s="417" t="n">
         <v>45349</v>
       </c>
-      <c r="J22" s="392">
+      <c r="I22" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C22,'SAERTEX-prijstabel'!$B$2:$B$496,$D22,'SAERTEX-prijstabel'!$C$2:$C$496,$E22,'SAERTEX-prijstabel'!$D$2:$D$496,$F22),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K22" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G22)+N($H22))=0,0,IF((N($G22)+N($H22))&lt;15,0.25,IF((N($G22)+N($H22))&lt;=50,0.035,IF((N($G22)+N($H22))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L22" s="392">
-        <f>IF($J22=0,0,$G22*$J22*(1+$K22))</f>
-        <v/>
-      </c>
-      <c r="M22" s="392">
-        <f>N($H22)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N22" s="398">
-        <f>$L22+$M22</f>
-        <v/>
-      </c>
-      <c r="O22" s="401">
-        <f>IF($I22="","nog te plannen",IFERROR(LOOKUP($I22,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J22" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G22)=0,0,IF($G22&lt;15,0.25,IF($G22&lt;=50,0.035,IF($G22&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K22" s="398">
+        <f>IF($I22=0,0,$G22*$I22*(1+$J22))</f>
+        <v/>
+      </c>
+      <c r="L22" s="401">
+        <f>IF($H22="","nog te plannen",IFERROR(LOOKUP($H22,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5775,34 +5550,23 @@
       <c r="G23" s="391" t="n">
         <v>123.6</v>
       </c>
-      <c r="H23" s="391" t="n">
-        <v>5.19</v>
-      </c>
-      <c r="I23" s="417" t="n">
+      <c r="H23" s="417" t="n">
         <v>45352</v>
       </c>
-      <c r="J23" s="392">
+      <c r="I23" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C23,'SAERTEX-prijstabel'!$B$2:$B$496,$D23,'SAERTEX-prijstabel'!$C$2:$C$496,$E23,'SAERTEX-prijstabel'!$D$2:$D$496,$F23),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K23" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G23)+N($H23))=0,0,IF((N($G23)+N($H23))&lt;15,0.25,IF((N($G23)+N($H23))&lt;=50,0.035,IF((N($G23)+N($H23))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L23" s="392">
-        <f>IF($J23=0,0,$G23*$J23*(1+$K23))</f>
-        <v/>
-      </c>
-      <c r="M23" s="392">
-        <f>N($H23)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N23" s="398">
-        <f>$L23+$M23</f>
-        <v/>
-      </c>
-      <c r="O23" s="401">
-        <f>IF($I23="","nog te plannen",IFERROR(LOOKUP($I23,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J23" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G23)=0,0,IF($G23&lt;15,0.25,IF($G23&lt;=50,0.035,IF($G23&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K23" s="398">
+        <f>IF($I23=0,0,$G23*$I23*(1+$J23))</f>
+        <v/>
+      </c>
+      <c r="L23" s="401">
+        <f>IF($H23="","nog te plannen",IFERROR(LOOKUP($H23,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5836,34 +5600,23 @@
       <c r="G24" s="391" t="n">
         <v>87.59999999999999</v>
       </c>
-      <c r="H24" s="391" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="I24" s="417" t="n">
+      <c r="H24" s="417" t="n">
         <v>45355</v>
       </c>
-      <c r="J24" s="392">
+      <c r="I24" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C24,'SAERTEX-prijstabel'!$B$2:$B$496,$D24,'SAERTEX-prijstabel'!$C$2:$C$496,$E24,'SAERTEX-prijstabel'!$D$2:$D$496,$F24),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K24" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G24)+N($H24))=0,0,IF((N($G24)+N($H24))&lt;15,0.25,IF((N($G24)+N($H24))&lt;=50,0.035,IF((N($G24)+N($H24))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L24" s="392">
-        <f>IF($J24=0,0,$G24*$J24*(1+$K24))</f>
-        <v/>
-      </c>
-      <c r="M24" s="392">
-        <f>N($H24)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N24" s="398">
-        <f>$L24+$M24</f>
-        <v/>
-      </c>
-      <c r="O24" s="401">
-        <f>IF($I24="","nog te plannen",IFERROR(LOOKUP($I24,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J24" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G24)=0,0,IF($G24&lt;15,0.25,IF($G24&lt;=50,0.035,IF($G24&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K24" s="398">
+        <f>IF($I24=0,0,$G24*$I24*(1+$J24))</f>
+        <v/>
+      </c>
+      <c r="L24" s="401">
+        <f>IF($H24="","nog te plannen",IFERROR(LOOKUP($H24,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5897,34 +5650,23 @@
       <c r="G25" s="391" t="n">
         <v>121.4</v>
       </c>
-      <c r="H25" s="391" t="n">
-        <v>5.21</v>
-      </c>
-      <c r="I25" s="417" t="n">
+      <c r="H25" s="417" t="n">
         <v>45358</v>
       </c>
-      <c r="J25" s="392">
+      <c r="I25" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C25,'SAERTEX-prijstabel'!$B$2:$B$496,$D25,'SAERTEX-prijstabel'!$C$2:$C$496,$E25,'SAERTEX-prijstabel'!$D$2:$D$496,$F25),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K25" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G25)+N($H25))=0,0,IF((N($G25)+N($H25))&lt;15,0.25,IF((N($G25)+N($H25))&lt;=50,0.035,IF((N($G25)+N($H25))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L25" s="392">
-        <f>IF($J25=0,0,$G25*$J25*(1+$K25))</f>
-        <v/>
-      </c>
-      <c r="M25" s="392">
-        <f>N($H25)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N25" s="398">
-        <f>$L25+$M25</f>
-        <v/>
-      </c>
-      <c r="O25" s="401">
-        <f>IF($I25="","nog te plannen",IFERROR(LOOKUP($I25,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J25" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G25)=0,0,IF($G25&lt;15,0.25,IF($G25&lt;=50,0.035,IF($G25&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K25" s="398">
+        <f>IF($I25=0,0,$G25*$I25*(1+$J25))</f>
+        <v/>
+      </c>
+      <c r="L25" s="401">
+        <f>IF($H25="","nog te plannen",IFERROR(LOOKUP($H25,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -5958,34 +5700,23 @@
       <c r="G26" s="391" t="n">
         <v>93.8</v>
       </c>
-      <c r="H26" s="391" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="I26" s="417" t="n">
+      <c r="H26" s="417" t="n">
         <v>45361</v>
       </c>
-      <c r="J26" s="392">
+      <c r="I26" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C26,'SAERTEX-prijstabel'!$B$2:$B$496,$D26,'SAERTEX-prijstabel'!$C$2:$C$496,$E26,'SAERTEX-prijstabel'!$D$2:$D$496,$F26),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K26" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G26)+N($H26))=0,0,IF((N($G26)+N($H26))&lt;15,0.25,IF((N($G26)+N($H26))&lt;=50,0.035,IF((N($G26)+N($H26))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L26" s="392">
-        <f>IF($J26=0,0,$G26*$J26*(1+$K26))</f>
-        <v/>
-      </c>
-      <c r="M26" s="392">
-        <f>N($H26)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N26" s="398">
-        <f>$L26+$M26</f>
-        <v/>
-      </c>
-      <c r="O26" s="401">
-        <f>IF($I26="","nog te plannen",IFERROR(LOOKUP($I26,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J26" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G26)=0,0,IF($G26&lt;15,0.25,IF($G26&lt;=50,0.035,IF($G26&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K26" s="398">
+        <f>IF($I26=0,0,$G26*$I26*(1+$J26))</f>
+        <v/>
+      </c>
+      <c r="L26" s="401">
+        <f>IF($H26="","nog te plannen",IFERROR(LOOKUP($H26,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6019,34 +5750,23 @@
       <c r="G27" s="391" t="n">
         <v>60.9</v>
       </c>
-      <c r="H27" s="391" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="I27" s="417" t="n">
+      <c r="H27" s="417" t="n">
         <v>45364</v>
       </c>
-      <c r="J27" s="392">
+      <c r="I27" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C27,'SAERTEX-prijstabel'!$B$2:$B$496,$D27,'SAERTEX-prijstabel'!$C$2:$C$496,$E27,'SAERTEX-prijstabel'!$D$2:$D$496,$F27),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K27" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G27)+N($H27))=0,0,IF((N($G27)+N($H27))&lt;15,0.25,IF((N($G27)+N($H27))&lt;=50,0.035,IF((N($G27)+N($H27))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L27" s="392">
-        <f>IF($J27=0,0,$G27*$J27*(1+$K27))</f>
-        <v/>
-      </c>
-      <c r="M27" s="392">
-        <f>N($H27)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N27" s="398">
-        <f>$L27+$M27</f>
-        <v/>
-      </c>
-      <c r="O27" s="401">
-        <f>IF($I27="","nog te plannen",IFERROR(LOOKUP($I27,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J27" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G27)=0,0,IF($G27&lt;15,0.25,IF($G27&lt;=50,0.035,IF($G27&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K27" s="398">
+        <f>IF($I27=0,0,$G27*$I27*(1+$J27))</f>
+        <v/>
+      </c>
+      <c r="L27" s="401">
+        <f>IF($H27="","nog te plannen",IFERROR(LOOKUP($H27,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6080,34 +5800,23 @@
       <c r="G28" s="391" t="n">
         <v>49.2</v>
       </c>
-      <c r="H28" s="391" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I28" s="417" t="n">
+      <c r="H28" s="417" t="n">
         <v>45367</v>
       </c>
-      <c r="J28" s="392">
+      <c r="I28" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C28,'SAERTEX-prijstabel'!$B$2:$B$496,$D28,'SAERTEX-prijstabel'!$C$2:$C$496,$E28,'SAERTEX-prijstabel'!$D$2:$D$496,$F28),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K28" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G28)+N($H28))=0,0,IF((N($G28)+N($H28))&lt;15,0.25,IF((N($G28)+N($H28))&lt;=50,0.035,IF((N($G28)+N($H28))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L28" s="392">
-        <f>IF($J28=0,0,$G28*$J28*(1+$K28))</f>
-        <v/>
-      </c>
-      <c r="M28" s="392">
-        <f>N($H28)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N28" s="398">
-        <f>$L28+$M28</f>
-        <v/>
-      </c>
-      <c r="O28" s="401">
-        <f>IF($I28="","nog te plannen",IFERROR(LOOKUP($I28,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J28" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G28)=0,0,IF($G28&lt;15,0.25,IF($G28&lt;=50,0.035,IF($G28&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K28" s="398">
+        <f>IF($I28=0,0,$G28*$I28*(1+$J28))</f>
+        <v/>
+      </c>
+      <c r="L28" s="401">
+        <f>IF($H28="","nog te plannen",IFERROR(LOOKUP($H28,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6141,34 +5850,23 @@
       <c r="G29" s="391" t="n">
         <v>106.1</v>
       </c>
-      <c r="H29" s="391" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I29" s="417" t="n">
+      <c r="H29" s="417" t="n">
         <v>45370</v>
       </c>
-      <c r="J29" s="392">
+      <c r="I29" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C29,'SAERTEX-prijstabel'!$B$2:$B$496,$D29,'SAERTEX-prijstabel'!$C$2:$C$496,$E29,'SAERTEX-prijstabel'!$D$2:$D$496,$F29),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K29" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G29)+N($H29))=0,0,IF((N($G29)+N($H29))&lt;15,0.25,IF((N($G29)+N($H29))&lt;=50,0.035,IF((N($G29)+N($H29))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L29" s="392">
-        <f>IF($J29=0,0,$G29*$J29*(1+$K29))</f>
-        <v/>
-      </c>
-      <c r="M29" s="392">
-        <f>N($H29)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N29" s="398">
-        <f>$L29+$M29</f>
-        <v/>
-      </c>
-      <c r="O29" s="401">
-        <f>IF($I29="","nog te plannen",IFERROR(LOOKUP($I29,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J29" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G29)=0,0,IF($G29&lt;15,0.25,IF($G29&lt;=50,0.035,IF($G29&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K29" s="398">
+        <f>IF($I29=0,0,$G29*$I29*(1+$J29))</f>
+        <v/>
+      </c>
+      <c r="L29" s="401">
+        <f>IF($H29="","nog te plannen",IFERROR(LOOKUP($H29,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6180,30 +5878,21 @@
       <c r="E30" s="306" t="n"/>
       <c r="F30" s="306" t="n"/>
       <c r="G30" s="391" t="n"/>
-      <c r="H30" s="391" t="n"/>
-      <c r="I30" s="388" t="n"/>
-      <c r="J30" s="392">
+      <c r="H30" s="388" t="n"/>
+      <c r="I30" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C30,'SAERTEX-prijstabel'!$B$2:$B$496,$D30,'SAERTEX-prijstabel'!$C$2:$C$496,$E30,'SAERTEX-prijstabel'!$D$2:$D$496,$F30),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K30" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G30)+N($H30))=0,0,IF((N($G30)+N($H30))&lt;15,0.25,IF((N($G30)+N($H30))&lt;=50,0.035,IF((N($G30)+N($H30))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L30" s="392">
-        <f>IF($J30=0,0,$G30*$J30*(1+$K30))</f>
-        <v/>
-      </c>
-      <c r="M30" s="392">
-        <f>N($H30)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N30" s="398">
-        <f>$L30+$M30</f>
-        <v/>
-      </c>
-      <c r="O30" s="401">
-        <f>IF($I30="","nog te plannen",IFERROR(LOOKUP($I30,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J30" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G30)=0,0,IF($G30&lt;15,0.25,IF($G30&lt;=50,0.035,IF($G30&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K30" s="398">
+        <f>IF($I30=0,0,$G30*$I30*(1+$J30))</f>
+        <v/>
+      </c>
+      <c r="L30" s="401">
+        <f>IF($H30="","nog te plannen",IFERROR(LOOKUP($H30,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6215,30 +5904,21 @@
       <c r="E31" s="306" t="n"/>
       <c r="F31" s="306" t="n"/>
       <c r="G31" s="391" t="n"/>
-      <c r="H31" s="391" t="n"/>
-      <c r="I31" s="388" t="n"/>
-      <c r="J31" s="392">
+      <c r="H31" s="388" t="n"/>
+      <c r="I31" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C31,'SAERTEX-prijstabel'!$B$2:$B$496,$D31,'SAERTEX-prijstabel'!$C$2:$C$496,$E31,'SAERTEX-prijstabel'!$D$2:$D$496,$F31),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K31" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G31)+N($H31))=0,0,IF((N($G31)+N($H31))&lt;15,0.25,IF((N($G31)+N($H31))&lt;=50,0.035,IF((N($G31)+N($H31))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L31" s="392">
-        <f>IF($J31=0,0,$G31*$J31*(1+$K31))</f>
-        <v/>
-      </c>
-      <c r="M31" s="392">
-        <f>N($H31)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N31" s="398">
-        <f>$L31+$M31</f>
-        <v/>
-      </c>
-      <c r="O31" s="401">
-        <f>IF($I31="","nog te plannen",IFERROR(LOOKUP($I31,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J31" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G31)=0,0,IF($G31&lt;15,0.25,IF($G31&lt;=50,0.035,IF($G31&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K31" s="398">
+        <f>IF($I31=0,0,$G31*$I31*(1+$J31))</f>
+        <v/>
+      </c>
+      <c r="L31" s="401">
+        <f>IF($H31="","nog te plannen",IFERROR(LOOKUP($H31,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6250,30 +5930,21 @@
       <c r="E32" s="306" t="n"/>
       <c r="F32" s="306" t="n"/>
       <c r="G32" s="391" t="n"/>
-      <c r="H32" s="391" t="n"/>
-      <c r="I32" s="388" t="n"/>
-      <c r="J32" s="392">
+      <c r="H32" s="388" t="n"/>
+      <c r="I32" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C32,'SAERTEX-prijstabel'!$B$2:$B$496,$D32,'SAERTEX-prijstabel'!$C$2:$C$496,$E32,'SAERTEX-prijstabel'!$D$2:$D$496,$F32),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K32" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G32)+N($H32))=0,0,IF((N($G32)+N($H32))&lt;15,0.25,IF((N($G32)+N($H32))&lt;=50,0.035,IF((N($G32)+N($H32))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L32" s="392">
-        <f>IF($J32=0,0,$G32*$J32*(1+$K32))</f>
-        <v/>
-      </c>
-      <c r="M32" s="392">
-        <f>N($H32)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N32" s="398">
-        <f>$L32+$M32</f>
-        <v/>
-      </c>
-      <c r="O32" s="401">
-        <f>IF($I32="","nog te plannen",IFERROR(LOOKUP($I32,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J32" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G32)=0,0,IF($G32&lt;15,0.25,IF($G32&lt;=50,0.035,IF($G32&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K32" s="398">
+        <f>IF($I32=0,0,$G32*$I32*(1+$J32))</f>
+        <v/>
+      </c>
+      <c r="L32" s="401">
+        <f>IF($H32="","nog te plannen",IFERROR(LOOKUP($H32,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6285,30 +5956,21 @@
       <c r="E33" s="306" t="n"/>
       <c r="F33" s="306" t="n"/>
       <c r="G33" s="391" t="n"/>
-      <c r="H33" s="391" t="n"/>
-      <c r="I33" s="388" t="n"/>
-      <c r="J33" s="392">
+      <c r="H33" s="388" t="n"/>
+      <c r="I33" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C33,'SAERTEX-prijstabel'!$B$2:$B$496,$D33,'SAERTEX-prijstabel'!$C$2:$C$496,$E33,'SAERTEX-prijstabel'!$D$2:$D$496,$F33),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K33" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G33)+N($H33))=0,0,IF((N($G33)+N($H33))&lt;15,0.25,IF((N($G33)+N($H33))&lt;=50,0.035,IF((N($G33)+N($H33))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L33" s="392">
-        <f>IF($J33=0,0,$G33*$J33*(1+$K33))</f>
-        <v/>
-      </c>
-      <c r="M33" s="392">
-        <f>N($H33)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N33" s="398">
-        <f>$L33+$M33</f>
-        <v/>
-      </c>
-      <c r="O33" s="401">
-        <f>IF($I33="","nog te plannen",IFERROR(LOOKUP($I33,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J33" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G33)=0,0,IF($G33&lt;15,0.25,IF($G33&lt;=50,0.035,IF($G33&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K33" s="398">
+        <f>IF($I33=0,0,$G33*$I33*(1+$J33))</f>
+        <v/>
+      </c>
+      <c r="L33" s="401">
+        <f>IF($H33="","nog te plannen",IFERROR(LOOKUP($H33,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6320,30 +5982,21 @@
       <c r="E34" s="306" t="n"/>
       <c r="F34" s="306" t="n"/>
       <c r="G34" s="391" t="n"/>
-      <c r="H34" s="391" t="n"/>
-      <c r="I34" s="388" t="n"/>
-      <c r="J34" s="392">
+      <c r="H34" s="388" t="n"/>
+      <c r="I34" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C34,'SAERTEX-prijstabel'!$B$2:$B$496,$D34,'SAERTEX-prijstabel'!$C$2:$C$496,$E34,'SAERTEX-prijstabel'!$D$2:$D$496,$F34),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K34" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G34)+N($H34))=0,0,IF((N($G34)+N($H34))&lt;15,0.25,IF((N($G34)+N($H34))&lt;=50,0.035,IF((N($G34)+N($H34))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L34" s="392">
-        <f>IF($J34=0,0,$G34*$J34*(1+$K34))</f>
-        <v/>
-      </c>
-      <c r="M34" s="392">
-        <f>N($H34)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N34" s="398">
-        <f>$L34+$M34</f>
-        <v/>
-      </c>
-      <c r="O34" s="401">
-        <f>IF($I34="","nog te plannen",IFERROR(LOOKUP($I34,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J34" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G34)=0,0,IF($G34&lt;15,0.25,IF($G34&lt;=50,0.035,IF($G34&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K34" s="398">
+        <f>IF($I34=0,0,$G34*$I34*(1+$J34))</f>
+        <v/>
+      </c>
+      <c r="L34" s="401">
+        <f>IF($H34="","nog te plannen",IFERROR(LOOKUP($H34,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6355,30 +6008,21 @@
       <c r="E35" s="306" t="n"/>
       <c r="F35" s="306" t="n"/>
       <c r="G35" s="391" t="n"/>
-      <c r="H35" s="391" t="n"/>
-      <c r="I35" s="388" t="n"/>
-      <c r="J35" s="392">
+      <c r="H35" s="388" t="n"/>
+      <c r="I35" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C35,'SAERTEX-prijstabel'!$B$2:$B$496,$D35,'SAERTEX-prijstabel'!$C$2:$C$496,$E35,'SAERTEX-prijstabel'!$D$2:$D$496,$F35),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K35" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G35)+N($H35))=0,0,IF((N($G35)+N($H35))&lt;15,0.25,IF((N($G35)+N($H35))&lt;=50,0.035,IF((N($G35)+N($H35))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L35" s="392">
-        <f>IF($J35=0,0,$G35*$J35*(1+$K35))</f>
-        <v/>
-      </c>
-      <c r="M35" s="392">
-        <f>N($H35)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N35" s="398">
-        <f>$L35+$M35</f>
-        <v/>
-      </c>
-      <c r="O35" s="401">
-        <f>IF($I35="","nog te plannen",IFERROR(LOOKUP($I35,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J35" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G35)=0,0,IF($G35&lt;15,0.25,IF($G35&lt;=50,0.035,IF($G35&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K35" s="398">
+        <f>IF($I35=0,0,$G35*$I35*(1+$J35))</f>
+        <v/>
+      </c>
+      <c r="L35" s="401">
+        <f>IF($H35="","nog te plannen",IFERROR(LOOKUP($H35,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6390,30 +6034,21 @@
       <c r="E36" s="306" t="n"/>
       <c r="F36" s="306" t="n"/>
       <c r="G36" s="391" t="n"/>
-      <c r="H36" s="391" t="n"/>
-      <c r="I36" s="388" t="n"/>
-      <c r="J36" s="392">
+      <c r="H36" s="388" t="n"/>
+      <c r="I36" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C36,'SAERTEX-prijstabel'!$B$2:$B$496,$D36,'SAERTEX-prijstabel'!$C$2:$C$496,$E36,'SAERTEX-prijstabel'!$D$2:$D$496,$F36),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K36" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G36)+N($H36))=0,0,IF((N($G36)+N($H36))&lt;15,0.25,IF((N($G36)+N($H36))&lt;=50,0.035,IF((N($G36)+N($H36))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L36" s="392">
-        <f>IF($J36=0,0,$G36*$J36*(1+$K36))</f>
-        <v/>
-      </c>
-      <c r="M36" s="392">
-        <f>N($H36)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N36" s="398">
-        <f>$L36+$M36</f>
-        <v/>
-      </c>
-      <c r="O36" s="401">
-        <f>IF($I36="","nog te plannen",IFERROR(LOOKUP($I36,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J36" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G36)=0,0,IF($G36&lt;15,0.25,IF($G36&lt;=50,0.035,IF($G36&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K36" s="398">
+        <f>IF($I36=0,0,$G36*$I36*(1+$J36))</f>
+        <v/>
+      </c>
+      <c r="L36" s="401">
+        <f>IF($H36="","nog te plannen",IFERROR(LOOKUP($H36,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6425,30 +6060,21 @@
       <c r="E37" s="306" t="n"/>
       <c r="F37" s="306" t="n"/>
       <c r="G37" s="391" t="n"/>
-      <c r="H37" s="391" t="n"/>
-      <c r="I37" s="388" t="n"/>
-      <c r="J37" s="392">
+      <c r="H37" s="388" t="n"/>
+      <c r="I37" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C37,'SAERTEX-prijstabel'!$B$2:$B$496,$D37,'SAERTEX-prijstabel'!$C$2:$C$496,$E37,'SAERTEX-prijstabel'!$D$2:$D$496,$F37),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K37" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G37)+N($H37))=0,0,IF((N($G37)+N($H37))&lt;15,0.25,IF((N($G37)+N($H37))&lt;=50,0.035,IF((N($G37)+N($H37))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L37" s="392">
-        <f>IF($J37=0,0,$G37*$J37*(1+$K37))</f>
-        <v/>
-      </c>
-      <c r="M37" s="392">
-        <f>N($H37)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N37" s="398">
-        <f>$L37+$M37</f>
-        <v/>
-      </c>
-      <c r="O37" s="401">
-        <f>IF($I37="","nog te plannen",IFERROR(LOOKUP($I37,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J37" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G37)=0,0,IF($G37&lt;15,0.25,IF($G37&lt;=50,0.035,IF($G37&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K37" s="398">
+        <f>IF($I37=0,0,$G37*$I37*(1+$J37))</f>
+        <v/>
+      </c>
+      <c r="L37" s="401">
+        <f>IF($H37="","nog te plannen",IFERROR(LOOKUP($H37,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6460,30 +6086,21 @@
       <c r="E38" s="306" t="n"/>
       <c r="F38" s="306" t="n"/>
       <c r="G38" s="391" t="n"/>
-      <c r="H38" s="391" t="n"/>
-      <c r="I38" s="388" t="n"/>
-      <c r="J38" s="392">
+      <c r="H38" s="388" t="n"/>
+      <c r="I38" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C38,'SAERTEX-prijstabel'!$B$2:$B$496,$D38,'SAERTEX-prijstabel'!$C$2:$C$496,$E38,'SAERTEX-prijstabel'!$D$2:$D$496,$F38),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K38" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G38)+N($H38))=0,0,IF((N($G38)+N($H38))&lt;15,0.25,IF((N($G38)+N($H38))&lt;=50,0.035,IF((N($G38)+N($H38))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L38" s="392">
-        <f>IF($J38=0,0,$G38*$J38*(1+$K38))</f>
-        <v/>
-      </c>
-      <c r="M38" s="392">
-        <f>N($H38)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N38" s="398">
-        <f>$L38+$M38</f>
-        <v/>
-      </c>
-      <c r="O38" s="401">
-        <f>IF($I38="","nog te plannen",IFERROR(LOOKUP($I38,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J38" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G38)=0,0,IF($G38&lt;15,0.25,IF($G38&lt;=50,0.035,IF($G38&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K38" s="398">
+        <f>IF($I38=0,0,$G38*$I38*(1+$J38))</f>
+        <v/>
+      </c>
+      <c r="L38" s="401">
+        <f>IF($H38="","nog te plannen",IFERROR(LOOKUP($H38,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6495,30 +6112,21 @@
       <c r="E39" s="306" t="n"/>
       <c r="F39" s="306" t="n"/>
       <c r="G39" s="391" t="n"/>
-      <c r="H39" s="391" t="n"/>
-      <c r="I39" s="388" t="n"/>
-      <c r="J39" s="392">
+      <c r="H39" s="388" t="n"/>
+      <c r="I39" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C39,'SAERTEX-prijstabel'!$B$2:$B$496,$D39,'SAERTEX-prijstabel'!$C$2:$C$496,$E39,'SAERTEX-prijstabel'!$D$2:$D$496,$F39),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K39" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G39)+N($H39))=0,0,IF((N($G39)+N($H39))&lt;15,0.25,IF((N($G39)+N($H39))&lt;=50,0.035,IF((N($G39)+N($H39))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L39" s="392">
-        <f>IF($J39=0,0,$G39*$J39*(1+$K39))</f>
-        <v/>
-      </c>
-      <c r="M39" s="392">
-        <f>N($H39)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N39" s="398">
-        <f>$L39+$M39</f>
-        <v/>
-      </c>
-      <c r="O39" s="401">
-        <f>IF($I39="","nog te plannen",IFERROR(LOOKUP($I39,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J39" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G39)=0,0,IF($G39&lt;15,0.25,IF($G39&lt;=50,0.035,IF($G39&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K39" s="398">
+        <f>IF($I39=0,0,$G39*$I39*(1+$J39))</f>
+        <v/>
+      </c>
+      <c r="L39" s="401">
+        <f>IF($H39="","nog te plannen",IFERROR(LOOKUP($H39,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6530,30 +6138,21 @@
       <c r="E40" s="306" t="n"/>
       <c r="F40" s="306" t="n"/>
       <c r="G40" s="391" t="n"/>
-      <c r="H40" s="391" t="n"/>
-      <c r="I40" s="388" t="n"/>
-      <c r="J40" s="392">
+      <c r="H40" s="388" t="n"/>
+      <c r="I40" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C40,'SAERTEX-prijstabel'!$B$2:$B$496,$D40,'SAERTEX-prijstabel'!$C$2:$C$496,$E40,'SAERTEX-prijstabel'!$D$2:$D$496,$F40),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K40" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G40)+N($H40))=0,0,IF((N($G40)+N($H40))&lt;15,0.25,IF((N($G40)+N($H40))&lt;=50,0.035,IF((N($G40)+N($H40))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L40" s="392">
-        <f>IF($J40=0,0,$G40*$J40*(1+$K40))</f>
-        <v/>
-      </c>
-      <c r="M40" s="392">
-        <f>N($H40)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N40" s="398">
-        <f>$L40+$M40</f>
-        <v/>
-      </c>
-      <c r="O40" s="401">
-        <f>IF($I40="","nog te plannen",IFERROR(LOOKUP($I40,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J40" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G40)=0,0,IF($G40&lt;15,0.25,IF($G40&lt;=50,0.035,IF($G40&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K40" s="398">
+        <f>IF($I40=0,0,$G40*$I40*(1+$J40))</f>
+        <v/>
+      </c>
+      <c r="L40" s="401">
+        <f>IF($H40="","nog te plannen",IFERROR(LOOKUP($H40,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6565,30 +6164,21 @@
       <c r="E41" s="306" t="n"/>
       <c r="F41" s="306" t="n"/>
       <c r="G41" s="391" t="n"/>
-      <c r="H41" s="391" t="n"/>
-      <c r="I41" s="388" t="n"/>
-      <c r="J41" s="392">
+      <c r="H41" s="388" t="n"/>
+      <c r="I41" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C41,'SAERTEX-prijstabel'!$B$2:$B$496,$D41,'SAERTEX-prijstabel'!$C$2:$C$496,$E41,'SAERTEX-prijstabel'!$D$2:$D$496,$F41),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K41" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G41)+N($H41))=0,0,IF((N($G41)+N($H41))&lt;15,0.25,IF((N($G41)+N($H41))&lt;=50,0.035,IF((N($G41)+N($H41))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L41" s="392">
-        <f>IF($J41=0,0,$G41*$J41*(1+$K41))</f>
-        <v/>
-      </c>
-      <c r="M41" s="392">
-        <f>N($H41)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N41" s="398">
-        <f>$L41+$M41</f>
-        <v/>
-      </c>
-      <c r="O41" s="401">
-        <f>IF($I41="","nog te plannen",IFERROR(LOOKUP($I41,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J41" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G41)=0,0,IF($G41&lt;15,0.25,IF($G41&lt;=50,0.035,IF($G41&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K41" s="398">
+        <f>IF($I41=0,0,$G41*$I41*(1+$J41))</f>
+        <v/>
+      </c>
+      <c r="L41" s="401">
+        <f>IF($H41="","nog te plannen",IFERROR(LOOKUP($H41,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6600,30 +6190,21 @@
       <c r="E42" s="306" t="n"/>
       <c r="F42" s="306" t="n"/>
       <c r="G42" s="391" t="n"/>
-      <c r="H42" s="391" t="n"/>
-      <c r="I42" s="388" t="n"/>
-      <c r="J42" s="392">
+      <c r="H42" s="388" t="n"/>
+      <c r="I42" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C42,'SAERTEX-prijstabel'!$B$2:$B$496,$D42,'SAERTEX-prijstabel'!$C$2:$C$496,$E42,'SAERTEX-prijstabel'!$D$2:$D$496,$F42),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K42" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G42)+N($H42))=0,0,IF((N($G42)+N($H42))&lt;15,0.25,IF((N($G42)+N($H42))&lt;=50,0.035,IF((N($G42)+N($H42))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L42" s="392">
-        <f>IF($J42=0,0,$G42*$J42*(1+$K42))</f>
-        <v/>
-      </c>
-      <c r="M42" s="392">
-        <f>N($H42)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N42" s="398">
-        <f>$L42+$M42</f>
-        <v/>
-      </c>
-      <c r="O42" s="401">
-        <f>IF($I42="","nog te plannen",IFERROR(LOOKUP($I42,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J42" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G42)=0,0,IF($G42&lt;15,0.25,IF($G42&lt;=50,0.035,IF($G42&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K42" s="398">
+        <f>IF($I42=0,0,$G42*$I42*(1+$J42))</f>
+        <v/>
+      </c>
+      <c r="L42" s="401">
+        <f>IF($H42="","nog te plannen",IFERROR(LOOKUP($H42,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6635,30 +6216,21 @@
       <c r="E43" s="306" t="n"/>
       <c r="F43" s="306" t="n"/>
       <c r="G43" s="391" t="n"/>
-      <c r="H43" s="391" t="n"/>
-      <c r="I43" s="388" t="n"/>
-      <c r="J43" s="392">
+      <c r="H43" s="388" t="n"/>
+      <c r="I43" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C43,'SAERTEX-prijstabel'!$B$2:$B$496,$D43,'SAERTEX-prijstabel'!$C$2:$C$496,$E43,'SAERTEX-prijstabel'!$D$2:$D$496,$F43),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K43" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G43)+N($H43))=0,0,IF((N($G43)+N($H43))&lt;15,0.25,IF((N($G43)+N($H43))&lt;=50,0.035,IF((N($G43)+N($H43))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L43" s="392">
-        <f>IF($J43=0,0,$G43*$J43*(1+$K43))</f>
-        <v/>
-      </c>
-      <c r="M43" s="392">
-        <f>N($H43)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N43" s="398">
-        <f>$L43+$M43</f>
-        <v/>
-      </c>
-      <c r="O43" s="401">
-        <f>IF($I43="","nog te plannen",IFERROR(LOOKUP($I43,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J43" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G43)=0,0,IF($G43&lt;15,0.25,IF($G43&lt;=50,0.035,IF($G43&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K43" s="398">
+        <f>IF($I43=0,0,$G43*$I43*(1+$J43))</f>
+        <v/>
+      </c>
+      <c r="L43" s="401">
+        <f>IF($H43="","nog te plannen",IFERROR(LOOKUP($H43,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6670,30 +6242,21 @@
       <c r="E44" s="306" t="n"/>
       <c r="F44" s="306" t="n"/>
       <c r="G44" s="391" t="n"/>
-      <c r="H44" s="391" t="n"/>
-      <c r="I44" s="388" t="n"/>
-      <c r="J44" s="392">
+      <c r="H44" s="388" t="n"/>
+      <c r="I44" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C44,'SAERTEX-prijstabel'!$B$2:$B$496,$D44,'SAERTEX-prijstabel'!$C$2:$C$496,$E44,'SAERTEX-prijstabel'!$D$2:$D$496,$F44),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K44" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G44)+N($H44))=0,0,IF((N($G44)+N($H44))&lt;15,0.25,IF((N($G44)+N($H44))&lt;=50,0.035,IF((N($G44)+N($H44))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L44" s="392">
-        <f>IF($J44=0,0,$G44*$J44*(1+$K44))</f>
-        <v/>
-      </c>
-      <c r="M44" s="392">
-        <f>N($H44)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N44" s="398">
-        <f>$L44+$M44</f>
-        <v/>
-      </c>
-      <c r="O44" s="401">
-        <f>IF($I44="","nog te plannen",IFERROR(LOOKUP($I44,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J44" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G44)=0,0,IF($G44&lt;15,0.25,IF($G44&lt;=50,0.035,IF($G44&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K44" s="398">
+        <f>IF($I44=0,0,$G44*$I44*(1+$J44))</f>
+        <v/>
+      </c>
+      <c r="L44" s="401">
+        <f>IF($H44="","nog te plannen",IFERROR(LOOKUP($H44,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6705,30 +6268,21 @@
       <c r="E45" s="306" t="n"/>
       <c r="F45" s="306" t="n"/>
       <c r="G45" s="391" t="n"/>
-      <c r="H45" s="391" t="n"/>
-      <c r="I45" s="388" t="n"/>
-      <c r="J45" s="392">
+      <c r="H45" s="388" t="n"/>
+      <c r="I45" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C45,'SAERTEX-prijstabel'!$B$2:$B$496,$D45,'SAERTEX-prijstabel'!$C$2:$C$496,$E45,'SAERTEX-prijstabel'!$D$2:$D$496,$F45),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K45" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G45)+N($H45))=0,0,IF((N($G45)+N($H45))&lt;15,0.25,IF((N($G45)+N($H45))&lt;=50,0.035,IF((N($G45)+N($H45))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L45" s="392">
-        <f>IF($J45=0,0,$G45*$J45*(1+$K45))</f>
-        <v/>
-      </c>
-      <c r="M45" s="392">
-        <f>N($H45)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N45" s="398">
-        <f>$L45+$M45</f>
-        <v/>
-      </c>
-      <c r="O45" s="401">
-        <f>IF($I45="","nog te plannen",IFERROR(LOOKUP($I45,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J45" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G45)=0,0,IF($G45&lt;15,0.25,IF($G45&lt;=50,0.035,IF($G45&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K45" s="398">
+        <f>IF($I45=0,0,$G45*$I45*(1+$J45))</f>
+        <v/>
+      </c>
+      <c r="L45" s="401">
+        <f>IF($H45="","nog te plannen",IFERROR(LOOKUP($H45,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6740,30 +6294,21 @@
       <c r="E46" s="306" t="n"/>
       <c r="F46" s="306" t="n"/>
       <c r="G46" s="391" t="n"/>
-      <c r="H46" s="391" t="n"/>
-      <c r="I46" s="388" t="n"/>
-      <c r="J46" s="392">
+      <c r="H46" s="388" t="n"/>
+      <c r="I46" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C46,'SAERTEX-prijstabel'!$B$2:$B$496,$D46,'SAERTEX-prijstabel'!$C$2:$C$496,$E46,'SAERTEX-prijstabel'!$D$2:$D$496,$F46),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K46" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G46)+N($H46))=0,0,IF((N($G46)+N($H46))&lt;15,0.25,IF((N($G46)+N($H46))&lt;=50,0.035,IF((N($G46)+N($H46))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L46" s="392">
-        <f>IF($J46=0,0,$G46*$J46*(1+$K46))</f>
-        <v/>
-      </c>
-      <c r="M46" s="392">
-        <f>N($H46)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N46" s="398">
-        <f>$L46+$M46</f>
-        <v/>
-      </c>
-      <c r="O46" s="401">
-        <f>IF($I46="","nog te plannen",IFERROR(LOOKUP($I46,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J46" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G46)=0,0,IF($G46&lt;15,0.25,IF($G46&lt;=50,0.035,IF($G46&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K46" s="398">
+        <f>IF($I46=0,0,$G46*$I46*(1+$J46))</f>
+        <v/>
+      </c>
+      <c r="L46" s="401">
+        <f>IF($H46="","nog te plannen",IFERROR(LOOKUP($H46,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6775,30 +6320,21 @@
       <c r="E47" s="306" t="n"/>
       <c r="F47" s="306" t="n"/>
       <c r="G47" s="391" t="n"/>
-      <c r="H47" s="391" t="n"/>
-      <c r="I47" s="388" t="n"/>
-      <c r="J47" s="392">
+      <c r="H47" s="388" t="n"/>
+      <c r="I47" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C47,'SAERTEX-prijstabel'!$B$2:$B$496,$D47,'SAERTEX-prijstabel'!$C$2:$C$496,$E47,'SAERTEX-prijstabel'!$D$2:$D$496,$F47),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K47" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G47)+N($H47))=0,0,IF((N($G47)+N($H47))&lt;15,0.25,IF((N($G47)+N($H47))&lt;=50,0.035,IF((N($G47)+N($H47))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L47" s="392">
-        <f>IF($J47=0,0,$G47*$J47*(1+$K47))</f>
-        <v/>
-      </c>
-      <c r="M47" s="392">
-        <f>N($H47)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N47" s="398">
-        <f>$L47+$M47</f>
-        <v/>
-      </c>
-      <c r="O47" s="401">
-        <f>IF($I47="","nog te plannen",IFERROR(LOOKUP($I47,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J47" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G47)=0,0,IF($G47&lt;15,0.25,IF($G47&lt;=50,0.035,IF($G47&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K47" s="398">
+        <f>IF($I47=0,0,$G47*$I47*(1+$J47))</f>
+        <v/>
+      </c>
+      <c r="L47" s="401">
+        <f>IF($H47="","nog te plannen",IFERROR(LOOKUP($H47,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6810,30 +6346,21 @@
       <c r="E48" s="306" t="n"/>
       <c r="F48" s="306" t="n"/>
       <c r="G48" s="391" t="n"/>
-      <c r="H48" s="391" t="n"/>
-      <c r="I48" s="388" t="n"/>
-      <c r="J48" s="392">
+      <c r="H48" s="388" t="n"/>
+      <c r="I48" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C48,'SAERTEX-prijstabel'!$B$2:$B$496,$D48,'SAERTEX-prijstabel'!$C$2:$C$496,$E48,'SAERTEX-prijstabel'!$D$2:$D$496,$F48),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K48" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G48)+N($H48))=0,0,IF((N($G48)+N($H48))&lt;15,0.25,IF((N($G48)+N($H48))&lt;=50,0.035,IF((N($G48)+N($H48))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L48" s="392">
-        <f>IF($J48=0,0,$G48*$J48*(1+$K48))</f>
-        <v/>
-      </c>
-      <c r="M48" s="392">
-        <f>N($H48)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N48" s="398">
-        <f>$L48+$M48</f>
-        <v/>
-      </c>
-      <c r="O48" s="401">
-        <f>IF($I48="","nog te plannen",IFERROR(LOOKUP($I48,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J48" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G48)=0,0,IF($G48&lt;15,0.25,IF($G48&lt;=50,0.035,IF($G48&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K48" s="398">
+        <f>IF($I48=0,0,$G48*$I48*(1+$J48))</f>
+        <v/>
+      </c>
+      <c r="L48" s="401">
+        <f>IF($H48="","nog te plannen",IFERROR(LOOKUP($H48,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6845,30 +6372,21 @@
       <c r="E49" s="306" t="n"/>
       <c r="F49" s="306" t="n"/>
       <c r="G49" s="391" t="n"/>
-      <c r="H49" s="391" t="n"/>
-      <c r="I49" s="388" t="n"/>
-      <c r="J49" s="392">
+      <c r="H49" s="388" t="n"/>
+      <c r="I49" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C49,'SAERTEX-prijstabel'!$B$2:$B$496,$D49,'SAERTEX-prijstabel'!$C$2:$C$496,$E49,'SAERTEX-prijstabel'!$D$2:$D$496,$F49),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K49" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G49)+N($H49))=0,0,IF((N($G49)+N($H49))&lt;15,0.25,IF((N($G49)+N($H49))&lt;=50,0.035,IF((N($G49)+N($H49))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L49" s="392">
-        <f>IF($J49=0,0,$G49*$J49*(1+$K49))</f>
-        <v/>
-      </c>
-      <c r="M49" s="392">
-        <f>N($H49)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N49" s="398">
-        <f>$L49+$M49</f>
-        <v/>
-      </c>
-      <c r="O49" s="401">
-        <f>IF($I49="","nog te plannen",IFERROR(LOOKUP($I49,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J49" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G49)=0,0,IF($G49&lt;15,0.25,IF($G49&lt;=50,0.035,IF($G49&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K49" s="398">
+        <f>IF($I49=0,0,$G49*$I49*(1+$J49))</f>
+        <v/>
+      </c>
+      <c r="L49" s="401">
+        <f>IF($H49="","nog te plannen",IFERROR(LOOKUP($H49,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6880,30 +6398,21 @@
       <c r="E50" s="306" t="n"/>
       <c r="F50" s="306" t="n"/>
       <c r="G50" s="391" t="n"/>
-      <c r="H50" s="391" t="n"/>
-      <c r="I50" s="388" t="n"/>
-      <c r="J50" s="392">
+      <c r="H50" s="388" t="n"/>
+      <c r="I50" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C50,'SAERTEX-prijstabel'!$B$2:$B$496,$D50,'SAERTEX-prijstabel'!$C$2:$C$496,$E50,'SAERTEX-prijstabel'!$D$2:$D$496,$F50),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K50" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G50)+N($H50))=0,0,IF((N($G50)+N($H50))&lt;15,0.25,IF((N($G50)+N($H50))&lt;=50,0.035,IF((N($G50)+N($H50))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L50" s="392">
-        <f>IF($J50=0,0,$G50*$J50*(1+$K50))</f>
-        <v/>
-      </c>
-      <c r="M50" s="392">
-        <f>N($H50)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N50" s="398">
-        <f>$L50+$M50</f>
-        <v/>
-      </c>
-      <c r="O50" s="401">
-        <f>IF($I50="","nog te plannen",IFERROR(LOOKUP($I50,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J50" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G50)=0,0,IF($G50&lt;15,0.25,IF($G50&lt;=50,0.035,IF($G50&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K50" s="398">
+        <f>IF($I50=0,0,$G50*$I50*(1+$J50))</f>
+        <v/>
+      </c>
+      <c r="L50" s="401">
+        <f>IF($H50="","nog te plannen",IFERROR(LOOKUP($H50,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6915,30 +6424,21 @@
       <c r="E51" s="306" t="n"/>
       <c r="F51" s="306" t="n"/>
       <c r="G51" s="391" t="n"/>
-      <c r="H51" s="391" t="n"/>
-      <c r="I51" s="388" t="n"/>
-      <c r="J51" s="392">
+      <c r="H51" s="388" t="n"/>
+      <c r="I51" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C51,'SAERTEX-prijstabel'!$B$2:$B$496,$D51,'SAERTEX-prijstabel'!$C$2:$C$496,$E51,'SAERTEX-prijstabel'!$D$2:$D$496,$F51),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K51" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G51)+N($H51))=0,0,IF((N($G51)+N($H51))&lt;15,0.25,IF((N($G51)+N($H51))&lt;=50,0.035,IF((N($G51)+N($H51))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L51" s="392">
-        <f>IF($J51=0,0,$G51*$J51*(1+$K51))</f>
-        <v/>
-      </c>
-      <c r="M51" s="392">
-        <f>N($H51)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N51" s="398">
-        <f>$L51+$M51</f>
-        <v/>
-      </c>
-      <c r="O51" s="401">
-        <f>IF($I51="","nog te plannen",IFERROR(LOOKUP($I51,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J51" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G51)=0,0,IF($G51&lt;15,0.25,IF($G51&lt;=50,0.035,IF($G51&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K51" s="398">
+        <f>IF($I51=0,0,$G51*$I51*(1+$J51))</f>
+        <v/>
+      </c>
+      <c r="L51" s="401">
+        <f>IF($H51="","nog te plannen",IFERROR(LOOKUP($H51,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6950,30 +6450,21 @@
       <c r="E52" s="306" t="n"/>
       <c r="F52" s="306" t="n"/>
       <c r="G52" s="391" t="n"/>
-      <c r="H52" s="391" t="n"/>
-      <c r="I52" s="388" t="n"/>
-      <c r="J52" s="392">
+      <c r="H52" s="388" t="n"/>
+      <c r="I52" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C52,'SAERTEX-prijstabel'!$B$2:$B$496,$D52,'SAERTEX-prijstabel'!$C$2:$C$496,$E52,'SAERTEX-prijstabel'!$D$2:$D$496,$F52),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K52" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G52)+N($H52))=0,0,IF((N($G52)+N($H52))&lt;15,0.25,IF((N($G52)+N($H52))&lt;=50,0.035,IF((N($G52)+N($H52))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L52" s="392">
-        <f>IF($J52=0,0,$G52*$J52*(1+$K52))</f>
-        <v/>
-      </c>
-      <c r="M52" s="392">
-        <f>N($H52)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N52" s="398">
-        <f>$L52+$M52</f>
-        <v/>
-      </c>
-      <c r="O52" s="401">
-        <f>IF($I52="","nog te plannen",IFERROR(LOOKUP($I52,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J52" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G52)=0,0,IF($G52&lt;15,0.25,IF($G52&lt;=50,0.035,IF($G52&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K52" s="398">
+        <f>IF($I52=0,0,$G52*$I52*(1+$J52))</f>
+        <v/>
+      </c>
+      <c r="L52" s="401">
+        <f>IF($H52="","nog te plannen",IFERROR(LOOKUP($H52,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -6985,30 +6476,21 @@
       <c r="E53" s="306" t="n"/>
       <c r="F53" s="306" t="n"/>
       <c r="G53" s="391" t="n"/>
-      <c r="H53" s="391" t="n"/>
-      <c r="I53" s="388" t="n"/>
-      <c r="J53" s="392">
+      <c r="H53" s="388" t="n"/>
+      <c r="I53" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C53,'SAERTEX-prijstabel'!$B$2:$B$496,$D53,'SAERTEX-prijstabel'!$C$2:$C$496,$E53,'SAERTEX-prijstabel'!$D$2:$D$496,$F53),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K53" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G53)+N($H53))=0,0,IF((N($G53)+N($H53))&lt;15,0.25,IF((N($G53)+N($H53))&lt;=50,0.035,IF((N($G53)+N($H53))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L53" s="392">
-        <f>IF($J53=0,0,$G53*$J53*(1+$K53))</f>
-        <v/>
-      </c>
-      <c r="M53" s="392">
-        <f>N($H53)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N53" s="398">
-        <f>$L53+$M53</f>
-        <v/>
-      </c>
-      <c r="O53" s="401">
-        <f>IF($I53="","nog te plannen",IFERROR(LOOKUP($I53,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J53" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G53)=0,0,IF($G53&lt;15,0.25,IF($G53&lt;=50,0.035,IF($G53&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K53" s="398">
+        <f>IF($I53=0,0,$G53*$I53*(1+$J53))</f>
+        <v/>
+      </c>
+      <c r="L53" s="401">
+        <f>IF($H53="","nog te plannen",IFERROR(LOOKUP($H53,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7020,30 +6502,21 @@
       <c r="E54" s="306" t="n"/>
       <c r="F54" s="306" t="n"/>
       <c r="G54" s="391" t="n"/>
-      <c r="H54" s="391" t="n"/>
-      <c r="I54" s="388" t="n"/>
-      <c r="J54" s="392">
+      <c r="H54" s="388" t="n"/>
+      <c r="I54" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C54,'SAERTEX-prijstabel'!$B$2:$B$496,$D54,'SAERTEX-prijstabel'!$C$2:$C$496,$E54,'SAERTEX-prijstabel'!$D$2:$D$496,$F54),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K54" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G54)+N($H54))=0,0,IF((N($G54)+N($H54))&lt;15,0.25,IF((N($G54)+N($H54))&lt;=50,0.035,IF((N($G54)+N($H54))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L54" s="392">
-        <f>IF($J54=0,0,$G54*$J54*(1+$K54))</f>
-        <v/>
-      </c>
-      <c r="M54" s="392">
-        <f>N($H54)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N54" s="398">
-        <f>$L54+$M54</f>
-        <v/>
-      </c>
-      <c r="O54" s="401">
-        <f>IF($I54="","nog te plannen",IFERROR(LOOKUP($I54,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J54" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G54)=0,0,IF($G54&lt;15,0.25,IF($G54&lt;=50,0.035,IF($G54&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K54" s="398">
+        <f>IF($I54=0,0,$G54*$I54*(1+$J54))</f>
+        <v/>
+      </c>
+      <c r="L54" s="401">
+        <f>IF($H54="","nog te plannen",IFERROR(LOOKUP($H54,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7055,30 +6528,21 @@
       <c r="E55" s="306" t="n"/>
       <c r="F55" s="306" t="n"/>
       <c r="G55" s="391" t="n"/>
-      <c r="H55" s="391" t="n"/>
-      <c r="I55" s="388" t="n"/>
-      <c r="J55" s="392">
+      <c r="H55" s="388" t="n"/>
+      <c r="I55" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C55,'SAERTEX-prijstabel'!$B$2:$B$496,$D55,'SAERTEX-prijstabel'!$C$2:$C$496,$E55,'SAERTEX-prijstabel'!$D$2:$D$496,$F55),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K55" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G55)+N($H55))=0,0,IF((N($G55)+N($H55))&lt;15,0.25,IF((N($G55)+N($H55))&lt;=50,0.035,IF((N($G55)+N($H55))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L55" s="392">
-        <f>IF($J55=0,0,$G55*$J55*(1+$K55))</f>
-        <v/>
-      </c>
-      <c r="M55" s="392">
-        <f>N($H55)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N55" s="398">
-        <f>$L55+$M55</f>
-        <v/>
-      </c>
-      <c r="O55" s="401">
-        <f>IF($I55="","nog te plannen",IFERROR(LOOKUP($I55,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J55" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G55)=0,0,IF($G55&lt;15,0.25,IF($G55&lt;=50,0.035,IF($G55&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K55" s="398">
+        <f>IF($I55=0,0,$G55*$I55*(1+$J55))</f>
+        <v/>
+      </c>
+      <c r="L55" s="401">
+        <f>IF($H55="","nog te plannen",IFERROR(LOOKUP($H55,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7090,30 +6554,21 @@
       <c r="E56" s="306" t="n"/>
       <c r="F56" s="306" t="n"/>
       <c r="G56" s="391" t="n"/>
-      <c r="H56" s="391" t="n"/>
-      <c r="I56" s="388" t="n"/>
-      <c r="J56" s="392">
+      <c r="H56" s="388" t="n"/>
+      <c r="I56" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C56,'SAERTEX-prijstabel'!$B$2:$B$496,$D56,'SAERTEX-prijstabel'!$C$2:$C$496,$E56,'SAERTEX-prijstabel'!$D$2:$D$496,$F56),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K56" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G56)+N($H56))=0,0,IF((N($G56)+N($H56))&lt;15,0.25,IF((N($G56)+N($H56))&lt;=50,0.035,IF((N($G56)+N($H56))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L56" s="392">
-        <f>IF($J56=0,0,$G56*$J56*(1+$K56))</f>
-        <v/>
-      </c>
-      <c r="M56" s="392">
-        <f>N($H56)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N56" s="398">
-        <f>$L56+$M56</f>
-        <v/>
-      </c>
-      <c r="O56" s="401">
-        <f>IF($I56="","nog te plannen",IFERROR(LOOKUP($I56,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J56" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G56)=0,0,IF($G56&lt;15,0.25,IF($G56&lt;=50,0.035,IF($G56&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K56" s="398">
+        <f>IF($I56=0,0,$G56*$I56*(1+$J56))</f>
+        <v/>
+      </c>
+      <c r="L56" s="401">
+        <f>IF($H56="","nog te plannen",IFERROR(LOOKUP($H56,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7125,30 +6580,21 @@
       <c r="E57" s="306" t="n"/>
       <c r="F57" s="306" t="n"/>
       <c r="G57" s="391" t="n"/>
-      <c r="H57" s="391" t="n"/>
-      <c r="I57" s="388" t="n"/>
-      <c r="J57" s="392">
+      <c r="H57" s="388" t="n"/>
+      <c r="I57" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C57,'SAERTEX-prijstabel'!$B$2:$B$496,$D57,'SAERTEX-prijstabel'!$C$2:$C$496,$E57,'SAERTEX-prijstabel'!$D$2:$D$496,$F57),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K57" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G57)+N($H57))=0,0,IF((N($G57)+N($H57))&lt;15,0.25,IF((N($G57)+N($H57))&lt;=50,0.035,IF((N($G57)+N($H57))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L57" s="392">
-        <f>IF($J57=0,0,$G57*$J57*(1+$K57))</f>
-        <v/>
-      </c>
-      <c r="M57" s="392">
-        <f>N($H57)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N57" s="398">
-        <f>$L57+$M57</f>
-        <v/>
-      </c>
-      <c r="O57" s="401">
-        <f>IF($I57="","nog te plannen",IFERROR(LOOKUP($I57,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J57" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G57)=0,0,IF($G57&lt;15,0.25,IF($G57&lt;=50,0.035,IF($G57&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K57" s="398">
+        <f>IF($I57=0,0,$G57*$I57*(1+$J57))</f>
+        <v/>
+      </c>
+      <c r="L57" s="401">
+        <f>IF($H57="","nog te plannen",IFERROR(LOOKUP($H57,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7160,30 +6606,21 @@
       <c r="E58" s="306" t="n"/>
       <c r="F58" s="306" t="n"/>
       <c r="G58" s="391" t="n"/>
-      <c r="H58" s="391" t="n"/>
-      <c r="I58" s="388" t="n"/>
-      <c r="J58" s="392">
+      <c r="H58" s="388" t="n"/>
+      <c r="I58" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C58,'SAERTEX-prijstabel'!$B$2:$B$496,$D58,'SAERTEX-prijstabel'!$C$2:$C$496,$E58,'SAERTEX-prijstabel'!$D$2:$D$496,$F58),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K58" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G58)+N($H58))=0,0,IF((N($G58)+N($H58))&lt;15,0.25,IF((N($G58)+N($H58))&lt;=50,0.035,IF((N($G58)+N($H58))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L58" s="392">
-        <f>IF($J58=0,0,$G58*$J58*(1+$K58))</f>
-        <v/>
-      </c>
-      <c r="M58" s="392">
-        <f>N($H58)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N58" s="398">
-        <f>$L58+$M58</f>
-        <v/>
-      </c>
-      <c r="O58" s="401">
-        <f>IF($I58="","nog te plannen",IFERROR(LOOKUP($I58,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J58" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G58)=0,0,IF($G58&lt;15,0.25,IF($G58&lt;=50,0.035,IF($G58&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K58" s="398">
+        <f>IF($I58=0,0,$G58*$I58*(1+$J58))</f>
+        <v/>
+      </c>
+      <c r="L58" s="401">
+        <f>IF($H58="","nog te plannen",IFERROR(LOOKUP($H58,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7195,30 +6632,21 @@
       <c r="E59" s="306" t="n"/>
       <c r="F59" s="306" t="n"/>
       <c r="G59" s="391" t="n"/>
-      <c r="H59" s="391" t="n"/>
-      <c r="I59" s="388" t="n"/>
-      <c r="J59" s="392">
+      <c r="H59" s="388" t="n"/>
+      <c r="I59" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C59,'SAERTEX-prijstabel'!$B$2:$B$496,$D59,'SAERTEX-prijstabel'!$C$2:$C$496,$E59,'SAERTEX-prijstabel'!$D$2:$D$496,$F59),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K59" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G59)+N($H59))=0,0,IF((N($G59)+N($H59))&lt;15,0.25,IF((N($G59)+N($H59))&lt;=50,0.035,IF((N($G59)+N($H59))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L59" s="392">
-        <f>IF($J59=0,0,$G59*$J59*(1+$K59))</f>
-        <v/>
-      </c>
-      <c r="M59" s="392">
-        <f>N($H59)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N59" s="398">
-        <f>$L59+$M59</f>
-        <v/>
-      </c>
-      <c r="O59" s="401">
-        <f>IF($I59="","nog te plannen",IFERROR(LOOKUP($I59,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J59" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G59)=0,0,IF($G59&lt;15,0.25,IF($G59&lt;=50,0.035,IF($G59&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K59" s="398">
+        <f>IF($I59=0,0,$G59*$I59*(1+$J59))</f>
+        <v/>
+      </c>
+      <c r="L59" s="401">
+        <f>IF($H59="","nog te plannen",IFERROR(LOOKUP($H59,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7230,30 +6658,21 @@
       <c r="E60" s="306" t="n"/>
       <c r="F60" s="306" t="n"/>
       <c r="G60" s="391" t="n"/>
-      <c r="H60" s="391" t="n"/>
-      <c r="I60" s="388" t="n"/>
-      <c r="J60" s="392">
+      <c r="H60" s="388" t="n"/>
+      <c r="I60" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C60,'SAERTEX-prijstabel'!$B$2:$B$496,$D60,'SAERTEX-prijstabel'!$C$2:$C$496,$E60,'SAERTEX-prijstabel'!$D$2:$D$496,$F60),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K60" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G60)+N($H60))=0,0,IF((N($G60)+N($H60))&lt;15,0.25,IF((N($G60)+N($H60))&lt;=50,0.035,IF((N($G60)+N($H60))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L60" s="392">
-        <f>IF($J60=0,0,$G60*$J60*(1+$K60))</f>
-        <v/>
-      </c>
-      <c r="M60" s="392">
-        <f>N($H60)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N60" s="398">
-        <f>$L60+$M60</f>
-        <v/>
-      </c>
-      <c r="O60" s="401">
-        <f>IF($I60="","nog te plannen",IFERROR(LOOKUP($I60,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J60" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G60)=0,0,IF($G60&lt;15,0.25,IF($G60&lt;=50,0.035,IF($G60&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K60" s="398">
+        <f>IF($I60=0,0,$G60*$I60*(1+$J60))</f>
+        <v/>
+      </c>
+      <c r="L60" s="401">
+        <f>IF($H60="","nog te plannen",IFERROR(LOOKUP($H60,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7265,30 +6684,21 @@
       <c r="E61" s="306" t="n"/>
       <c r="F61" s="306" t="n"/>
       <c r="G61" s="391" t="n"/>
-      <c r="H61" s="391" t="n"/>
-      <c r="I61" s="388" t="n"/>
-      <c r="J61" s="392">
+      <c r="H61" s="388" t="n"/>
+      <c r="I61" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C61,'SAERTEX-prijstabel'!$B$2:$B$496,$D61,'SAERTEX-prijstabel'!$C$2:$C$496,$E61,'SAERTEX-prijstabel'!$D$2:$D$496,$F61),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K61" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G61)+N($H61))=0,0,IF((N($G61)+N($H61))&lt;15,0.25,IF((N($G61)+N($H61))&lt;=50,0.035,IF((N($G61)+N($H61))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L61" s="392">
-        <f>IF($J61=0,0,$G61*$J61*(1+$K61))</f>
-        <v/>
-      </c>
-      <c r="M61" s="392">
-        <f>N($H61)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N61" s="398">
-        <f>$L61+$M61</f>
-        <v/>
-      </c>
-      <c r="O61" s="401">
-        <f>IF($I61="","nog te plannen",IFERROR(LOOKUP($I61,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J61" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G61)=0,0,IF($G61&lt;15,0.25,IF($G61&lt;=50,0.035,IF($G61&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K61" s="398">
+        <f>IF($I61=0,0,$G61*$I61*(1+$J61))</f>
+        <v/>
+      </c>
+      <c r="L61" s="401">
+        <f>IF($H61="","nog te plannen",IFERROR(LOOKUP($H61,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7300,30 +6710,21 @@
       <c r="E62" s="306" t="n"/>
       <c r="F62" s="306" t="n"/>
       <c r="G62" s="391" t="n"/>
-      <c r="H62" s="391" t="n"/>
-      <c r="I62" s="388" t="n"/>
-      <c r="J62" s="392">
+      <c r="H62" s="388" t="n"/>
+      <c r="I62" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C62,'SAERTEX-prijstabel'!$B$2:$B$496,$D62,'SAERTEX-prijstabel'!$C$2:$C$496,$E62,'SAERTEX-prijstabel'!$D$2:$D$496,$F62),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K62" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G62)+N($H62))=0,0,IF((N($G62)+N($H62))&lt;15,0.25,IF((N($G62)+N($H62))&lt;=50,0.035,IF((N($G62)+N($H62))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L62" s="392">
-        <f>IF($J62=0,0,$G62*$J62*(1+$K62))</f>
-        <v/>
-      </c>
-      <c r="M62" s="392">
-        <f>N($H62)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N62" s="398">
-        <f>$L62+$M62</f>
-        <v/>
-      </c>
-      <c r="O62" s="401">
-        <f>IF($I62="","nog te plannen",IFERROR(LOOKUP($I62,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J62" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G62)=0,0,IF($G62&lt;15,0.25,IF($G62&lt;=50,0.035,IF($G62&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K62" s="398">
+        <f>IF($I62=0,0,$G62*$I62*(1+$J62))</f>
+        <v/>
+      </c>
+      <c r="L62" s="401">
+        <f>IF($H62="","nog te plannen",IFERROR(LOOKUP($H62,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7335,30 +6736,21 @@
       <c r="E63" s="306" t="n"/>
       <c r="F63" s="306" t="n"/>
       <c r="G63" s="391" t="n"/>
-      <c r="H63" s="391" t="n"/>
-      <c r="I63" s="388" t="n"/>
-      <c r="J63" s="392">
+      <c r="H63" s="388" t="n"/>
+      <c r="I63" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C63,'SAERTEX-prijstabel'!$B$2:$B$496,$D63,'SAERTEX-prijstabel'!$C$2:$C$496,$E63,'SAERTEX-prijstabel'!$D$2:$D$496,$F63),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K63" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G63)+N($H63))=0,0,IF((N($G63)+N($H63))&lt;15,0.25,IF((N($G63)+N($H63))&lt;=50,0.035,IF((N($G63)+N($H63))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L63" s="392">
-        <f>IF($J63=0,0,$G63*$J63*(1+$K63))</f>
-        <v/>
-      </c>
-      <c r="M63" s="392">
-        <f>N($H63)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N63" s="398">
-        <f>$L63+$M63</f>
-        <v/>
-      </c>
-      <c r="O63" s="401">
-        <f>IF($I63="","nog te plannen",IFERROR(LOOKUP($I63,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J63" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G63)=0,0,IF($G63&lt;15,0.25,IF($G63&lt;=50,0.035,IF($G63&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K63" s="398">
+        <f>IF($I63=0,0,$G63*$I63*(1+$J63))</f>
+        <v/>
+      </c>
+      <c r="L63" s="401">
+        <f>IF($H63="","nog te plannen",IFERROR(LOOKUP($H63,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7370,30 +6762,21 @@
       <c r="E64" s="306" t="n"/>
       <c r="F64" s="306" t="n"/>
       <c r="G64" s="391" t="n"/>
-      <c r="H64" s="391" t="n"/>
-      <c r="I64" s="388" t="n"/>
-      <c r="J64" s="392">
+      <c r="H64" s="388" t="n"/>
+      <c r="I64" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C64,'SAERTEX-prijstabel'!$B$2:$B$496,$D64,'SAERTEX-prijstabel'!$C$2:$C$496,$E64,'SAERTEX-prijstabel'!$D$2:$D$496,$F64),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K64" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G64)+N($H64))=0,0,IF((N($G64)+N($H64))&lt;15,0.25,IF((N($G64)+N($H64))&lt;=50,0.035,IF((N($G64)+N($H64))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L64" s="392">
-        <f>IF($J64=0,0,$G64*$J64*(1+$K64))</f>
-        <v/>
-      </c>
-      <c r="M64" s="392">
-        <f>N($H64)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N64" s="398">
-        <f>$L64+$M64</f>
-        <v/>
-      </c>
-      <c r="O64" s="401">
-        <f>IF($I64="","nog te plannen",IFERROR(LOOKUP($I64,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J64" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G64)=0,0,IF($G64&lt;15,0.25,IF($G64&lt;=50,0.035,IF($G64&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K64" s="398">
+        <f>IF($I64=0,0,$G64*$I64*(1+$J64))</f>
+        <v/>
+      </c>
+      <c r="L64" s="401">
+        <f>IF($H64="","nog te plannen",IFERROR(LOOKUP($H64,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7405,30 +6788,21 @@
       <c r="E65" s="306" t="n"/>
       <c r="F65" s="306" t="n"/>
       <c r="G65" s="391" t="n"/>
-      <c r="H65" s="391" t="n"/>
-      <c r="I65" s="388" t="n"/>
-      <c r="J65" s="392">
+      <c r="H65" s="388" t="n"/>
+      <c r="I65" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C65,'SAERTEX-prijstabel'!$B$2:$B$496,$D65,'SAERTEX-prijstabel'!$C$2:$C$496,$E65,'SAERTEX-prijstabel'!$D$2:$D$496,$F65),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K65" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G65)+N($H65))=0,0,IF((N($G65)+N($H65))&lt;15,0.25,IF((N($G65)+N($H65))&lt;=50,0.035,IF((N($G65)+N($H65))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L65" s="392">
-        <f>IF($J65=0,0,$G65*$J65*(1+$K65))</f>
-        <v/>
-      </c>
-      <c r="M65" s="392">
-        <f>N($H65)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N65" s="398">
-        <f>$L65+$M65</f>
-        <v/>
-      </c>
-      <c r="O65" s="401">
-        <f>IF($I65="","nog te plannen",IFERROR(LOOKUP($I65,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J65" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G65)=0,0,IF($G65&lt;15,0.25,IF($G65&lt;=50,0.035,IF($G65&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K65" s="398">
+        <f>IF($I65=0,0,$G65*$I65*(1+$J65))</f>
+        <v/>
+      </c>
+      <c r="L65" s="401">
+        <f>IF($H65="","nog te plannen",IFERROR(LOOKUP($H65,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7440,30 +6814,21 @@
       <c r="E66" s="306" t="n"/>
       <c r="F66" s="306" t="n"/>
       <c r="G66" s="391" t="n"/>
-      <c r="H66" s="391" t="n"/>
-      <c r="I66" s="388" t="n"/>
-      <c r="J66" s="392">
+      <c r="H66" s="388" t="n"/>
+      <c r="I66" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C66,'SAERTEX-prijstabel'!$B$2:$B$496,$D66,'SAERTEX-prijstabel'!$C$2:$C$496,$E66,'SAERTEX-prijstabel'!$D$2:$D$496,$F66),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K66" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G66)+N($H66))=0,0,IF((N($G66)+N($H66))&lt;15,0.25,IF((N($G66)+N($H66))&lt;=50,0.035,IF((N($G66)+N($H66))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L66" s="392">
-        <f>IF($J66=0,0,$G66*$J66*(1+$K66))</f>
-        <v/>
-      </c>
-      <c r="M66" s="392">
-        <f>N($H66)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N66" s="398">
-        <f>$L66+$M66</f>
-        <v/>
-      </c>
-      <c r="O66" s="401">
-        <f>IF($I66="","nog te plannen",IFERROR(LOOKUP($I66,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J66" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G66)=0,0,IF($G66&lt;15,0.25,IF($G66&lt;=50,0.035,IF($G66&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K66" s="398">
+        <f>IF($I66=0,0,$G66*$I66*(1+$J66))</f>
+        <v/>
+      </c>
+      <c r="L66" s="401">
+        <f>IF($H66="","nog te plannen",IFERROR(LOOKUP($H66,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7475,30 +6840,21 @@
       <c r="E67" s="306" t="n"/>
       <c r="F67" s="306" t="n"/>
       <c r="G67" s="391" t="n"/>
-      <c r="H67" s="391" t="n"/>
-      <c r="I67" s="388" t="n"/>
-      <c r="J67" s="392">
+      <c r="H67" s="388" t="n"/>
+      <c r="I67" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C67,'SAERTEX-prijstabel'!$B$2:$B$496,$D67,'SAERTEX-prijstabel'!$C$2:$C$496,$E67,'SAERTEX-prijstabel'!$D$2:$D$496,$F67),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K67" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G67)+N($H67))=0,0,IF((N($G67)+N($H67))&lt;15,0.25,IF((N($G67)+N($H67))&lt;=50,0.035,IF((N($G67)+N($H67))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L67" s="392">
-        <f>IF($J67=0,0,$G67*$J67*(1+$K67))</f>
-        <v/>
-      </c>
-      <c r="M67" s="392">
-        <f>N($H67)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N67" s="398">
-        <f>$L67+$M67</f>
-        <v/>
-      </c>
-      <c r="O67" s="401">
-        <f>IF($I67="","nog te plannen",IFERROR(LOOKUP($I67,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J67" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G67)=0,0,IF($G67&lt;15,0.25,IF($G67&lt;=50,0.035,IF($G67&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K67" s="398">
+        <f>IF($I67=0,0,$G67*$I67*(1+$J67))</f>
+        <v/>
+      </c>
+      <c r="L67" s="401">
+        <f>IF($H67="","nog te plannen",IFERROR(LOOKUP($H67,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7510,30 +6866,21 @@
       <c r="E68" s="306" t="n"/>
       <c r="F68" s="306" t="n"/>
       <c r="G68" s="391" t="n"/>
-      <c r="H68" s="391" t="n"/>
-      <c r="I68" s="388" t="n"/>
-      <c r="J68" s="392">
+      <c r="H68" s="388" t="n"/>
+      <c r="I68" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C68,'SAERTEX-prijstabel'!$B$2:$B$496,$D68,'SAERTEX-prijstabel'!$C$2:$C$496,$E68,'SAERTEX-prijstabel'!$D$2:$D$496,$F68),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K68" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G68)+N($H68))=0,0,IF((N($G68)+N($H68))&lt;15,0.25,IF((N($G68)+N($H68))&lt;=50,0.035,IF((N($G68)+N($H68))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L68" s="392">
-        <f>IF($J68=0,0,$G68*$J68*(1+$K68))</f>
-        <v/>
-      </c>
-      <c r="M68" s="392">
-        <f>N($H68)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N68" s="398">
-        <f>$L68+$M68</f>
-        <v/>
-      </c>
-      <c r="O68" s="401">
-        <f>IF($I68="","nog te plannen",IFERROR(LOOKUP($I68,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J68" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G68)=0,0,IF($G68&lt;15,0.25,IF($G68&lt;=50,0.035,IF($G68&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K68" s="398">
+        <f>IF($I68=0,0,$G68*$I68*(1+$J68))</f>
+        <v/>
+      </c>
+      <c r="L68" s="401">
+        <f>IF($H68="","nog te plannen",IFERROR(LOOKUP($H68,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7545,30 +6892,21 @@
       <c r="E69" s="306" t="n"/>
       <c r="F69" s="306" t="n"/>
       <c r="G69" s="391" t="n"/>
-      <c r="H69" s="391" t="n"/>
-      <c r="I69" s="388" t="n"/>
-      <c r="J69" s="392">
+      <c r="H69" s="388" t="n"/>
+      <c r="I69" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C69,'SAERTEX-prijstabel'!$B$2:$B$496,$D69,'SAERTEX-prijstabel'!$C$2:$C$496,$E69,'SAERTEX-prijstabel'!$D$2:$D$496,$F69),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K69" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G69)+N($H69))=0,0,IF((N($G69)+N($H69))&lt;15,0.25,IF((N($G69)+N($H69))&lt;=50,0.035,IF((N($G69)+N($H69))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L69" s="392">
-        <f>IF($J69=0,0,$G69*$J69*(1+$K69))</f>
-        <v/>
-      </c>
-      <c r="M69" s="392">
-        <f>N($H69)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N69" s="398">
-        <f>$L69+$M69</f>
-        <v/>
-      </c>
-      <c r="O69" s="401">
-        <f>IF($I69="","nog te plannen",IFERROR(LOOKUP($I69,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J69" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G69)=0,0,IF($G69&lt;15,0.25,IF($G69&lt;=50,0.035,IF($G69&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K69" s="398">
+        <f>IF($I69=0,0,$G69*$I69*(1+$J69))</f>
+        <v/>
+      </c>
+      <c r="L69" s="401">
+        <f>IF($H69="","nog te plannen",IFERROR(LOOKUP($H69,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7580,30 +6918,21 @@
       <c r="E70" s="306" t="n"/>
       <c r="F70" s="306" t="n"/>
       <c r="G70" s="391" t="n"/>
-      <c r="H70" s="391" t="n"/>
-      <c r="I70" s="388" t="n"/>
-      <c r="J70" s="392">
+      <c r="H70" s="388" t="n"/>
+      <c r="I70" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C70,'SAERTEX-prijstabel'!$B$2:$B$496,$D70,'SAERTEX-prijstabel'!$C$2:$C$496,$E70,'SAERTEX-prijstabel'!$D$2:$D$496,$F70),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K70" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G70)+N($H70))=0,0,IF((N($G70)+N($H70))&lt;15,0.25,IF((N($G70)+N($H70))&lt;=50,0.035,IF((N($G70)+N($H70))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L70" s="392">
-        <f>IF($J70=0,0,$G70*$J70*(1+$K70))</f>
-        <v/>
-      </c>
-      <c r="M70" s="392">
-        <f>N($H70)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N70" s="398">
-        <f>$L70+$M70</f>
-        <v/>
-      </c>
-      <c r="O70" s="401">
-        <f>IF($I70="","nog te plannen",IFERROR(LOOKUP($I70,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J70" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G70)=0,0,IF($G70&lt;15,0.25,IF($G70&lt;=50,0.035,IF($G70&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K70" s="398">
+        <f>IF($I70=0,0,$G70*$I70*(1+$J70))</f>
+        <v/>
+      </c>
+      <c r="L70" s="401">
+        <f>IF($H70="","nog te plannen",IFERROR(LOOKUP($H70,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7615,30 +6944,21 @@
       <c r="E71" s="306" t="n"/>
       <c r="F71" s="306" t="n"/>
       <c r="G71" s="391" t="n"/>
-      <c r="H71" s="391" t="n"/>
-      <c r="I71" s="388" t="n"/>
-      <c r="J71" s="392">
+      <c r="H71" s="388" t="n"/>
+      <c r="I71" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C71,'SAERTEX-prijstabel'!$B$2:$B$496,$D71,'SAERTEX-prijstabel'!$C$2:$C$496,$E71,'SAERTEX-prijstabel'!$D$2:$D$496,$F71),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K71" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G71)+N($H71))=0,0,IF((N($G71)+N($H71))&lt;15,0.25,IF((N($G71)+N($H71))&lt;=50,0.035,IF((N($G71)+N($H71))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L71" s="392">
-        <f>IF($J71=0,0,$G71*$J71*(1+$K71))</f>
-        <v/>
-      </c>
-      <c r="M71" s="392">
-        <f>N($H71)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N71" s="398">
-        <f>$L71+$M71</f>
-        <v/>
-      </c>
-      <c r="O71" s="401">
-        <f>IF($I71="","nog te plannen",IFERROR(LOOKUP($I71,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J71" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G71)=0,0,IF($G71&lt;15,0.25,IF($G71&lt;=50,0.035,IF($G71&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K71" s="398">
+        <f>IF($I71=0,0,$G71*$I71*(1+$J71))</f>
+        <v/>
+      </c>
+      <c r="L71" s="401">
+        <f>IF($H71="","nog te plannen",IFERROR(LOOKUP($H71,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7650,30 +6970,21 @@
       <c r="E72" s="306" t="n"/>
       <c r="F72" s="306" t="n"/>
       <c r="G72" s="391" t="n"/>
-      <c r="H72" s="391" t="n"/>
-      <c r="I72" s="388" t="n"/>
-      <c r="J72" s="392">
+      <c r="H72" s="388" t="n"/>
+      <c r="I72" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C72,'SAERTEX-prijstabel'!$B$2:$B$496,$D72,'SAERTEX-prijstabel'!$C$2:$C$496,$E72,'SAERTEX-prijstabel'!$D$2:$D$496,$F72),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K72" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G72)+N($H72))=0,0,IF((N($G72)+N($H72))&lt;15,0.25,IF((N($G72)+N($H72))&lt;=50,0.035,IF((N($G72)+N($H72))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L72" s="392">
-        <f>IF($J72=0,0,$G72*$J72*(1+$K72))</f>
-        <v/>
-      </c>
-      <c r="M72" s="392">
-        <f>N($H72)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N72" s="398">
-        <f>$L72+$M72</f>
-        <v/>
-      </c>
-      <c r="O72" s="401">
-        <f>IF($I72="","nog te plannen",IFERROR(LOOKUP($I72,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J72" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G72)=0,0,IF($G72&lt;15,0.25,IF($G72&lt;=50,0.035,IF($G72&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K72" s="398">
+        <f>IF($I72=0,0,$G72*$I72*(1+$J72))</f>
+        <v/>
+      </c>
+      <c r="L72" s="401">
+        <f>IF($H72="","nog te plannen",IFERROR(LOOKUP($H72,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7685,30 +6996,21 @@
       <c r="E73" s="306" t="n"/>
       <c r="F73" s="306" t="n"/>
       <c r="G73" s="391" t="n"/>
-      <c r="H73" s="391" t="n"/>
-      <c r="I73" s="388" t="n"/>
-      <c r="J73" s="392">
+      <c r="H73" s="388" t="n"/>
+      <c r="I73" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C73,'SAERTEX-prijstabel'!$B$2:$B$496,$D73,'SAERTEX-prijstabel'!$C$2:$C$496,$E73,'SAERTEX-prijstabel'!$D$2:$D$496,$F73),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K73" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G73)+N($H73))=0,0,IF((N($G73)+N($H73))&lt;15,0.25,IF((N($G73)+N($H73))&lt;=50,0.035,IF((N($G73)+N($H73))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L73" s="392">
-        <f>IF($J73=0,0,$G73*$J73*(1+$K73))</f>
-        <v/>
-      </c>
-      <c r="M73" s="392">
-        <f>N($H73)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N73" s="398">
-        <f>$L73+$M73</f>
-        <v/>
-      </c>
-      <c r="O73" s="401">
-        <f>IF($I73="","nog te plannen",IFERROR(LOOKUP($I73,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J73" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G73)=0,0,IF($G73&lt;15,0.25,IF($G73&lt;=50,0.035,IF($G73&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K73" s="398">
+        <f>IF($I73=0,0,$G73*$I73*(1+$J73))</f>
+        <v/>
+      </c>
+      <c r="L73" s="401">
+        <f>IF($H73="","nog te plannen",IFERROR(LOOKUP($H73,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7720,30 +7022,21 @@
       <c r="E74" s="306" t="n"/>
       <c r="F74" s="306" t="n"/>
       <c r="G74" s="391" t="n"/>
-      <c r="H74" s="391" t="n"/>
-      <c r="I74" s="388" t="n"/>
-      <c r="J74" s="392">
+      <c r="H74" s="388" t="n"/>
+      <c r="I74" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C74,'SAERTEX-prijstabel'!$B$2:$B$496,$D74,'SAERTEX-prijstabel'!$C$2:$C$496,$E74,'SAERTEX-prijstabel'!$D$2:$D$496,$F74),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K74" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G74)+N($H74))=0,0,IF((N($G74)+N($H74))&lt;15,0.25,IF((N($G74)+N($H74))&lt;=50,0.035,IF((N($G74)+N($H74))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L74" s="392">
-        <f>IF($J74=0,0,$G74*$J74*(1+$K74))</f>
-        <v/>
-      </c>
-      <c r="M74" s="392">
-        <f>N($H74)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N74" s="398">
-        <f>$L74+$M74</f>
-        <v/>
-      </c>
-      <c r="O74" s="401">
-        <f>IF($I74="","nog te plannen",IFERROR(LOOKUP($I74,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J74" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G74)=0,0,IF($G74&lt;15,0.25,IF($G74&lt;=50,0.035,IF($G74&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K74" s="398">
+        <f>IF($I74=0,0,$G74*$I74*(1+$J74))</f>
+        <v/>
+      </c>
+      <c r="L74" s="401">
+        <f>IF($H74="","nog te plannen",IFERROR(LOOKUP($H74,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7755,30 +7048,21 @@
       <c r="E75" s="306" t="n"/>
       <c r="F75" s="306" t="n"/>
       <c r="G75" s="391" t="n"/>
-      <c r="H75" s="391" t="n"/>
-      <c r="I75" s="388" t="n"/>
-      <c r="J75" s="392">
+      <c r="H75" s="388" t="n"/>
+      <c r="I75" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C75,'SAERTEX-prijstabel'!$B$2:$B$496,$D75,'SAERTEX-prijstabel'!$C$2:$C$496,$E75,'SAERTEX-prijstabel'!$D$2:$D$496,$F75),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K75" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G75)+N($H75))=0,0,IF((N($G75)+N($H75))&lt;15,0.25,IF((N($G75)+N($H75))&lt;=50,0.035,IF((N($G75)+N($H75))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L75" s="392">
-        <f>IF($J75=0,0,$G75*$J75*(1+$K75))</f>
-        <v/>
-      </c>
-      <c r="M75" s="392">
-        <f>N($H75)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N75" s="398">
-        <f>$L75+$M75</f>
-        <v/>
-      </c>
-      <c r="O75" s="401">
-        <f>IF($I75="","nog te plannen",IFERROR(LOOKUP($I75,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J75" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G75)=0,0,IF($G75&lt;15,0.25,IF($G75&lt;=50,0.035,IF($G75&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K75" s="398">
+        <f>IF($I75=0,0,$G75*$I75*(1+$J75))</f>
+        <v/>
+      </c>
+      <c r="L75" s="401">
+        <f>IF($H75="","nog te plannen",IFERROR(LOOKUP($H75,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7790,30 +7074,21 @@
       <c r="E76" s="306" t="n"/>
       <c r="F76" s="306" t="n"/>
       <c r="G76" s="391" t="n"/>
-      <c r="H76" s="391" t="n"/>
-      <c r="I76" s="388" t="n"/>
-      <c r="J76" s="392">
+      <c r="H76" s="388" t="n"/>
+      <c r="I76" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C76,'SAERTEX-prijstabel'!$B$2:$B$496,$D76,'SAERTEX-prijstabel'!$C$2:$C$496,$E76,'SAERTEX-prijstabel'!$D$2:$D$496,$F76),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K76" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G76)+N($H76))=0,0,IF((N($G76)+N($H76))&lt;15,0.25,IF((N($G76)+N($H76))&lt;=50,0.035,IF((N($G76)+N($H76))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L76" s="392">
-        <f>IF($J76=0,0,$G76*$J76*(1+$K76))</f>
-        <v/>
-      </c>
-      <c r="M76" s="392">
-        <f>N($H76)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N76" s="398">
-        <f>$L76+$M76</f>
-        <v/>
-      </c>
-      <c r="O76" s="401">
-        <f>IF($I76="","nog te plannen",IFERROR(LOOKUP($I76,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J76" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G76)=0,0,IF($G76&lt;15,0.25,IF($G76&lt;=50,0.035,IF($G76&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K76" s="398">
+        <f>IF($I76=0,0,$G76*$I76*(1+$J76))</f>
+        <v/>
+      </c>
+      <c r="L76" s="401">
+        <f>IF($H76="","nog te plannen",IFERROR(LOOKUP($H76,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7825,30 +7100,21 @@
       <c r="E77" s="306" t="n"/>
       <c r="F77" s="306" t="n"/>
       <c r="G77" s="391" t="n"/>
-      <c r="H77" s="391" t="n"/>
-      <c r="I77" s="388" t="n"/>
-      <c r="J77" s="392">
+      <c r="H77" s="388" t="n"/>
+      <c r="I77" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C77,'SAERTEX-prijstabel'!$B$2:$B$496,$D77,'SAERTEX-prijstabel'!$C$2:$C$496,$E77,'SAERTEX-prijstabel'!$D$2:$D$496,$F77),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K77" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G77)+N($H77))=0,0,IF((N($G77)+N($H77))&lt;15,0.25,IF((N($G77)+N($H77))&lt;=50,0.035,IF((N($G77)+N($H77))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L77" s="392">
-        <f>IF($J77=0,0,$G77*$J77*(1+$K77))</f>
-        <v/>
-      </c>
-      <c r="M77" s="392">
-        <f>N($H77)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N77" s="398">
-        <f>$L77+$M77</f>
-        <v/>
-      </c>
-      <c r="O77" s="401">
-        <f>IF($I77="","nog te plannen",IFERROR(LOOKUP($I77,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J77" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G77)=0,0,IF($G77&lt;15,0.25,IF($G77&lt;=50,0.035,IF($G77&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K77" s="398">
+        <f>IF($I77=0,0,$G77*$I77*(1+$J77))</f>
+        <v/>
+      </c>
+      <c r="L77" s="401">
+        <f>IF($H77="","nog te plannen",IFERROR(LOOKUP($H77,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7860,30 +7126,21 @@
       <c r="E78" s="306" t="n"/>
       <c r="F78" s="306" t="n"/>
       <c r="G78" s="391" t="n"/>
-      <c r="H78" s="391" t="n"/>
-      <c r="I78" s="388" t="n"/>
-      <c r="J78" s="392">
+      <c r="H78" s="388" t="n"/>
+      <c r="I78" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C78,'SAERTEX-prijstabel'!$B$2:$B$496,$D78,'SAERTEX-prijstabel'!$C$2:$C$496,$E78,'SAERTEX-prijstabel'!$D$2:$D$496,$F78),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K78" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G78)+N($H78))=0,0,IF((N($G78)+N($H78))&lt;15,0.25,IF((N($G78)+N($H78))&lt;=50,0.035,IF((N($G78)+N($H78))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L78" s="392">
-        <f>IF($J78=0,0,$G78*$J78*(1+$K78))</f>
-        <v/>
-      </c>
-      <c r="M78" s="392">
-        <f>N($H78)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N78" s="398">
-        <f>$L78+$M78</f>
-        <v/>
-      </c>
-      <c r="O78" s="401">
-        <f>IF($I78="","nog te plannen",IFERROR(LOOKUP($I78,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J78" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G78)=0,0,IF($G78&lt;15,0.25,IF($G78&lt;=50,0.035,IF($G78&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K78" s="398">
+        <f>IF($I78=0,0,$G78*$I78*(1+$J78))</f>
+        <v/>
+      </c>
+      <c r="L78" s="401">
+        <f>IF($H78="","nog te plannen",IFERROR(LOOKUP($H78,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7895,30 +7152,21 @@
       <c r="E79" s="306" t="n"/>
       <c r="F79" s="306" t="n"/>
       <c r="G79" s="391" t="n"/>
-      <c r="H79" s="391" t="n"/>
-      <c r="I79" s="388" t="n"/>
-      <c r="J79" s="392">
+      <c r="H79" s="388" t="n"/>
+      <c r="I79" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C79,'SAERTEX-prijstabel'!$B$2:$B$496,$D79,'SAERTEX-prijstabel'!$C$2:$C$496,$E79,'SAERTEX-prijstabel'!$D$2:$D$496,$F79),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K79" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G79)+N($H79))=0,0,IF((N($G79)+N($H79))&lt;15,0.25,IF((N($G79)+N($H79))&lt;=50,0.035,IF((N($G79)+N($H79))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L79" s="392">
-        <f>IF($J79=0,0,$G79*$J79*(1+$K79))</f>
-        <v/>
-      </c>
-      <c r="M79" s="392">
-        <f>N($H79)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N79" s="398">
-        <f>$L79+$M79</f>
-        <v/>
-      </c>
-      <c r="O79" s="401">
-        <f>IF($I79="","nog te plannen",IFERROR(LOOKUP($I79,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J79" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G79)=0,0,IF($G79&lt;15,0.25,IF($G79&lt;=50,0.035,IF($G79&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K79" s="398">
+        <f>IF($I79=0,0,$G79*$I79*(1+$J79))</f>
+        <v/>
+      </c>
+      <c r="L79" s="401">
+        <f>IF($H79="","nog te plannen",IFERROR(LOOKUP($H79,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
@@ -7930,41 +7178,32 @@
       <c r="E80" s="306" t="n"/>
       <c r="F80" s="306" t="n"/>
       <c r="G80" s="391" t="n"/>
-      <c r="H80" s="391" t="n"/>
-      <c r="I80" s="388" t="n"/>
-      <c r="J80" s="392">
+      <c r="H80" s="388" t="n"/>
+      <c r="I80" s="392">
         <f>IFERROR(SUMIFS('SAERTEX-prijstabel'!$E$2:$E$496,'SAERTEX-prijstabel'!$A$2:$A$496,$C80,'SAERTEX-prijstabel'!$B$2:$B$496,$D80,'SAERTEX-prijstabel'!$C$2:$C$496,$E80,'SAERTEX-prijstabel'!$D$2:$D$496,$F80),0)*(1+'SAERTEX 2026'!$B$3)</f>
         <v/>
       </c>
-      <c r="K80" s="423">
-        <f>IF($B$3&lt;&gt;"ja",0,IF((N($G80)+N($H80))=0,0,IF((N($G80)+N($H80))&lt;15,0.25,IF((N($G80)+N($H80))&lt;=50,0.035,IF((N($G80)+N($H80))&lt;=200,0.025,0.01)))))</f>
-        <v/>
-      </c>
-      <c r="L80" s="392">
-        <f>IF($J80=0,0,$G80*$J80*(1+$K80))</f>
-        <v/>
-      </c>
-      <c r="M80" s="392">
-        <f>N($H80)*$E$3</f>
-        <v/>
-      </c>
-      <c r="N80" s="398">
-        <f>$L80+$M80</f>
-        <v/>
-      </c>
-      <c r="O80" s="401">
-        <f>IF($I80="","nog te plannen",IFERROR(LOOKUP($I80,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
+      <c r="J80" s="423">
+        <f>IF($B$3&lt;&gt;"ja",0,IF(N($G80)=0,0,IF($G80&lt;15,0.25,IF($G80&lt;=50,0.035,IF($G80&lt;=200,0.025,0.01)))))</f>
+        <v/>
+      </c>
+      <c r="K80" s="398">
+        <f>IF($I80=0,0,$G80*$I80*(1+$J80))</f>
+        <v/>
+      </c>
+      <c r="L80" s="401">
+        <f>IF($H80="","nog te plannen",IFERROR(LOOKUP($H80,'Periode-overzicht'!$B$25:$B$37,'Periode-overzicht'!$A$25:$A$37),"&lt;P1"))</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="M81" s="402" t="inlineStr">
+      <c r="J81" s="402" t="inlineStr">
         <is>
           <t>TOTAAL</t>
         </is>
       </c>
-      <c r="N81" s="403">
-        <f>SUM(N5:N80)</f>
+      <c r="K81" s="403">
+        <f>SUM(K5:K80)</f>
         <v/>
       </c>
     </row>
@@ -8176,7 +7415,7 @@
       <c r="D14" s="306" t="n"/>
       <c r="E14" s="410" t="n"/>
       <c r="F14" s="411">
-        <f>'Kousen'!N81</f>
+        <f>'Kousen'!K81</f>
         <v/>
       </c>
       <c r="G14" s="410" t="n"/>

</xml_diff>